<commit_message>
Add V4.1 shared KV and conditional PD estimates to EP sweep
</commit_message>
<xml_diff>
--- a/examples/kv-ep-sweep/kv-ep32-ep256.xlsx
+++ b/examples/kv-ep-sweep/kv-ep32-ep256.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规格汇总" sheetId="1" r:id="R151062668cff4f63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KV明细" sheetId="2" r:id="Ra8d89f14d63a4800"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EP通信" sheetId="3" r:id="Rd8d65e6068054d39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规格汇总" sheetId="1" r:id="R13bd640b94e84542"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KV明细" sheetId="2" r:id="R7b68b400227b4bb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EP通信" sheetId="3" r:id="R425b3e88a8784639"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,7 +20,7 @@
     <x:numFmt numFmtId="201" formatCode="#,##0.000"/>
     <x:numFmt numFmtId="202" formatCode="#,##0.000000"/>
   </x:numFmts>
-  <x:fonts count="5">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -46,6 +46,11 @@
       <x:b/>
       <x:sz val="14"/>
       <x:color rgb="FF202C3B"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF955700"/>
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
@@ -78,7 +83,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="16">
+  <x:cellXfs count="17">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -121,6 +126,9 @@
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="202" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
@@ -474,27 +482,27 @@
     </x:row>
     <x:row r="6" ht="25" customHeight="1">
       <x:c r="A6" s="2" t="str">
-        <x:f>A22</x:f>
+        <x:f>A24</x:f>
         <x:v>DS V4 10T</x:v>
       </x:c>
       <x:c r="B6" s="2" t="n">
-        <x:f>B22</x:f>
+        <x:f>B24</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="C6" s="2" t="n">
-        <x:f>C22</x:f>
+        <x:f>C24</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D6" s="2" t="n">
-        <x:f>D22</x:f>
+        <x:f>D24</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="E6" s="2" t="n">
-        <x:f>E22</x:f>
+        <x:f>E24</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="F6" s="2" t="n">
-        <x:f>F22</x:f>
+        <x:f>F24</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="G6" s="8" t="n">
@@ -522,33 +530,33 @@
         <x:v>1.257193922996521</x:v>
       </x:c>
       <x:c r="M6" s="2" t="str">
-        <x:f>M22</x:f>
+        <x:f>M24</x:f>
         <x:v>专家数整除；未实机验证</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="25" customHeight="1">
       <x:c r="A7" s="2" t="str">
-        <x:f>A23</x:f>
+        <x:f>A25</x:f>
         <x:v>DS V4 10T</x:v>
       </x:c>
       <x:c r="B7" s="2" t="n">
-        <x:f>B23</x:f>
+        <x:f>B25</x:f>
         <x:v>256</x:v>
       </x:c>
       <x:c r="C7" s="2" t="n">
-        <x:f>C23</x:f>
+        <x:f>C25</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D7" s="2" t="n">
-        <x:f>D23</x:f>
+        <x:f>D25</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="E7" s="2" t="n">
-        <x:f>E23</x:f>
+        <x:f>E25</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="F7" s="2" t="n">
-        <x:f>F23</x:f>
+        <x:f>F25</x:f>
         <x:v>256</x:v>
       </x:c>
       <x:c r="G7" s="8" t="n">
@@ -576,33 +584,33 @@
         <x:v>1.292911022901535</x:v>
       </x:c>
       <x:c r="M7" s="2" t="str">
-        <x:f>M23</x:f>
+        <x:f>M25</x:f>
         <x:v>需补齐128槽并验证EPLB</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="25" customHeight="1">
       <x:c r="A8" s="2" t="str">
-        <x:f>A24</x:f>
+        <x:f>A26</x:f>
         <x:v>DS V4 Pro</x:v>
       </x:c>
       <x:c r="B8" s="2" t="n">
-        <x:f>B24</x:f>
+        <x:f>B26</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="C8" s="2" t="n">
-        <x:f>C24</x:f>
+        <x:f>C26</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D8" s="2" t="n">
-        <x:f>D24</x:f>
+        <x:f>D26</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="E8" s="2" t="n">
-        <x:f>E24</x:f>
+        <x:f>E26</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="F8" s="2" t="n">
-        <x:f>F24</x:f>
+        <x:f>F26</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="G8" s="8" t="n">
@@ -630,33 +638,33 @@
         <x:v>1.257193922996521</x:v>
       </x:c>
       <x:c r="M8" s="2" t="str">
-        <x:f>M24</x:f>
+        <x:f>M26</x:f>
         <x:v>专家数整除；未实机验证</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="25" customHeight="1">
       <x:c r="A9" s="2" t="str">
-        <x:f>A25</x:f>
+        <x:f>A27</x:f>
         <x:v>DS V4 Pro</x:v>
       </x:c>
       <x:c r="B9" s="2" t="n">
-        <x:f>B25</x:f>
+        <x:f>B27</x:f>
         <x:v>256</x:v>
       </x:c>
       <x:c r="C9" s="2" t="n">
-        <x:f>C25</x:f>
+        <x:f>C27</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D9" s="2" t="n">
-        <x:f>D25</x:f>
+        <x:f>D27</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="E9" s="2" t="n">
-        <x:f>E25</x:f>
+        <x:f>E27</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="F9" s="2" t="n">
-        <x:f>F25</x:f>
+        <x:f>F27</x:f>
         <x:v>256</x:v>
       </x:c>
       <x:c r="G9" s="8" t="n">
@@ -684,33 +692,33 @@
         <x:v>1.292911022901535</x:v>
       </x:c>
       <x:c r="M9" s="2" t="str">
-        <x:f>M25</x:f>
+        <x:f>M27</x:f>
         <x:v>需补齐128槽并验证EPLB</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="25" customHeight="1">
       <x:c r="A10" s="2" t="str">
-        <x:f>A26</x:f>
+        <x:f>A28</x:f>
         <x:v>GLM5.3</x:v>
       </x:c>
       <x:c r="B10" s="2" t="n">
-        <x:f>B26</x:f>
+        <x:f>B28</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="C10" s="2" t="n">
-        <x:f>C26</x:f>
+        <x:f>C28</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D10" s="2" t="n">
-        <x:f>D26</x:f>
+        <x:f>D28</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="E10" s="2" t="n">
-        <x:f>E26</x:f>
+        <x:f>E28</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="F10" s="2" t="n">
-        <x:f>F26</x:f>
+        <x:f>F28</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="G10" s="8" t="n">
@@ -738,33 +746,33 @@
         <x:v>1.7766058444976807</x:v>
       </x:c>
       <x:c r="M10" s="2" t="str">
-        <x:f>M26</x:f>
+        <x:f>M28</x:f>
         <x:v>专家数整除；未实机验证</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="25" customHeight="1">
       <x:c r="A11" s="2" t="str">
-        <x:f>A27</x:f>
+        <x:f>A29</x:f>
         <x:v>GLM5.3</x:v>
       </x:c>
       <x:c r="B11" s="2" t="n">
-        <x:f>B27</x:f>
+        <x:f>B29</x:f>
         <x:v>256</x:v>
       </x:c>
       <x:c r="C11" s="2" t="n">
-        <x:f>C27</x:f>
+        <x:f>C29</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D11" s="2" t="n">
-        <x:f>D27</x:f>
+        <x:f>D29</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="E11" s="2" t="n">
-        <x:f>E27</x:f>
+        <x:f>E29</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="F11" s="2" t="n">
-        <x:f>F27</x:f>
+        <x:f>F29</x:f>
         <x:v>256</x:v>
       </x:c>
       <x:c r="G11" s="8" t="n">
@@ -792,33 +800,33 @@
         <x:v>1.8267519772052765</x:v>
       </x:c>
       <x:c r="M11" s="2" t="str">
-        <x:f>M27</x:f>
+        <x:f>M29</x:f>
         <x:v>专家数整除；未实机验证</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="25" customHeight="1">
       <x:c r="A12" s="2" t="str">
-        <x:f>A28</x:f>
+        <x:f>A30</x:f>
         <x:v>KimiK3</x:v>
       </x:c>
       <x:c r="B12" s="2" t="n">
-        <x:f>B28</x:f>
+        <x:f>B30</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="C12" s="2" t="n">
-        <x:f>C28</x:f>
+        <x:f>C30</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D12" s="2" t="n">
-        <x:f>D28</x:f>
+        <x:f>D30</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="E12" s="2" t="n">
-        <x:f>E28</x:f>
+        <x:f>E30</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="F12" s="2" t="n">
-        <x:f>F28</x:f>
+        <x:f>F30</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="G12" s="8" t="n">
@@ -846,33 +854,33 @@
         <x:v>0.6340718269348145</x:v>
       </x:c>
       <x:c r="M12" s="2" t="str">
-        <x:f>M28</x:f>
+        <x:f>M30</x:f>
         <x:v>专家数整除；未实机验证</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="25" customHeight="1">
       <x:c r="A13" s="2" t="str">
-        <x:f>A29</x:f>
+        <x:f>A31</x:f>
         <x:v>KimiK3</x:v>
       </x:c>
       <x:c r="B13" s="2" t="n">
-        <x:f>B29</x:f>
+        <x:f>B31</x:f>
         <x:v>256</x:v>
       </x:c>
       <x:c r="C13" s="2" t="n">
-        <x:f>C29</x:f>
+        <x:f>C31</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D13" s="2" t="n">
-        <x:f>D29</x:f>
+        <x:f>D31</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="E13" s="2" t="n">
-        <x:f>E29</x:f>
+        <x:f>E31</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="F13" s="2" t="n">
-        <x:f>F29</x:f>
+        <x:f>F31</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="G13" s="8" t="n">
@@ -900,33 +908,33 @@
         <x:v>0.6523185968399048</x:v>
       </x:c>
       <x:c r="M13" s="2" t="str">
-        <x:f>M29</x:f>
+        <x:f>M31</x:f>
         <x:v>需补齐128槽并验证EPLB</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="25" customHeight="1">
       <x:c r="A14" s="2" t="str">
-        <x:f>A30</x:f>
+        <x:f>A32</x:f>
         <x:v>Qwen3.8 2.4T</x:v>
       </x:c>
       <x:c r="B14" s="2" t="n">
-        <x:f>B30</x:f>
+        <x:f>B32</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="C14" s="2" t="n">
-        <x:f>C30</x:f>
+        <x:f>C32</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D14" s="2" t="n">
-        <x:f>D30</x:f>
+        <x:f>D32</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="E14" s="2" t="n">
-        <x:f>E30</x:f>
+        <x:f>E32</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="F14" s="2" t="n">
-        <x:f>F30</x:f>
+        <x:f>F32</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="G14" s="8" t="n">
@@ -954,33 +962,33 @@
         <x:v>0.45736467838287354</x:v>
       </x:c>
       <x:c r="M14" s="2" t="str">
-        <x:f>M30</x:f>
+        <x:f>M32</x:f>
         <x:v>专家数整除；未实机验证</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="25" customHeight="1">
       <x:c r="A15" s="2" t="str">
-        <x:f>A31</x:f>
+        <x:f>A33</x:f>
         <x:v>Qwen3.8 2.4T</x:v>
       </x:c>
       <x:c r="B15" s="2" t="n">
-        <x:f>B31</x:f>
+        <x:f>B33</x:f>
         <x:v>256</x:v>
       </x:c>
       <x:c r="C15" s="2" t="n">
-        <x:f>C31</x:f>
+        <x:f>C33</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D15" s="2" t="n">
-        <x:f>D31</x:f>
+        <x:f>D33</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="E15" s="2" t="n">
-        <x:f>E31</x:f>
+        <x:f>E33</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="F15" s="2" t="n">
-        <x:f>F31</x:f>
+        <x:f>F33</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="G15" s="8" t="n">
@@ -1008,44 +1016,120 @@
         <x:v>0.4702741652727127</x:v>
       </x:c>
       <x:c r="M15" s="2" t="str">
-        <x:f>M31</x:f>
+        <x:f>M33</x:f>
         <x:v>专家数整除；未实机验证</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="25" customHeight="1">
-      <x:c r="A16" s="2"/>
-      <x:c r="B16" s="2"/>
-      <x:c r="C16" s="2"/>
-      <x:c r="D16" s="2"/>
-      <x:c r="E16" s="2"/>
-      <x:c r="F16" s="2"/>
-      <x:c r="G16" s="2"/>
-      <x:c r="H16" s="2"/>
-      <x:c r="I16" s="2"/>
-      <x:c r="J16" s="2"/>
-      <x:c r="K16" s="2"/>
-      <x:c r="L16" s="2"/>
-      <x:c r="M16" s="2"/>
+      <x:c r="A16" s="2" t="str">
+        <x:f>A34</x:f>
+        <x:v>DS V4.1 Flash</x:v>
+      </x:c>
+      <x:c r="B16" s="2" t="n">
+        <x:f>B34</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C16" s="2" t="n">
+        <x:f>C34</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D16" s="2" t="n">
+        <x:f>D34</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E16" s="2" t="n">
+        <x:f>E34</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F16" s="2" t="n">
+        <x:f>F34</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="G16" s="8" t="n">
+        <x:f>'EP通信'!K20*B16</x:f>
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="H16" s="8" t="n">
+        <x:f>'EP通信'!L20*B16</x:f>
+        <x:v>4096</x:v>
+      </x:c>
+      <x:c r="I16" s="9" t="n">
+        <x:f>'EP通信'!F34</x:f>
+        <x:v>290.6817626953125</x:v>
+      </x:c>
+      <x:c r="J16" s="9" t="n">
+        <x:f>'EP通信'!K34</x:f>
+        <x:v>19.114837646484375</x:v>
+      </x:c>
+      <x:c r="K16" s="9" t="n">
+        <x:f>I16/B16</x:f>
+        <x:v>9.083805084228516</x:v>
+      </x:c>
+      <x:c r="L16" s="9" t="n">
+        <x:f>J16/B16</x:f>
+        <x:v>0.5973386764526367</x:v>
+      </x:c>
+      <x:c r="M16" s="2" t="str">
+        <x:f>M34</x:f>
+        <x:v>取为规划值；迁移未支持</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="25" customHeight="1">
-      <x:c r="A17" s="2"/>
-      <x:c r="B17" s="2"/>
-      <x:c r="C17" s="2"/>
-      <x:c r="D17" s="2"/>
-      <x:c r="E17" s="2"/>
-      <x:c r="F17" s="2"/>
-      <x:c r="G17" s="2"/>
-      <x:c r="H17" s="2"/>
-      <x:c r="I17" s="2"/>
-      <x:c r="J17" s="2"/>
-      <x:c r="K17" s="2"/>
-      <x:c r="L17" s="2"/>
-      <x:c r="M17" s="2"/>
+      <x:c r="A17" s="2" t="str">
+        <x:f>A35</x:f>
+        <x:v>DS V4.1 Flash</x:v>
+      </x:c>
+      <x:c r="B17" s="2" t="n">
+        <x:f>B35</x:f>
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="C17" s="2" t="n">
+        <x:f>C35</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D17" s="2" t="n">
+        <x:f>D35</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="E17" s="2" t="n">
+        <x:f>E35</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F17" s="2" t="n">
+        <x:f>F35</x:f>
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G17" s="8" t="n">
+        <x:f>'EP通信'!K21*B17</x:f>
+        <x:v>524288</x:v>
+      </x:c>
+      <x:c r="H17" s="8" t="n">
+        <x:f>'EP通信'!L21*B17</x:f>
+        <x:v>32768</x:v>
+      </x:c>
+      <x:c r="I17" s="9" t="n">
+        <x:f>'EP通信'!F35</x:f>
+        <x:v>2395.60546875</x:v>
+      </x:c>
+      <x:c r="J17" s="9" t="n">
+        <x:f>'EP通信'!K35</x:f>
+        <x:v>157.27386474609375</x:v>
+      </x:c>
+      <x:c r="K17" s="9" t="n">
+        <x:f>I17/B17</x:f>
+        <x:v>9.357833862304688</x:v>
+      </x:c>
+      <x:c r="L17" s="9" t="n">
+        <x:f>J17/B17</x:f>
+        <x:v>0.6143510341644287</x:v>
+      </x:c>
+      <x:c r="M17" s="2" t="str">
+        <x:f>M35</x:f>
+        <x:v>补128槽并验证；取为规划值</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="25" customHeight="1">
-      <x:c r="A18" s="10" t="str">
-        <x:v>配套 KV 存取 · 每请求 / 每 P DP 批 / P 整组</x:v>
-      </x:c>
+      <x:c r="A18" s="2"/>
       <x:c r="B18" s="2"/>
       <x:c r="C18" s="2"/>
       <x:c r="D18" s="2"/>
@@ -1060,9 +1144,7 @@
       <x:c r="M18" s="2"/>
     </x:row>
     <x:row r="19" ht="25" customHeight="1">
-      <x:c r="A19" s="2" t="str">
-        <x:v>单位 GiB。存＝生成 KV 行＋最终辅助状态；取＝P→D 拉取。主干层，不含 draft/MTP 网络。</x:v>
-      </x:c>
+      <x:c r="A19" s="2"/>
       <x:c r="B19" s="2"/>
       <x:c r="C19" s="2"/>
       <x:c r="D19" s="2"/>
@@ -1077,7 +1159,9 @@
       <x:c r="M19" s="2"/>
     </x:row>
     <x:row r="20" ht="25" customHeight="1">
-      <x:c r="A20" s="2"/>
+      <x:c r="A20" s="10" t="str">
+        <x:v>配套 KV 存取 · 每请求 / 每 P DP 批 / P 整组</x:v>
+      </x:c>
       <x:c r="B20" s="2"/>
       <x:c r="C20" s="2"/>
       <x:c r="D20" s="2"/>
@@ -1091,166 +1175,90 @@
       <x:c r="L20" s="2"/>
       <x:c r="M20" s="2"/>
     </x:row>
-    <x:row r="21" ht="40" customHeight="1">
-      <x:c r="A21" s="7" t="str">
+    <x:row r="21" ht="25" customHeight="1">
+      <x:c r="A21" s="2" t="str">
+        <x:v>单位 GiB。存＝生成 KV 行＋最终辅助状态；取＝P→D 张量字节。V4.1 的取仅为规划值，main 未支持迁移。</x:v>
+      </x:c>
+      <x:c r="B21" s="2"/>
+      <x:c r="C21" s="2"/>
+      <x:c r="D21" s="2"/>
+      <x:c r="E21" s="2"/>
+      <x:c r="F21" s="2"/>
+      <x:c r="G21" s="2"/>
+      <x:c r="H21" s="2"/>
+      <x:c r="I21" s="2"/>
+      <x:c r="J21" s="2"/>
+      <x:c r="K21" s="2"/>
+      <x:c r="L21" s="2"/>
+      <x:c r="M21" s="2"/>
+    </x:row>
+    <x:row r="22" ht="25" customHeight="1">
+      <x:c r="A22" s="2"/>
+      <x:c r="B22" s="2"/>
+      <x:c r="C22" s="2"/>
+      <x:c r="D22" s="2"/>
+      <x:c r="E22" s="2"/>
+      <x:c r="F22" s="2"/>
+      <x:c r="G22" s="2"/>
+      <x:c r="H22" s="2"/>
+      <x:c r="I22" s="2"/>
+      <x:c r="J22" s="2"/>
+      <x:c r="K22" s="2"/>
+      <x:c r="L22" s="2"/>
+      <x:c r="M22" s="2"/>
+    </x:row>
+    <x:row r="23" ht="40" customHeight="1">
+      <x:c r="A23" s="7" t="str">
         <x:v>模型</x:v>
       </x:c>
-      <x:c r="B21" s="7" t="str">
+      <x:c r="B23" s="7" t="str">
         <x:v>EP</x:v>
       </x:c>
-      <x:c r="C21" s="7" t="str">
+      <x:c r="C23" s="7" t="str">
         <x:v>P TP</x:v>
       </x:c>
-      <x:c r="D21" s="7" t="str">
+      <x:c r="D23" s="7" t="str">
         <x:v>P DP</x:v>
       </x:c>
-      <x:c r="E21" s="7" t="str">
+      <x:c r="E23" s="7" t="str">
         <x:v>D TP</x:v>
       </x:c>
-      <x:c r="F21" s="7" t="str">
+      <x:c r="F23" s="7" t="str">
         <x:v>D DP</x:v>
       </x:c>
-      <x:c r="G21" s="7" t="str">
+      <x:c r="G23" s="7" t="str">
         <x:v>存/请求</x:v>
       </x:c>
-      <x:c r="H21" s="7" t="str">
-        <x:v>取/请求</x:v>
-      </x:c>
-      <x:c r="I21" s="7" t="str">
+      <x:c r="H23" s="7" t="str">
+        <x:v>取或规划取/请求</x:v>
+      </x:c>
+      <x:c r="I23" s="7" t="str">
         <x:v>存/P DP批</x:v>
       </x:c>
-      <x:c r="J21" s="7" t="str">
-        <x:v>取/P DP批</x:v>
-      </x:c>
-      <x:c r="K21" s="7" t="str">
+      <x:c r="J23" s="7" t="str">
+        <x:v>取或规划取/批</x:v>
+      </x:c>
+      <x:c r="K23" s="7" t="str">
         <x:v>存/P整组</x:v>
       </x:c>
-      <x:c r="L21" s="7" t="str">
-        <x:v>取/P整组</x:v>
-      </x:c>
-      <x:c r="M21" s="7" t="str">
-        <x:v>部署条件</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="25" customHeight="1">
-      <x:c r="A22" s="2" t="str">
+      <x:c r="L23" s="7" t="str">
+        <x:v>取或规划取/整组</x:v>
+      </x:c>
+      <x:c r="M23" s="7" t="str">
+        <x:v>部署 / 迁移条件</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="25" customHeight="1">
+      <x:c r="A24" s="2" t="str">
         <x:f>'EP通信'!A10</x:f>
         <x:v>DS V4 10T</x:v>
       </x:c>
-      <x:c r="B22" s="2" t="n">
+      <x:c r="B24" s="2" t="n">
         <x:f>'EP通信'!B10</x:f>
         <x:v>32</x:v>
       </x:c>
-      <x:c r="C22" s="2" t="n">
+      <x:c r="C24" s="2" t="n">
         <x:f>'EP通信'!I10</x:f>
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="D22" s="2" t="n">
-        <x:f>B22/C22</x:f>
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="E22" s="2" t="n">
-        <x:f>'EP通信'!J10</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F22" s="2" t="n">
-        <x:f>B22/E22</x:f>
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="G22" s="9" t="n">
-        <x:f>'KV明细'!J16</x:f>
-        <x:v>139.52711632847786</x:v>
-      </x:c>
-      <x:c r="H22" s="9" t="n">
-        <x:f>'KV明细'!L16</x:f>
-        <x:v>2.21197509765625</x:v>
-      </x:c>
-      <x:c r="I22" s="9" t="n">
-        <x:f>G22*'KV明细'!$K$5</x:f>
-        <x:v>2232.4338612556458</x:v>
-      </x:c>
-      <x:c r="J22" s="9" t="n">
-        <x:f>H22*'KV明细'!$K$5</x:f>
-        <x:v>35.3916015625</x:v>
-      </x:c>
-      <x:c r="K22" s="9" t="n">
-        <x:f>I22*D22</x:f>
-        <x:v>8929.735445022583</x:v>
-      </x:c>
-      <x:c r="L22" s="9" t="n">
-        <x:f>J22*D22</x:f>
-        <x:v>141.56640625</x:v>
-      </x:c>
-      <x:c r="M22" s="2" t="str">
-        <x:f>IF('EP通信'!H10&gt;0,"需补齐128槽并验证EPLB","专家数整除；未实机验证")</x:f>
-        <x:v>专家数整除；未实机验证</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="25" customHeight="1">
-      <x:c r="A23" s="2" t="str">
-        <x:f>'EP通信'!A11</x:f>
-        <x:v>DS V4 10T</x:v>
-      </x:c>
-      <x:c r="B23" s="2" t="n">
-        <x:f>'EP通信'!B11</x:f>
-        <x:v>256</x:v>
-      </x:c>
-      <x:c r="C23" s="2" t="n">
-        <x:f>'EP通信'!I11</x:f>
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="D23" s="2" t="n">
-        <x:f>B23/C23</x:f>
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="E23" s="2" t="n">
-        <x:f>'EP通信'!J11</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F23" s="2" t="n">
-        <x:f>B23/E23</x:f>
-        <x:v>256</x:v>
-      </x:c>
-      <x:c r="G23" s="9" t="n">
-        <x:f>'KV明细'!J16</x:f>
-        <x:v>139.52711632847786</x:v>
-      </x:c>
-      <x:c r="H23" s="9" t="n">
-        <x:f>'KV明细'!L16</x:f>
-        <x:v>2.21197509765625</x:v>
-      </x:c>
-      <x:c r="I23" s="9" t="n">
-        <x:f>G23*'KV明细'!$K$5</x:f>
-        <x:v>2232.4338612556458</x:v>
-      </x:c>
-      <x:c r="J23" s="9" t="n">
-        <x:f>H23*'KV明细'!$K$5</x:f>
-        <x:v>35.3916015625</x:v>
-      </x:c>
-      <x:c r="K23" s="9" t="n">
-        <x:f>I23*D23</x:f>
-        <x:v>71437.88356018066</x:v>
-      </x:c>
-      <x:c r="L23" s="9" t="n">
-        <x:f>J23*D23</x:f>
-        <x:v>1132.53125</x:v>
-      </x:c>
-      <x:c r="M23" s="2" t="str">
-        <x:f>IF('EP通信'!H11&gt;0,"需补齐128槽并验证EPLB","专家数整除；未实机验证")</x:f>
-        <x:v>需补齐128槽并验证EPLB</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="25" customHeight="1">
-      <x:c r="A24" s="2" t="str">
-        <x:f>'EP通信'!A12</x:f>
-        <x:v>DS V4 Pro</x:v>
-      </x:c>
-      <x:c r="B24" s="2" t="n">
-        <x:f>'EP通信'!B12</x:f>
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="C24" s="2" t="n">
-        <x:f>'EP通信'!I12</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D24" s="2" t="n">
@@ -1258,7 +1266,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="E24" s="2" t="n">
-        <x:f>'EP通信'!J12</x:f>
+        <x:f>'EP通信'!J10</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="F24" s="2" t="n">
@@ -1266,11 +1274,11 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="G24" s="9" t="n">
-        <x:f>'KV明细'!J25</x:f>
+        <x:f>'KV明细'!J16</x:f>
         <x:v>139.52711632847786</x:v>
       </x:c>
       <x:c r="H24" s="9" t="n">
-        <x:f>'KV明细'!L25</x:f>
+        <x:f>'KV明细'!L16</x:f>
         <x:v>2.21197509765625</x:v>
       </x:c>
       <x:c r="I24" s="9" t="n">
@@ -1290,21 +1298,21 @@
         <x:v>141.56640625</x:v>
       </x:c>
       <x:c r="M24" s="2" t="str">
-        <x:f>IF('EP通信'!H12&gt;0,"需补齐128槽并验证EPLB","专家数整除；未实机验证")</x:f>
+        <x:f>IF('EP通信'!H10&gt;0,"需补齐128槽并验证EPLB","专家数整除；未实机验证")</x:f>
         <x:v>专家数整除；未实机验证</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="25" customHeight="1">
       <x:c r="A25" s="2" t="str">
-        <x:f>'EP通信'!A13</x:f>
-        <x:v>DS V4 Pro</x:v>
+        <x:f>'EP通信'!A11</x:f>
+        <x:v>DS V4 10T</x:v>
       </x:c>
       <x:c r="B25" s="2" t="n">
-        <x:f>'EP通信'!B13</x:f>
+        <x:f>'EP通信'!B11</x:f>
         <x:v>256</x:v>
       </x:c>
       <x:c r="C25" s="2" t="n">
-        <x:f>'EP通信'!I13</x:f>
+        <x:f>'EP通信'!I11</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D25" s="2" t="n">
@@ -1312,7 +1320,7 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="E25" s="2" t="n">
-        <x:f>'EP通信'!J13</x:f>
+        <x:f>'EP通信'!J11</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="F25" s="2" t="n">
@@ -1320,11 +1328,11 @@
         <x:v>256</x:v>
       </x:c>
       <x:c r="G25" s="9" t="n">
-        <x:f>'KV明细'!J25</x:f>
+        <x:f>'KV明细'!J16</x:f>
         <x:v>139.52711632847786</x:v>
       </x:c>
       <x:c r="H25" s="9" t="n">
-        <x:f>'KV明细'!L25</x:f>
+        <x:f>'KV明细'!L16</x:f>
         <x:v>2.21197509765625</x:v>
       </x:c>
       <x:c r="I25" s="9" t="n">
@@ -1344,21 +1352,21 @@
         <x:v>1132.53125</x:v>
       </x:c>
       <x:c r="M25" s="2" t="str">
-        <x:f>IF('EP通信'!H13&gt;0,"需补齐128槽并验证EPLB","专家数整除；未实机验证")</x:f>
+        <x:f>IF('EP通信'!H11&gt;0,"需补齐128槽并验证EPLB","专家数整除；未实机验证")</x:f>
         <x:v>需补齐128槽并验证EPLB</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="25" customHeight="1">
       <x:c r="A26" s="2" t="str">
-        <x:f>'EP通信'!A14</x:f>
-        <x:v>GLM5.3</x:v>
+        <x:f>'EP通信'!A12</x:f>
+        <x:v>DS V4 Pro</x:v>
       </x:c>
       <x:c r="B26" s="2" t="n">
-        <x:f>'EP通信'!B14</x:f>
+        <x:f>'EP通信'!B12</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="C26" s="2" t="n">
-        <x:f>'EP通信'!I14</x:f>
+        <x:f>'EP通信'!I12</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D26" s="2" t="n">
@@ -1366,7 +1374,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="E26" s="2" t="n">
-        <x:f>'EP通信'!J14</x:f>
+        <x:f>'EP通信'!J12</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="F26" s="2" t="n">
@@ -1374,45 +1382,45 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="G26" s="9" t="n">
-        <x:f>'KV明细'!J29</x:f>
-        <x:v>186</x:v>
+        <x:f>'KV明细'!J25</x:f>
+        <x:v>139.52711632847786</x:v>
       </x:c>
       <x:c r="H26" s="9" t="n">
-        <x:f>'KV明细'!L29</x:f>
-        <x:v>23.25</x:v>
+        <x:f>'KV明细'!L25</x:f>
+        <x:v>2.21197509765625</x:v>
       </x:c>
       <x:c r="I26" s="9" t="n">
         <x:f>G26*'KV明细'!$K$5</x:f>
-        <x:v>2976</x:v>
+        <x:v>2232.4338612556458</x:v>
       </x:c>
       <x:c r="J26" s="9" t="n">
         <x:f>H26*'KV明细'!$K$5</x:f>
-        <x:v>372</x:v>
+        <x:v>35.3916015625</x:v>
       </x:c>
       <x:c r="K26" s="9" t="n">
         <x:f>I26*D26</x:f>
-        <x:v>11904</x:v>
+        <x:v>8929.735445022583</x:v>
       </x:c>
       <x:c r="L26" s="9" t="n">
         <x:f>J26*D26</x:f>
-        <x:v>1488</x:v>
+        <x:v>141.56640625</x:v>
       </x:c>
       <x:c r="M26" s="2" t="str">
-        <x:f>IF('EP通信'!H14&gt;0,"需补齐128槽并验证EPLB","专家数整除；未实机验证")</x:f>
+        <x:f>IF('EP通信'!H12&gt;0,"需补齐128槽并验证EPLB","专家数整除；未实机验证")</x:f>
         <x:v>专家数整除；未实机验证</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="25" customHeight="1">
       <x:c r="A27" s="2" t="str">
-        <x:f>'EP通信'!A15</x:f>
-        <x:v>GLM5.3</x:v>
+        <x:f>'EP通信'!A13</x:f>
+        <x:v>DS V4 Pro</x:v>
       </x:c>
       <x:c r="B27" s="2" t="n">
-        <x:f>'EP通信'!B15</x:f>
+        <x:f>'EP通信'!B13</x:f>
         <x:v>256</x:v>
       </x:c>
       <x:c r="C27" s="2" t="n">
-        <x:f>'EP通信'!I15</x:f>
+        <x:f>'EP通信'!I13</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D27" s="2" t="n">
@@ -1420,7 +1428,7 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="E27" s="2" t="n">
-        <x:f>'EP通信'!J15</x:f>
+        <x:f>'EP通信'!J13</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="F27" s="2" t="n">
@@ -1428,45 +1436,45 @@
         <x:v>256</x:v>
       </x:c>
       <x:c r="G27" s="9" t="n">
-        <x:f>'KV明细'!J29</x:f>
-        <x:v>186</x:v>
+        <x:f>'KV明细'!J25</x:f>
+        <x:v>139.52711632847786</x:v>
       </x:c>
       <x:c r="H27" s="9" t="n">
-        <x:f>'KV明细'!L29</x:f>
-        <x:v>23.25</x:v>
+        <x:f>'KV明细'!L25</x:f>
+        <x:v>2.21197509765625</x:v>
       </x:c>
       <x:c r="I27" s="9" t="n">
         <x:f>G27*'KV明细'!$K$5</x:f>
-        <x:v>2976</x:v>
+        <x:v>2232.4338612556458</x:v>
       </x:c>
       <x:c r="J27" s="9" t="n">
         <x:f>H27*'KV明细'!$K$5</x:f>
-        <x:v>372</x:v>
+        <x:v>35.3916015625</x:v>
       </x:c>
       <x:c r="K27" s="9" t="n">
         <x:f>I27*D27</x:f>
-        <x:v>95232</x:v>
+        <x:v>71437.88356018066</x:v>
       </x:c>
       <x:c r="L27" s="9" t="n">
         <x:f>J27*D27</x:f>
-        <x:v>11904</x:v>
+        <x:v>1132.53125</x:v>
       </x:c>
       <x:c r="M27" s="2" t="str">
-        <x:f>IF('EP通信'!H15&gt;0,"需补齐128槽并验证EPLB","专家数整除；未实机验证")</x:f>
-        <x:v>专家数整除；未实机验证</x:v>
+        <x:f>IF('EP通信'!H13&gt;0,"需补齐128槽并验证EPLB","专家数整除；未实机验证")</x:f>
+        <x:v>需补齐128槽并验证EPLB</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="25" customHeight="1">
       <x:c r="A28" s="2" t="str">
-        <x:f>'EP通信'!A16</x:f>
-        <x:v>KimiK3</x:v>
+        <x:f>'EP通信'!A14</x:f>
+        <x:v>GLM5.3</x:v>
       </x:c>
       <x:c r="B28" s="2" t="n">
-        <x:f>'EP通信'!B16</x:f>
+        <x:f>'EP通信'!B14</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="C28" s="2" t="n">
-        <x:f>'EP通信'!I16</x:f>
+        <x:f>'EP通信'!I14</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D28" s="2" t="n">
@@ -1474,53 +1482,53 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="E28" s="2" t="n">
-        <x:f>'EP通信'!J16</x:f>
-        <x:v>8</x:v>
+        <x:f>'EP通信'!J14</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F28" s="2" t="n">
         <x:f>B28/E28</x:f>
-        <x:v>4</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="G28" s="9" t="n">
-        <x:f>'KV明细'!J34</x:f>
-        <x:v>54.418304443359375</x:v>
+        <x:f>'KV明细'!J29</x:f>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="H28" s="9" t="n">
-        <x:f>'KV明细'!L34</x:f>
-        <x:v>54.45167541503906</x:v>
+        <x:f>'KV明细'!L29</x:f>
+        <x:v>23.25</x:v>
       </x:c>
       <x:c r="I28" s="9" t="n">
         <x:f>G28*'KV明细'!$K$5</x:f>
-        <x:v>870.69287109375</x:v>
+        <x:v>2976</x:v>
       </x:c>
       <x:c r="J28" s="9" t="n">
         <x:f>H28*'KV明细'!$K$5</x:f>
-        <x:v>871.226806640625</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="K28" s="9" t="n">
         <x:f>I28*D28</x:f>
-        <x:v>3482.771484375</x:v>
+        <x:v>11904</x:v>
       </x:c>
       <x:c r="L28" s="9" t="n">
         <x:f>J28*D28</x:f>
-        <x:v>3484.9072265625</x:v>
+        <x:v>1488</x:v>
       </x:c>
       <x:c r="M28" s="2" t="str">
-        <x:f>IF('EP通信'!H16&gt;0,"需补齐128槽并验证EPLB","专家数整除；未实机验证")</x:f>
+        <x:f>IF('EP通信'!H14&gt;0,"需补齐128槽并验证EPLB","专家数整除；未实机验证")</x:f>
         <x:v>专家数整除；未实机验证</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="25" customHeight="1">
       <x:c r="A29" s="2" t="str">
-        <x:f>'EP通信'!A17</x:f>
-        <x:v>KimiK3</x:v>
+        <x:f>'EP通信'!A15</x:f>
+        <x:v>GLM5.3</x:v>
       </x:c>
       <x:c r="B29" s="2" t="n">
-        <x:f>'EP通信'!B17</x:f>
+        <x:f>'EP通信'!B15</x:f>
         <x:v>256</x:v>
       </x:c>
       <x:c r="C29" s="2" t="n">
-        <x:f>'EP通信'!I17</x:f>
+        <x:f>'EP通信'!I15</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D29" s="2" t="n">
@@ -1528,53 +1536,53 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="E29" s="2" t="n">
-        <x:f>'EP通信'!J17</x:f>
-        <x:v>8</x:v>
+        <x:f>'EP通信'!J15</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F29" s="2" t="n">
         <x:f>B29/E29</x:f>
-        <x:v>32</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="G29" s="9" t="n">
-        <x:f>'KV明细'!J34</x:f>
-        <x:v>54.418304443359375</x:v>
+        <x:f>'KV明细'!J29</x:f>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="H29" s="9" t="n">
-        <x:f>'KV明细'!L34</x:f>
-        <x:v>54.45167541503906</x:v>
+        <x:f>'KV明细'!L29</x:f>
+        <x:v>23.25</x:v>
       </x:c>
       <x:c r="I29" s="9" t="n">
         <x:f>G29*'KV明细'!$K$5</x:f>
-        <x:v>870.69287109375</x:v>
+        <x:v>2976</x:v>
       </x:c>
       <x:c r="J29" s="9" t="n">
         <x:f>H29*'KV明细'!$K$5</x:f>
-        <x:v>871.226806640625</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="K29" s="9" t="n">
         <x:f>I29*D29</x:f>
-        <x:v>27862.171875</x:v>
+        <x:v>95232</x:v>
       </x:c>
       <x:c r="L29" s="9" t="n">
         <x:f>J29*D29</x:f>
-        <x:v>27879.2578125</x:v>
+        <x:v>11904</x:v>
       </x:c>
       <x:c r="M29" s="2" t="str">
-        <x:f>IF('EP通信'!H17&gt;0,"需补齐128槽并验证EPLB","专家数整除；未实机验证")</x:f>
-        <x:v>需补齐128槽并验证EPLB</x:v>
+        <x:f>IF('EP通信'!H15&gt;0,"需补齐128槽并验证EPLB","专家数整除；未实机验证")</x:f>
+        <x:v>专家数整除；未实机验证</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="25" customHeight="1">
       <x:c r="A30" s="2" t="str">
-        <x:f>'EP通信'!A18</x:f>
-        <x:v>Qwen3.8 2.4T</x:v>
+        <x:f>'EP通信'!A16</x:f>
+        <x:v>KimiK3</x:v>
       </x:c>
       <x:c r="B30" s="2" t="n">
-        <x:f>'EP通信'!B18</x:f>
+        <x:f>'EP通信'!B16</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="C30" s="2" t="n">
-        <x:f>'EP通信'!I18</x:f>
+        <x:f>'EP通信'!I16</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D30" s="2" t="n">
@@ -1582,7 +1590,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="E30" s="2" t="n">
-        <x:f>'EP通信'!J18</x:f>
+        <x:f>'EP通信'!J16</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="F30" s="2" t="n">
@@ -1590,45 +1598,45 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G30" s="9" t="n">
-        <x:f>'KV明细'!J39</x:f>
-        <x:v>46.546783447265625</x:v>
+        <x:f>'KV明细'!J34</x:f>
+        <x:v>54.418304443359375</x:v>
       </x:c>
       <x:c r="H30" s="9" t="n">
-        <x:f>'KV明细'!L39</x:f>
-        <x:v>46.56538391113281</x:v>
+        <x:f>'KV明细'!L34</x:f>
+        <x:v>54.45167541503906</x:v>
       </x:c>
       <x:c r="I30" s="9" t="n">
         <x:f>G30*'KV明细'!$K$5</x:f>
-        <x:v>744.74853515625</x:v>
+        <x:v>870.69287109375</x:v>
       </x:c>
       <x:c r="J30" s="9" t="n">
         <x:f>H30*'KV明细'!$K$5</x:f>
-        <x:v>745.046142578125</x:v>
+        <x:v>871.226806640625</x:v>
       </x:c>
       <x:c r="K30" s="9" t="n">
         <x:f>I30*D30</x:f>
-        <x:v>2978.994140625</x:v>
+        <x:v>3482.771484375</x:v>
       </x:c>
       <x:c r="L30" s="9" t="n">
         <x:f>J30*D30</x:f>
-        <x:v>2980.1845703125</x:v>
+        <x:v>3484.9072265625</x:v>
       </x:c>
       <x:c r="M30" s="2" t="str">
-        <x:f>IF('EP通信'!H18&gt;0,"需补齐128槽并验证EPLB","专家数整除；未实机验证")</x:f>
+        <x:f>IF('EP通信'!H16&gt;0,"需补齐128槽并验证EPLB","专家数整除；未实机验证")</x:f>
         <x:v>专家数整除；未实机验证</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="25" customHeight="1">
       <x:c r="A31" s="2" t="str">
-        <x:f>'EP通信'!A19</x:f>
-        <x:v>Qwen3.8 2.4T</x:v>
+        <x:f>'EP通信'!A17</x:f>
+        <x:v>KimiK3</x:v>
       </x:c>
       <x:c r="B31" s="2" t="n">
-        <x:f>'EP通信'!B19</x:f>
+        <x:f>'EP通信'!B17</x:f>
         <x:v>256</x:v>
       </x:c>
       <x:c r="C31" s="2" t="n">
-        <x:f>'EP通信'!I19</x:f>
+        <x:f>'EP通信'!I17</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D31" s="2" t="n">
@@ -1636,7 +1644,7 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="E31" s="2" t="n">
-        <x:f>'EP通信'!J19</x:f>
+        <x:f>'EP通信'!J17</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="F31" s="2" t="n">
@@ -1644,101 +1652,252 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="G31" s="9" t="n">
+        <x:f>'KV明细'!J34</x:f>
+        <x:v>54.418304443359375</x:v>
+      </x:c>
+      <x:c r="H31" s="9" t="n">
+        <x:f>'KV明细'!L34</x:f>
+        <x:v>54.45167541503906</x:v>
+      </x:c>
+      <x:c r="I31" s="9" t="n">
+        <x:f>G31*'KV明细'!$K$5</x:f>
+        <x:v>870.69287109375</x:v>
+      </x:c>
+      <x:c r="J31" s="9" t="n">
+        <x:f>H31*'KV明细'!$K$5</x:f>
+        <x:v>871.226806640625</x:v>
+      </x:c>
+      <x:c r="K31" s="9" t="n">
+        <x:f>I31*D31</x:f>
+        <x:v>27862.171875</x:v>
+      </x:c>
+      <x:c r="L31" s="9" t="n">
+        <x:f>J31*D31</x:f>
+        <x:v>27879.2578125</x:v>
+      </x:c>
+      <x:c r="M31" s="2" t="str">
+        <x:f>IF('EP通信'!H17&gt;0,"需补齐128槽并验证EPLB","专家数整除；未实机验证")</x:f>
+        <x:v>需补齐128槽并验证EPLB</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="25" customHeight="1">
+      <x:c r="A32" s="2" t="str">
+        <x:f>'EP通信'!A18</x:f>
+        <x:v>Qwen3.8 2.4T</x:v>
+      </x:c>
+      <x:c r="B32" s="2" t="n">
+        <x:f>'EP通信'!B18</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C32" s="2" t="n">
+        <x:f>'EP通信'!I18</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D32" s="2" t="n">
+        <x:f>B32/C32</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E32" s="2" t="n">
+        <x:f>'EP通信'!J18</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F32" s="2" t="n">
+        <x:f>B32/E32</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G32" s="9" t="n">
         <x:f>'KV明细'!J39</x:f>
         <x:v>46.546783447265625</x:v>
       </x:c>
-      <x:c r="H31" s="9" t="n">
+      <x:c r="H32" s="9" t="n">
         <x:f>'KV明细'!L39</x:f>
         <x:v>46.56538391113281</x:v>
       </x:c>
-      <x:c r="I31" s="9" t="n">
-        <x:f>G31*'KV明细'!$K$5</x:f>
+      <x:c r="I32" s="9" t="n">
+        <x:f>G32*'KV明细'!$K$5</x:f>
         <x:v>744.74853515625</x:v>
       </x:c>
-      <x:c r="J31" s="9" t="n">
-        <x:f>H31*'KV明细'!$K$5</x:f>
+      <x:c r="J32" s="9" t="n">
+        <x:f>H32*'KV明细'!$K$5</x:f>
         <x:v>745.046142578125</x:v>
       </x:c>
-      <x:c r="K31" s="9" t="n">
-        <x:f>I31*D31</x:f>
+      <x:c r="K32" s="9" t="n">
+        <x:f>I32*D32</x:f>
+        <x:v>2978.994140625</x:v>
+      </x:c>
+      <x:c r="L32" s="9" t="n">
+        <x:f>J32*D32</x:f>
+        <x:v>2980.1845703125</x:v>
+      </x:c>
+      <x:c r="M32" s="2" t="str">
+        <x:f>IF('EP通信'!H18&gt;0,"需补齐128槽并验证EPLB","专家数整除；未实机验证")</x:f>
+        <x:v>专家数整除；未实机验证</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="25" customHeight="1">
+      <x:c r="A33" s="2" t="str">
+        <x:f>'EP通信'!A19</x:f>
+        <x:v>Qwen3.8 2.4T</x:v>
+      </x:c>
+      <x:c r="B33" s="2" t="n">
+        <x:f>'EP通信'!B19</x:f>
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="C33" s="2" t="n">
+        <x:f>'EP通信'!I19</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D33" s="2" t="n">
+        <x:f>B33/C33</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="E33" s="2" t="n">
+        <x:f>'EP通信'!J19</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F33" s="2" t="n">
+        <x:f>B33/E33</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="G33" s="9" t="n">
+        <x:f>'KV明细'!J39</x:f>
+        <x:v>46.546783447265625</x:v>
+      </x:c>
+      <x:c r="H33" s="9" t="n">
+        <x:f>'KV明细'!L39</x:f>
+        <x:v>46.56538391113281</x:v>
+      </x:c>
+      <x:c r="I33" s="9" t="n">
+        <x:f>G33*'KV明细'!$K$5</x:f>
+        <x:v>744.74853515625</x:v>
+      </x:c>
+      <x:c r="J33" s="9" t="n">
+        <x:f>H33*'KV明细'!$K$5</x:f>
+        <x:v>745.046142578125</x:v>
+      </x:c>
+      <x:c r="K33" s="9" t="n">
+        <x:f>I33*D33</x:f>
         <x:v>23831.953125</x:v>
       </x:c>
-      <x:c r="L31" s="9" t="n">
-        <x:f>J31*D31</x:f>
+      <x:c r="L33" s="9" t="n">
+        <x:f>J33*D33</x:f>
         <x:v>23841.4765625</x:v>
       </x:c>
-      <x:c r="M31" s="2" t="str">
+      <x:c r="M33" s="2" t="str">
         <x:f>IF('EP通信'!H19&gt;0,"需补齐128槽并验证EPLB","专家数整除；未实机验证")</x:f>
         <x:v>专家数整除；未实机验证</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="25" customHeight="1">
-      <x:c r="A32" s="2"/>
-      <x:c r="B32" s="2"/>
-      <x:c r="C32" s="2"/>
-      <x:c r="D32" s="2"/>
-      <x:c r="E32" s="2"/>
-      <x:c r="F32" s="2"/>
-      <x:c r="G32" s="2"/>
-      <x:c r="H32" s="2"/>
-      <x:c r="I32" s="2"/>
-      <x:c r="J32" s="2"/>
-      <x:c r="K32" s="2"/>
-      <x:c r="L32" s="2"/>
-      <x:c r="M32" s="2"/>
-    </x:row>
-    <x:row r="33" ht="25" customHeight="1">
-      <x:c r="A33" s="2"/>
-      <x:c r="B33" s="2"/>
-      <x:c r="C33" s="2"/>
-      <x:c r="D33" s="2"/>
-      <x:c r="E33" s="2"/>
-      <x:c r="F33" s="2"/>
-      <x:c r="G33" s="2"/>
-      <x:c r="H33" s="2"/>
-      <x:c r="I33" s="2"/>
-      <x:c r="J33" s="2"/>
-      <x:c r="K33" s="2"/>
-      <x:c r="L33" s="2"/>
-      <x:c r="M33" s="2"/>
-    </x:row>
     <x:row r="34" ht="25" customHeight="1">
       <x:c r="A34" s="2" t="str">
-        <x:v>EP256 条件：DS V4 / Kimi 需补齐 128 个物理专家槽并验证 EPLB；未改模型 checkpoint。</x:v>
-      </x:c>
-      <x:c r="B34" s="2"/>
-      <x:c r="C34" s="2"/>
-      <x:c r="D34" s="2"/>
-      <x:c r="E34" s="2"/>
-      <x:c r="F34" s="2"/>
-      <x:c r="G34" s="2"/>
-      <x:c r="H34" s="2"/>
-      <x:c r="I34" s="2"/>
-      <x:c r="J34" s="2"/>
-      <x:c r="K34" s="2"/>
-      <x:c r="L34" s="2"/>
-      <x:c r="M34" s="2"/>
+        <x:f>'EP通信'!A20</x:f>
+        <x:v>DS V4.1 Flash</x:v>
+      </x:c>
+      <x:c r="B34" s="2" t="n">
+        <x:f>'EP通信'!B20</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C34" s="2" t="n">
+        <x:f>'EP通信'!I20</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D34" s="2" t="n">
+        <x:f>B34/C34</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E34" s="2" t="n">
+        <x:f>'EP通信'!J20</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F34" s="2" t="n">
+        <x:f>B34/E34</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="G34" s="9" t="n">
+        <x:f>'KV明细'!J47</x:f>
+        <x:v>85.6376953125</x:v>
+      </x:c>
+      <x:c r="H34" s="16" t="n">
+        <x:f>'KV明细'!L47</x:f>
+        <x:v>0.7144775390625</x:v>
+      </x:c>
+      <x:c r="I34" s="9" t="n">
+        <x:f>G34*'KV明细'!$K$5</x:f>
+        <x:v>1370.203125</x:v>
+      </x:c>
+      <x:c r="J34" s="16" t="n">
+        <x:f>H34*'KV明细'!$K$5</x:f>
+        <x:v>11.431640625</x:v>
+      </x:c>
+      <x:c r="K34" s="9" t="n">
+        <x:f>I34*D34</x:f>
+        <x:v>5480.8125</x:v>
+      </x:c>
+      <x:c r="L34" s="16" t="n">
+        <x:f>J34*D34</x:f>
+        <x:v>45.7265625</x:v>
+      </x:c>
+      <x:c r="M34" s="2" t="str">
+        <x:f>IF('EP通信'!H20&gt;0,"补128槽并验证；取为规划值","取为规划值；迁移未支持")</x:f>
+        <x:v>取为规划值；迁移未支持</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="25" customHeight="1">
-      <x:c r="A35" s="2"/>
-      <x:c r="B35" s="2"/>
-      <x:c r="C35" s="2"/>
-      <x:c r="D35" s="2"/>
-      <x:c r="E35" s="2"/>
-      <x:c r="F35" s="2"/>
-      <x:c r="G35" s="2"/>
-      <x:c r="H35" s="2"/>
-      <x:c r="I35" s="2"/>
-      <x:c r="J35" s="2"/>
-      <x:c r="K35" s="2"/>
-      <x:c r="L35" s="2"/>
-      <x:c r="M35" s="2"/>
+      <x:c r="A35" s="2" t="str">
+        <x:f>'EP通信'!A21</x:f>
+        <x:v>DS V4.1 Flash</x:v>
+      </x:c>
+      <x:c r="B35" s="2" t="n">
+        <x:f>'EP通信'!B21</x:f>
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="C35" s="2" t="n">
+        <x:f>'EP通信'!I21</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D35" s="2" t="n">
+        <x:f>B35/C35</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="E35" s="2" t="n">
+        <x:f>'EP通信'!J21</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F35" s="2" t="n">
+        <x:f>B35/E35</x:f>
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G35" s="9" t="n">
+        <x:f>'KV明细'!J47</x:f>
+        <x:v>85.6376953125</x:v>
+      </x:c>
+      <x:c r="H35" s="16" t="n">
+        <x:f>'KV明细'!L47</x:f>
+        <x:v>0.7144775390625</x:v>
+      </x:c>
+      <x:c r="I35" s="9" t="n">
+        <x:f>G35*'KV明细'!$K$5</x:f>
+        <x:v>1370.203125</x:v>
+      </x:c>
+      <x:c r="J35" s="16" t="n">
+        <x:f>H35*'KV明细'!$K$5</x:f>
+        <x:v>11.431640625</x:v>
+      </x:c>
+      <x:c r="K35" s="9" t="n">
+        <x:f>I35*D35</x:f>
+        <x:v>43846.5</x:v>
+      </x:c>
+      <x:c r="L35" s="16" t="n">
+        <x:f>J35*D35</x:f>
+        <x:v>365.8125</x:v>
+      </x:c>
+      <x:c r="M35" s="2" t="str">
+        <x:f>IF('EP通信'!H21&gt;0,"补128槽并验证；取为规划值","取为规划值；迁移未支持")</x:f>
+        <x:v>补128槽并验证；取为规划值</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="25" customHeight="1">
-      <x:c r="A36" s="2" t="str">
-        <x:f>"P 整组批次：EP32 为 "&amp;'KV明细'!$K$5*4&amp;" 请求，EP256 为 "&amp;'KV明细'!$K$5*32&amp;" 请求；单请求 KV 不随 EP 改变。"</x:f>
-        <x:v>P 整组批次：EP32 为 64 请求，EP256 为 512 请求；单请求 KV 不随 EP 改变。</x:v>
-      </x:c>
+      <x:c r="A36" s="2"/>
       <x:c r="B36" s="2"/>
       <x:c r="C36" s="2"/>
       <x:c r="D36" s="2"/>
@@ -1769,7 +1928,7 @@
     </x:row>
     <x:row r="38" ht="25" customHeight="1">
       <x:c r="A38" s="2" t="str">
-        <x:v>DS 存量含整个 prompt 生成的 SWA 行；阶段末常驻量见 KV 明细，不能按生成量配 HBM。</x:v>
+        <x:v>EP256 条件：DS V4 / V4.1 / Kimi 需补齐 128 个物理专家槽并验证 EPLB；未改模型 checkpoint。</x:v>
       </x:c>
       <x:c r="B38" s="2"/>
       <x:c r="C38" s="2"/>
@@ -1801,7 +1960,8 @@
     </x:row>
     <x:row r="40" ht="25" customHeight="1">
       <x:c r="A40" s="2" t="str">
-        <x:v>MC2 未计轮询读、重试和物理协议开销；不是整机 HBM 访存或 RoCE/HCCS 实测总量。</x:v>
+        <x:f>"P 整组批次：EP32 为 "&amp;'KV明细'!$K$5*4&amp;" 请求，EP256 为 "&amp;'KV明细'!$K$5*32&amp;" 请求；单请求 KV 不随 EP 改变。"</x:f>
+        <x:v>P 整组批次：EP32 为 64 请求，EP256 为 512 请求；单请求 KV 不随 EP 改变。</x:v>
       </x:c>
       <x:c r="B40" s="2"/>
       <x:c r="C40" s="2"/>
@@ -1833,7 +1993,7 @@
     </x:row>
     <x:row r="42" ht="25" customHeight="1">
       <x:c r="A42" s="2" t="str">
-        <x:v>黄色输入可编辑；参数、公式与源码说明见 KV明细、EP通信及 analysis/KV-EP-SPECS.md。</x:v>
+        <x:v>DS 存量含整个 prompt 生成的 SWA 行；阶段末常驻量见 KV 明细，不能按生成量配 HBM。</x:v>
       </x:c>
       <x:c r="B42" s="2"/>
       <x:c r="C42" s="2"/>
@@ -1864,7 +2024,9 @@
       <x:c r="M43" s="2"/>
     </x:row>
     <x:row r="44" ht="25" customHeight="1">
-      <x:c r="A44" s="2"/>
+      <x:c r="A44" s="2" t="str">
+        <x:v>V4.1：完成 S tokens 后交接；长 KV / Indexer 只计 4 个源层，SWA 尾块和 32 行环形页按规划传输。</x:v>
+      </x:c>
       <x:c r="B44" s="2"/>
       <x:c r="C44" s="2"/>
       <x:c r="D44" s="2"/>
@@ -1894,7 +2056,9 @@
       <x:c r="M45" s="2"/>
     </x:row>
     <x:row r="46" ht="25" customHeight="1">
-      <x:c r="A46" s="2"/>
+      <x:c r="A46" s="2" t="str">
+        <x:v>MC2 未计轮询读、重试和物理协议开销；V4.1 Engram 通信另见模型分析，未叠加进 MoE EP。</x:v>
+      </x:c>
       <x:c r="B46" s="2"/>
       <x:c r="C46" s="2"/>
       <x:c r="D46" s="2"/>
@@ -1924,7 +2088,9 @@
       <x:c r="M47" s="2"/>
     </x:row>
     <x:row r="48" ht="25" customHeight="1">
-      <x:c r="A48" s="2"/>
+      <x:c r="A48" s="2" t="str">
+        <x:v>黄色输入可编辑；主干层，不含 draft/MTP；参数、公式与源码说明见明细及 analysis/KV-EP-SPECS.md。</x:v>
+      </x:c>
       <x:c r="B48" s="2"/>
       <x:c r="C48" s="2"/>
       <x:c r="D48" s="2"/>
@@ -2214,7 +2380,7 @@
     <x:col min="10" max="10" width="15" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="15" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="15" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="15" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="30" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="25" customHeight="1">
@@ -2362,7 +2528,7 @@
         <x:v>P 保留行</x:v>
       </x:c>
       <x:c r="G8" s="7" t="str">
-        <x:v>D 拉取行</x:v>
+        <x:v>D 取/规划行</x:v>
       </x:c>
       <x:c r="H8" s="7" t="str">
         <x:v>P 副本/分片</x:v>
@@ -2377,7 +2543,7 @@
         <x:v>保留 GiB</x:v>
       </x:c>
       <x:c r="L8" s="7" t="str">
-        <x:v>取 GiB</x:v>
+        <x:v>取/规划 GiB</x:v>
       </x:c>
       <x:c r="M8" s="2"/>
     </x:row>
@@ -3587,114 +3753,313 @@
       <x:c r="M40" s="2"/>
     </x:row>
     <x:row r="41" ht="25" customHeight="1">
-      <x:c r="A41" s="2"/>
-      <x:c r="B41" s="2"/>
-      <x:c r="C41" s="8"/>
-      <x:c r="D41" s="8"/>
-      <x:c r="E41" s="8"/>
-      <x:c r="F41" s="8"/>
-      <x:c r="G41" s="8"/>
-      <x:c r="H41" s="8"/>
-      <x:c r="I41" s="8"/>
-      <x:c r="J41" s="12"/>
-      <x:c r="K41" s="12"/>
-      <x:c r="L41" s="12"/>
-      <x:c r="M41" s="2"/>
+      <x:c r="A41" s="2" t="str">
+        <x:v>DS V4.1 Flash</x:v>
+      </x:c>
+      <x:c r="B41" s="2" t="str">
+        <x:v>SWA KV / BF16</x:v>
+      </x:c>
+      <x:c r="C41" s="8" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="D41" s="8" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="E41" s="8" t="n">
+        <x:f>$B$5</x:f>
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="F41" s="8" t="n">
+        <x:f>MIN($B$5,128)</x:f>
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="G41" s="8" t="n">
+        <x:f>MIN(ROUNDUP($B$5/$E$5,0),ROUNDUP(128/$E$5,0)+1)*$E$5</x:f>
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="H41" s="8" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I41" s="8" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J41" s="12" t="n">
+        <x:f>C41*D41*E41*H41/2^30</x:f>
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="K41" s="12" t="n">
+        <x:f>C41*D41*F41*H41/2^30</x:f>
+        <x:v>0.0390625</x:v>
+      </x:c>
+      <x:c r="L41" s="12" t="n">
+        <x:f>C41*D41*G41*I41/2^30</x:f>
+        <x:v>0.009765625</x:v>
+      </x:c>
+      <x:c r="M41" s="2" t="str">
+        <x:v>迁移未支持；取为规划值</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="25" customHeight="1">
       <x:c r="A42" s="2" t="str">
-        <x:v>实现：MooncakeConnector；P/D 同 block size、同 speculative 配置；无前缀命中、PCP/DCP=1。</x:v>
-      </x:c>
-      <x:c r="B42" s="2"/>
-      <x:c r="C42" s="8"/>
-      <x:c r="D42" s="8"/>
-      <x:c r="E42" s="8"/>
-      <x:c r="F42" s="8"/>
-      <x:c r="G42" s="8"/>
-      <x:c r="H42" s="8"/>
-      <x:c r="I42" s="8"/>
-      <x:c r="J42" s="12"/>
-      <x:c r="K42" s="12"/>
-      <x:c r="L42" s="12"/>
-      <x:c r="M42" s="2"/>
+        <x:v>DS V4.1 Flash</x:v>
+      </x:c>
+      <x:c r="B42" s="2" t="str">
+        <x:v>C2 shared KV / BF16</x:v>
+      </x:c>
+      <x:c r="C42" s="8" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D42" s="8" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="E42" s="8" t="n">
+        <x:f>INT($B$5/2)</x:f>
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="F42" s="8" t="n">
+        <x:f>INT($B$5/2)</x:f>
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G42" s="8" t="n">
+        <x:f>ROUNDUP(INT($B$5/2)/($E$5/2),0)*($E$5/2)</x:f>
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="H42" s="8" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I42" s="8" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J42" s="12" t="n">
+        <x:f>C42*D42*E42*H42/2^30</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K42" s="12" t="n">
+        <x:f>C42*D42*F42*H42/2^30</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L42" s="12" t="n">
+        <x:f>C42*D42*G42*I42/2^30</x:f>
+        <x:v>0.375</x:v>
+      </x:c>
+      <x:c r="M42" s="2" t="str">
+        <x:v>迁移未支持；取为规划值</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="25" customHeight="1">
-      <x:c r="A43" s="2"/>
-      <x:c r="B43" s="2"/>
-      <x:c r="C43" s="8"/>
-      <x:c r="D43" s="8"/>
-      <x:c r="E43" s="8"/>
-      <x:c r="F43" s="8"/>
-      <x:c r="G43" s="8"/>
-      <x:c r="H43" s="8"/>
-      <x:c r="I43" s="8"/>
-      <x:c r="J43" s="12"/>
-      <x:c r="K43" s="12"/>
-      <x:c r="L43" s="12"/>
-      <x:c r="M43" s="2"/>
+      <x:c r="A43" s="2" t="str">
+        <x:v>DS V4.1 Flash</x:v>
+      </x:c>
+      <x:c r="B43" s="2" t="str">
+        <x:v>C2 shared Indexer / INT8 + FP16 scale</x:v>
+      </x:c>
+      <x:c r="C43" s="8" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D43" s="8" t="n">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="E43" s="8" t="n">
+        <x:f>INT($B$5/2)</x:f>
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="F43" s="8" t="n">
+        <x:f>INT($B$5/2)</x:f>
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G43" s="8" t="n">
+        <x:f>ROUNDUP(INT($B$5/2)/($E$5/2),0)*($E$5/2)</x:f>
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="H43" s="8" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I43" s="8" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J43" s="12" t="n">
+        <x:f>C43*D43*E43*H43/2^30</x:f>
+        <x:v>0.380859375</x:v>
+      </x:c>
+      <x:c r="K43" s="12" t="n">
+        <x:f>C43*D43*F43*H43/2^30</x:f>
+        <x:v>0.380859375</x:v>
+      </x:c>
+      <x:c r="L43" s="12" t="n">
+        <x:f>C43*D43*G43*I43/2^30</x:f>
+        <x:v>0.047607421875</x:v>
+      </x:c>
+      <x:c r="M43" s="2" t="str">
+        <x:v>迁移未支持；取为规划值</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="25" customHeight="1">
       <x:c r="A44" s="2" t="str">
-        <x:v>GLM: 78 主干 / 21 Indexer；Kimi: 24 MLA + 69 KDA；Qwen: 23 GQA + 69 GDN。</x:v>
-      </x:c>
-      <x:c r="B44" s="2"/>
-      <x:c r="C44" s="8"/>
-      <x:c r="D44" s="8"/>
-      <x:c r="E44" s="8"/>
-      <x:c r="F44" s="8"/>
-      <x:c r="G44" s="8"/>
-      <x:c r="H44" s="8"/>
-      <x:c r="I44" s="8"/>
-      <x:c r="J44" s="12"/>
-      <x:c r="K44" s="12"/>
-      <x:c r="L44" s="12"/>
-      <x:c r="M44" s="2"/>
+        <x:v>DS V4.1 Flash</x:v>
+      </x:c>
+      <x:c r="B44" s="2" t="str">
+        <x:v>C1 shared KV / BF16</x:v>
+      </x:c>
+      <x:c r="C44" s="8" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D44" s="8" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="E44" s="8" t="n">
+        <x:f>INT($B$5/1)</x:f>
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="F44" s="8" t="n">
+        <x:f>INT($B$5/1)</x:f>
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G44" s="8" t="n">
+        <x:f>ROUNDUP(INT($B$5/1)/($E$5/1),0)*($E$5/1)</x:f>
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="H44" s="8" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I44" s="8" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J44" s="12" t="n">
+        <x:f>C44*D44*E44*H44/2^30</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K44" s="12" t="n">
+        <x:f>C44*D44*F44*H44/2^30</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L44" s="12" t="n">
+        <x:f>C44*D44*G44*I44/2^30</x:f>
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="M44" s="2" t="str">
+        <x:v>迁移未支持；取为规划值</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="25" customHeight="1">
-      <x:c r="A45" s="2"/>
-      <x:c r="B45" s="2"/>
-      <x:c r="C45" s="8"/>
-      <x:c r="D45" s="8"/>
-      <x:c r="E45" s="8"/>
-      <x:c r="F45" s="8"/>
-      <x:c r="G45" s="8"/>
-      <x:c r="H45" s="8"/>
-      <x:c r="I45" s="8"/>
-      <x:c r="J45" s="12"/>
-      <x:c r="K45" s="12"/>
-      <x:c r="L45" s="12"/>
-      <x:c r="M45" s="2"/>
+      <x:c r="A45" s="2" t="str">
+        <x:v>DS V4.1 Flash</x:v>
+      </x:c>
+      <x:c r="B45" s="2" t="str">
+        <x:v>C1 shared Indexer / INT8 + FP16 scale</x:v>
+      </x:c>
+      <x:c r="C45" s="8" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D45" s="8" t="n">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="E45" s="8" t="n">
+        <x:f>INT($B$5/1)</x:f>
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="F45" s="8" t="n">
+        <x:f>INT($B$5/1)</x:f>
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G45" s="8" t="n">
+        <x:f>ROUNDUP(INT($B$5/1)/($E$5/1),0)*($E$5/1)</x:f>
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="H45" s="8" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I45" s="8" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J45" s="12" t="n">
+        <x:f>C45*D45*E45*H45/2^30</x:f>
+        <x:v>0.25390625</x:v>
+      </x:c>
+      <x:c r="K45" s="12" t="n">
+        <x:f>C45*D45*F45*H45/2^30</x:f>
+        <x:v>0.25390625</x:v>
+      </x:c>
+      <x:c r="L45" s="12" t="n">
+        <x:f>C45*D45*G45*I45/2^30</x:f>
+        <x:v>0.03173828125</x:v>
+      </x:c>
+      <x:c r="M45" s="2" t="str">
+        <x:v>迁移未支持；取为规划值</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="25" customHeight="1">
       <x:c r="A46" s="2" t="str">
-        <x:v>来源：归档 config / VA 842b030f / vLLM c8438a3；已对照指定 main 1933f86；路径/哈希见源码清单。</x:v>
-      </x:c>
-      <x:c r="B46" s="2"/>
-      <x:c r="C46" s="8"/>
-      <x:c r="D46" s="8"/>
-      <x:c r="E46" s="8"/>
-      <x:c r="F46" s="8"/>
-      <x:c r="G46" s="8"/>
-      <x:c r="H46" s="8"/>
-      <x:c r="I46" s="8"/>
-      <x:c r="J46" s="12"/>
-      <x:c r="K46" s="12"/>
-      <x:c r="L46" s="12"/>
-      <x:c r="M46" s="2"/>
+        <x:v>DS V4.1 Flash</x:v>
+      </x:c>
+      <x:c r="B46" s="2" t="str">
+        <x:v>C2 circular ring / FP32 KV+score</x:v>
+      </x:c>
+      <x:c r="C46" s="8" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D46" s="8" t="n">
+        <x:v>4096</x:v>
+      </x:c>
+      <x:c r="E46" s="8" t="n">
+        <x:f>MIN($B$5,32)</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F46" s="8" t="n">
+        <x:f>MIN($B$5,32)</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="G46" s="8" t="n">
+        <x:f>32</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="H46" s="8" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I46" s="8" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J46" s="12" t="n">
+        <x:f>C46*D46*E46*H46/2^30</x:f>
+        <x:v>0.0029296875</x:v>
+      </x:c>
+      <x:c r="K46" s="12" t="n">
+        <x:f>C46*D46*F46*H46/2^30</x:f>
+        <x:v>0.0029296875</x:v>
+      </x:c>
+      <x:c r="L46" s="12" t="n">
+        <x:f>C46*D46*G46*I46/2^30</x:f>
+        <x:v>0.0003662109375</x:v>
+      </x:c>
+      <x:c r="M46" s="2" t="str">
+        <x:v>迁移未支持；取为规划值</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="25" customHeight="1">
-      <x:c r="A47" s="2"/>
-      <x:c r="B47" s="2"/>
-      <x:c r="C47" s="8"/>
-      <x:c r="D47" s="8"/>
-      <x:c r="E47" s="8"/>
-      <x:c r="F47" s="8"/>
-      <x:c r="G47" s="8"/>
-      <x:c r="H47" s="8"/>
-      <x:c r="I47" s="8"/>
-      <x:c r="J47" s="12"/>
-      <x:c r="K47" s="12"/>
-      <x:c r="L47" s="12"/>
+      <x:c r="A47" s="13" t="str">
+        <x:v>DS V4.1 Flash</x:v>
+      </x:c>
+      <x:c r="B47" s="13" t="str">
+        <x:v>单请求合计</x:v>
+      </x:c>
+      <x:c r="C47" s="14"/>
+      <x:c r="D47" s="14"/>
+      <x:c r="E47" s="14"/>
+      <x:c r="F47" s="14"/>
+      <x:c r="G47" s="14"/>
+      <x:c r="H47" s="14"/>
+      <x:c r="I47" s="14"/>
+      <x:c r="J47" s="15" t="n">
+        <x:f>SUM(J41:J46)</x:f>
+        <x:v>85.6376953125</x:v>
+      </x:c>
+      <x:c r="K47" s="15" t="n">
+        <x:f>SUM(K41:K46)</x:f>
+        <x:v>5.6767578125</x:v>
+      </x:c>
+      <x:c r="L47" s="15" t="n">
+        <x:f>SUM(L41:L46)</x:f>
+        <x:v>0.7144775390625</x:v>
+      </x:c>
       <x:c r="M47" s="2"/>
     </x:row>
     <x:row r="48" ht="25" customHeight="1">
@@ -3728,7 +4093,9 @@
       <x:c r="M49" s="2"/>
     </x:row>
     <x:row r="50" ht="25" customHeight="1">
-      <x:c r="A50" s="2"/>
+      <x:c r="A50" s="2" t="str">
+        <x:v>前五模型：MooncakeConnector；P/D 同 block size、同 speculative 配置；无前缀命中、PCP/DCP=1。</x:v>
+      </x:c>
       <x:c r="B50" s="2"/>
       <x:c r="C50" s="8"/>
       <x:c r="D50" s="8"/>
@@ -3758,7 +4125,9 @@
       <x:c r="M51" s="2"/>
     </x:row>
     <x:row r="52" ht="25" customHeight="1">
-      <x:c r="A52" s="2"/>
+      <x:c r="A52" s="2" t="str">
+        <x:v>GLM: 78 主干 / 21 Indexer；Kimi: 24 MLA + 69 KDA；Qwen: 23 GQA + 69 GDN。</x:v>
+      </x:c>
       <x:c r="B52" s="2"/>
       <x:c r="C52" s="8"/>
       <x:c r="D52" s="8"/>
@@ -3788,7 +4157,9 @@
       <x:c r="M53" s="2"/>
     </x:row>
     <x:row r="54" ht="25" customHeight="1">
-      <x:c r="A54" s="2"/>
+      <x:c r="A54" s="2" t="str">
+        <x:v>V4.1：S tokens 快照；C2 物理页 B/2 行，只计完成的压缩对；环形 state 规划传完整 32 行页。</x:v>
+      </x:c>
       <x:c r="B54" s="2"/>
       <x:c r="C54" s="8"/>
       <x:c r="D54" s="8"/>
@@ -3818,7 +4189,9 @@
       <x:c r="M55" s="2"/>
     </x:row>
     <x:row r="56" ht="25" customHeight="1">
-      <x:c r="A56" s="2"/>
+      <x:c r="A56" s="2" t="str">
+        <x:v>来源：归档 config / VA 842b030f / vLLM c8438a3；V4.1 main 1933f86；路径/哈希见源码清单。</x:v>
+      </x:c>
       <x:c r="B56" s="2"/>
       <x:c r="C56" s="8"/>
       <x:c r="D56" s="8"/>
@@ -4663,34 +5036,96 @@
       </x:c>
     </x:row>
     <x:row r="20" ht="25" customHeight="1">
-      <x:c r="A20" s="2"/>
-      <x:c r="B20" s="2"/>
-      <x:c r="C20" s="2"/>
-      <x:c r="D20" s="2"/>
-      <x:c r="E20" s="2"/>
-      <x:c r="F20" s="2"/>
-      <x:c r="G20" s="2"/>
-      <x:c r="H20" s="2"/>
-      <x:c r="I20" s="2"/>
-      <x:c r="J20" s="2"/>
-      <x:c r="K20" s="2"/>
-      <x:c r="L20" s="2"/>
-      <x:c r="M20" s="2"/>
+      <x:c r="A20" s="2" t="str">
+        <x:v>DS V4.1 Flash</x:v>
+      </x:c>
+      <x:c r="B20" s="2" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C20" s="2" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="D20" s="2" t="n">
+        <x:v>5120</x:v>
+      </x:c>
+      <x:c r="E20" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F20" s="2" t="n">
+        <x:v>384</x:v>
+      </x:c>
+      <x:c r="G20" s="2" t="n">
+        <x:f>ROUNDUP(F20/B20,0)*B20</x:f>
+        <x:v>384</x:v>
+      </x:c>
+      <x:c r="H20" s="2" t="n">
+        <x:f>G20-F20</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I20" s="2" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="J20" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K20" s="2" t="n">
+        <x:f>ROUNDUP($B$5/I20,0)</x:f>
+        <x:v>2048</x:v>
+      </x:c>
+      <x:c r="L20" s="2" t="n">
+        <x:f>ROUNDUP($D$5/J20,0)</x:f>
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="M20" s="2" t="n">
+        <x:f>ROUNDUP((ROUNDUP((ROUNDUP(D20*$F$5/32,0)*32+$H$5)/32,0)*32+32)/480,0)*512</x:f>
+        <x:v>11264</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="25" customHeight="1">
-      <x:c r="A21" s="2"/>
-      <x:c r="B21" s="2"/>
-      <x:c r="C21" s="2"/>
-      <x:c r="D21" s="2"/>
-      <x:c r="E21" s="2"/>
-      <x:c r="F21" s="2"/>
-      <x:c r="G21" s="2"/>
-      <x:c r="H21" s="2"/>
-      <x:c r="I21" s="2"/>
-      <x:c r="J21" s="2"/>
-      <x:c r="K21" s="2"/>
-      <x:c r="L21" s="2"/>
-      <x:c r="M21" s="2"/>
+      <x:c r="A21" s="2" t="str">
+        <x:v>DS V4.1 Flash</x:v>
+      </x:c>
+      <x:c r="B21" s="2" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="C21" s="2" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="D21" s="2" t="n">
+        <x:v>5120</x:v>
+      </x:c>
+      <x:c r="E21" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F21" s="2" t="n">
+        <x:v>384</x:v>
+      </x:c>
+      <x:c r="G21" s="2" t="n">
+        <x:f>ROUNDUP(F21/B21,0)*B21</x:f>
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="H21" s="2" t="n">
+        <x:f>G21-F21</x:f>
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="I21" s="2" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="J21" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K21" s="2" t="n">
+        <x:f>ROUNDUP($B$5/I21,0)</x:f>
+        <x:v>2048</x:v>
+      </x:c>
+      <x:c r="L21" s="2" t="n">
+        <x:f>ROUNDUP($D$5/J21,0)</x:f>
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="M21" s="2" t="n">
+        <x:f>ROUNDUP((ROUNDUP((ROUNDUP(D21*$F$5/32,0)*32+$H$5)/32,0)*32+32)/480,0)*512</x:f>
+        <x:v>11264</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="25" customHeight="1">
       <x:c r="A22" s="2"/>
@@ -5257,33 +5692,105 @@
       <x:c r="M33" s="2"/>
     </x:row>
     <x:row r="34" ht="25" customHeight="1">
-      <x:c r="A34" s="2"/>
-      <x:c r="B34" s="2"/>
-      <x:c r="C34" s="2"/>
-      <x:c r="D34" s="2"/>
-      <x:c r="E34" s="2"/>
-      <x:c r="F34" s="2"/>
-      <x:c r="G34" s="2"/>
-      <x:c r="H34" s="2"/>
-      <x:c r="I34" s="2"/>
-      <x:c r="J34" s="2"/>
-      <x:c r="K34" s="2"/>
-      <x:c r="L34" s="2"/>
+      <x:c r="A34" s="2" t="str">
+        <x:f>A20</x:f>
+        <x:v>DS V4.1 Flash</x:v>
+      </x:c>
+      <x:c r="B34" s="2" t="n">
+        <x:f>B20</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C34" s="12" t="n">
+        <x:f>IF(AND($J$5=2,OR(AND($F$5=2,$H$5=0),AND($F$5=1,$H$5=4))),(C20*K20*E20*(B20-1)*(D20*$F$5+$H$5))/2^30,NA())</x:f>
+        <x:v>145.3125</x:v>
+      </x:c>
+      <x:c r="D34" s="12" t="n">
+        <x:f>IF(AND($J$5=2,OR(AND($F$5=2,$H$5=0),AND($F$5=1,$H$5=4))),(C20*K20*E20*(B20-1)*D20*$J$5)/2^30,NA())</x:f>
+        <x:v>145.3125</x:v>
+      </x:c>
+      <x:c r="E34" s="12" t="n">
+        <x:f>IF(AND($J$5=2,OR(AND($F$5=2,$H$5=0),AND($F$5=1,$H$5=4))),(IF(K20=0,0,C20*G20*$L$5*B20*(B20-1)))/2^30,NA())</x:f>
+        <x:v>0.0567626953125</x:v>
+      </x:c>
+      <x:c r="F34" s="12" t="n">
+        <x:f>SUM(C34:E34)</x:f>
+        <x:v>290.6817626953125</x:v>
+      </x:c>
+      <x:c r="G34" s="12" t="n">
+        <x:f>IF(AND($J$5=2,OR(AND($F$5=2,$H$5=0),AND($F$5=1,$H$5=4))),(C20*L20*E20*(B20-1)*M20)/2^30,NA())</x:f>
+        <x:v>9.990234375</x:v>
+      </x:c>
+      <x:c r="H34" s="12" t="n">
+        <x:f>IF(AND($J$5=2,OR(AND($F$5=2,$H$5=0),AND($F$5=1,$H$5=4))),(IF(L20=0,0,C20*G20*(B20-1)*32))/2^30,NA())</x:f>
+        <x:v>0.014190673828125</x:v>
+      </x:c>
+      <x:c r="I34" s="12" t="n">
+        <x:f>IF(AND($J$5=2,OR(AND($F$5=2,$H$5=0),AND($F$5=1,$H$5=4))),(C20*L20*E20*(B20-1)*D20*$J$5)/2^30,NA())</x:f>
+        <x:v>9.08203125</x:v>
+      </x:c>
+      <x:c r="J34" s="12" t="n">
+        <x:f>IF(AND($J$5=2,OR(AND($F$5=2,$H$5=0),AND($F$5=1,$H$5=4))),(C20*L20*E20*(B20-1)*32)/2^30,NA())</x:f>
+        <x:v>0.02838134765625</x:v>
+      </x:c>
+      <x:c r="K34" s="12" t="n">
+        <x:f>SUM(G34:J34)</x:f>
+        <x:v>19.114837646484375</x:v>
+      </x:c>
+      <x:c r="L34" s="2" t="n">
+        <x:f>ROUNDUP((ROUNDUP(D20*$F$5/32,0)*32+$H$5)/32,0)*32+12</x:f>
+        <x:v>10252</x:v>
+      </x:c>
       <x:c r="M34" s="2"/>
     </x:row>
     <x:row r="35" ht="25" customHeight="1">
-      <x:c r="A35" s="2"/>
-      <x:c r="B35" s="2"/>
-      <x:c r="C35" s="2"/>
-      <x:c r="D35" s="2"/>
-      <x:c r="E35" s="2"/>
-      <x:c r="F35" s="2"/>
-      <x:c r="G35" s="2"/>
-      <x:c r="H35" s="2"/>
-      <x:c r="I35" s="2"/>
-      <x:c r="J35" s="2"/>
-      <x:c r="K35" s="2"/>
-      <x:c r="L35" s="2"/>
+      <x:c r="A35" s="2" t="str">
+        <x:f>A21</x:f>
+        <x:v>DS V4.1 Flash</x:v>
+      </x:c>
+      <x:c r="B35" s="2" t="n">
+        <x:f>B21</x:f>
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="C35" s="12" t="n">
+        <x:f>IF(AND($J$5=2,OR(AND($F$5=2,$H$5=0),AND($F$5=1,$H$5=4))),(C21*K21*E21*(B21-1)*(D21*$F$5+$H$5))/2^30,NA())</x:f>
+        <x:v>1195.3125</x:v>
+      </x:c>
+      <x:c r="D35" s="12" t="n">
+        <x:f>IF(AND($J$5=2,OR(AND($F$5=2,$H$5=0),AND($F$5=1,$H$5=4))),(C21*K21*E21*(B21-1)*D21*$J$5)/2^30,NA())</x:f>
+        <x:v>1195.3125</x:v>
+      </x:c>
+      <x:c r="E35" s="12" t="n">
+        <x:f>IF(AND($J$5=2,OR(AND($F$5=2,$H$5=0),AND($F$5=1,$H$5=4))),(IF(K21=0,0,C21*G21*$L$5*B21*(B21-1)))/2^30,NA())</x:f>
+        <x:v>4.98046875</x:v>
+      </x:c>
+      <x:c r="F35" s="12" t="n">
+        <x:f>SUM(C35:E35)</x:f>
+        <x:v>2395.60546875</x:v>
+      </x:c>
+      <x:c r="G35" s="12" t="n">
+        <x:f>IF(AND($J$5=2,OR(AND($F$5=2,$H$5=0),AND($F$5=1,$H$5=4))),(C21*L21*E21*(B21-1)*M21)/2^30,NA())</x:f>
+        <x:v>82.177734375</x:v>
+      </x:c>
+      <x:c r="H35" s="12" t="n">
+        <x:f>IF(AND($J$5=2,OR(AND($F$5=2,$H$5=0),AND($F$5=1,$H$5=4))),(IF(L21=0,0,C21*G21*(B21-1)*32))/2^30,NA())</x:f>
+        <x:v>0.1556396484375</x:v>
+      </x:c>
+      <x:c r="I35" s="12" t="n">
+        <x:f>IF(AND($J$5=2,OR(AND($F$5=2,$H$5=0),AND($F$5=1,$H$5=4))),(C21*L21*E21*(B21-1)*D21*$J$5)/2^30,NA())</x:f>
+        <x:v>74.70703125</x:v>
+      </x:c>
+      <x:c r="J35" s="12" t="n">
+        <x:f>IF(AND($J$5=2,OR(AND($F$5=2,$H$5=0),AND($F$5=1,$H$5=4))),(C21*L21*E21*(B21-1)*32)/2^30,NA())</x:f>
+        <x:v>0.23345947265625</x:v>
+      </x:c>
+      <x:c r="K35" s="12" t="n">
+        <x:f>SUM(G35:J35)</x:f>
+        <x:v>157.27386474609375</x:v>
+      </x:c>
+      <x:c r="L35" s="2" t="n">
+        <x:f>ROUNDUP((ROUNDUP(D21*$F$5/32,0)*32+$H$5)/32,0)*32+12</x:f>
+        <x:v>10252</x:v>
+      </x:c>
       <x:c r="M35" s="2"/>
     </x:row>
     <x:row r="36" ht="25" customHeight="1">
@@ -5750,7 +6257,7 @@
   <x:conditionalFormatting sqref="B7:B7">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="INVALID"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="H10:H19">
+  <x:conditionalFormatting sqref="H10:H21">
     <x:cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
       <x:formula>0</x:formula>
     </x:cfRule>

</xml_diff>

<commit_message>
Add editable bandwidth and PD contention timing to model workbooks
</commit_message>
<xml_diff>
--- a/examples/kv-ep-sweep/kv-ep32-ep256.xlsx
+++ b/examples/kv-ep-sweep/kv-ep32-ep256.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规格汇总" sheetId="1" r:id="R13bd640b94e84542"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KV明细" sheetId="2" r:id="R7b68b400227b4bb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EP通信" sheetId="3" r:id="R425b3e88a8784639"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规格汇总" sheetId="1" r:id="Raa03d22eb82f43e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KV明细" sheetId="2" r:id="R09003c5bc9c24f3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EP通信" sheetId="3" r:id="R039f1c84f86f4f2e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,12 +15,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="7">
     <x:numFmt numFmtId="200" formatCode="#,##0"/>
     <x:numFmt numFmtId="201" formatCode="#,##0.000"/>
     <x:numFmt numFmtId="202" formatCode="#,##0.000000"/>
+    <x:numFmt numFmtId="203" formatCode="0%"/>
+    <x:numFmt numFmtId="204" formatCode="0.000"/>
+    <x:numFmt numFmtId="205" formatCode="0.00%"/>
+    <x:numFmt numFmtId="206" formatCode="0.00"/>
   </x:numFmts>
-  <x:fonts count="6">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -53,8 +57,25 @@
       <x:color rgb="FF955700"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -76,6 +97,16 @@
         <x:fgColor rgb="FFE8EEF5"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9E2F3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -83,7 +114,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="17">
+  <x:cellXfs count="29">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -131,6 +162,40 @@
     <x:xf numFmtId="201" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -142,7 +207,7 @@
         <x:color rgb="FFA32020"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE9E7"/>
         </x:patternFill>
       </x:fill>
@@ -153,7 +218,7 @@
         <x:color rgb="FF955700"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0C2"/>
         </x:patternFill>
       </x:fill>
@@ -373,6 +438,8 @@
     <x:col min="11" max="11" width="15" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="15" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="33" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="18" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="36" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="25" customHeight="1">
@@ -2135,229 +2202,895 @@
       <x:c r="M50" s="2"/>
     </x:row>
     <x:row r="51" ht="25" customHeight="1">
-      <x:c r="A51" s="2"/>
-      <x:c r="B51" s="2"/>
-      <x:c r="C51" s="2"/>
-      <x:c r="D51" s="2"/>
-      <x:c r="E51" s="2"/>
-      <x:c r="F51" s="2"/>
-      <x:c r="G51" s="2"/>
-      <x:c r="H51" s="2"/>
-      <x:c r="I51" s="2"/>
-      <x:c r="J51" s="2"/>
-      <x:c r="K51" s="2"/>
-      <x:c r="L51" s="2"/>
-      <x:c r="M51" s="2"/>
+      <x:c r="A51" s="19" t="str">
+        <x:v>PD 带宽争用：EP32 / EP256</x:v>
+      </x:c>
+      <x:c r="B51" s="17"/>
+      <x:c r="C51" s="17"/>
+      <x:c r="D51" s="17"/>
+      <x:c r="E51" s="17"/>
+      <x:c r="F51" s="17"/>
+      <x:c r="G51" s="17"/>
+      <x:c r="H51" s="17"/>
+      <x:c r="I51" s="17"/>
+      <x:c r="J51" s="17"/>
+      <x:c r="K51" s="17"/>
+      <x:c r="L51" s="17"/>
+      <x:c r="M51" s="17"/>
+      <x:c r="N51" s="17"/>
+      <x:c r="O51" s="17"/>
     </x:row>
     <x:row r="52" ht="25" customHeight="1">
-      <x:c r="A52" s="2"/>
-      <x:c r="B52" s="2"/>
-      <x:c r="C52" s="2"/>
-      <x:c r="D52" s="2"/>
-      <x:c r="E52" s="2"/>
-      <x:c r="F52" s="2"/>
-      <x:c r="G52" s="2"/>
-      <x:c r="H52" s="2"/>
-      <x:c r="I52" s="2"/>
-      <x:c r="J52" s="2"/>
-      <x:c r="K52" s="2"/>
-      <x:c r="L52" s="2"/>
-      <x:c r="M52" s="2"/>
+      <x:c r="A52" s="17" t="str">
+        <x:v>只计 MoE EP 带宽项，单位 ms/Step/Rank。100 GB/s 是归一化示例；全组字节先除 EP，不能直接除单卡带宽。</x:v>
+      </x:c>
+      <x:c r="B52" s="17"/>
+      <x:c r="C52" s="17"/>
+      <x:c r="D52" s="17"/>
+      <x:c r="E52" s="17"/>
+      <x:c r="F52" s="17"/>
+      <x:c r="G52" s="17"/>
+      <x:c r="H52" s="17"/>
+      <x:c r="I52" s="17"/>
+      <x:c r="J52" s="17"/>
+      <x:c r="K52" s="17"/>
+      <x:c r="L52" s="17"/>
+      <x:c r="M52" s="17"/>
+      <x:c r="N52" s="17"/>
+      <x:c r="O52" s="17"/>
     </x:row>
     <x:row r="53" ht="25" customHeight="1">
-      <x:c r="A53" s="2"/>
-      <x:c r="B53" s="2"/>
-      <x:c r="C53" s="2"/>
-      <x:c r="D53" s="2"/>
-      <x:c r="E53" s="2"/>
-      <x:c r="F53" s="2"/>
-      <x:c r="G53" s="2"/>
-      <x:c r="H53" s="2"/>
-      <x:c r="I53" s="2"/>
-      <x:c r="J53" s="2"/>
-      <x:c r="K53" s="2"/>
-      <x:c r="L53" s="2"/>
-      <x:c r="M53" s="2"/>
-    </x:row>
-    <x:row r="54" ht="25" customHeight="1">
-      <x:c r="A54" s="2"/>
-      <x:c r="B54" s="2"/>
-      <x:c r="C54" s="2"/>
-      <x:c r="D54" s="2"/>
-      <x:c r="E54" s="2"/>
-      <x:c r="F54" s="2"/>
-      <x:c r="G54" s="2"/>
-      <x:c r="H54" s="2"/>
-      <x:c r="I54" s="2"/>
-      <x:c r="J54" s="2"/>
-      <x:c r="K54" s="2"/>
-      <x:c r="L54" s="2"/>
-      <x:c r="M54" s="2"/>
+      <x:c r="A53" s="17"/>
+      <x:c r="B53" s="17"/>
+      <x:c r="C53" s="17"/>
+      <x:c r="D53" s="17"/>
+      <x:c r="E53" s="17"/>
+      <x:c r="F53" s="17"/>
+      <x:c r="G53" s="17"/>
+      <x:c r="H53" s="17"/>
+      <x:c r="I53" s="17"/>
+      <x:c r="J53" s="17"/>
+      <x:c r="K53" s="17"/>
+      <x:c r="L53" s="17"/>
+      <x:c r="M53" s="17"/>
+      <x:c r="N53" s="17"/>
+      <x:c r="O53" s="17"/>
+    </x:row>
+    <x:row r="54" ht="38" customHeight="1">
+      <x:c r="A54" s="22" t="str">
+        <x:v>P GB/s</x:v>
+      </x:c>
+      <x:c r="B54" s="22" t="str">
+        <x:v>输入</x:v>
+      </x:c>
+      <x:c r="C54" s="22" t="str">
+        <x:v>D GB/s</x:v>
+      </x:c>
+      <x:c r="D54" s="22" t="str">
+        <x:v>输入</x:v>
+      </x:c>
+      <x:c r="E54" s="22" t="str">
+        <x:v>带宽降幅</x:v>
+      </x:c>
+      <x:c r="F54" s="22" t="str">
+        <x:v>输入</x:v>
+      </x:c>
+      <x:c r="G54" s="22" t="str">
+        <x:v>争用覆盖率</x:v>
+      </x:c>
+      <x:c r="H54" s="22" t="str">
+        <x:v>输入</x:v>
+      </x:c>
+      <x:c r="I54" s="22" t="str">
+        <x:v>暴露系数</x:v>
+      </x:c>
+      <x:c r="J54" s="22" t="str">
+        <x:v>输入</x:v>
+      </x:c>
+      <x:c r="K54" s="17"/>
+      <x:c r="L54" s="17"/>
+      <x:c r="M54" s="17"/>
+      <x:c r="N54" s="17"/>
+      <x:c r="O54" s="17"/>
     </x:row>
     <x:row r="55" ht="25" customHeight="1">
-      <x:c r="A55" s="2"/>
-      <x:c r="B55" s="2"/>
-      <x:c r="C55" s="2"/>
-      <x:c r="D55" s="2"/>
-      <x:c r="E55" s="2"/>
-      <x:c r="F55" s="2"/>
-      <x:c r="G55" s="2"/>
-      <x:c r="H55" s="2"/>
-      <x:c r="I55" s="2"/>
-      <x:c r="J55" s="2"/>
-      <x:c r="K55" s="2"/>
-      <x:c r="L55" s="2"/>
-      <x:c r="M55" s="2"/>
+      <x:c r="A55" s="17"/>
+      <x:c r="B55" s="23" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C55" s="17"/>
+      <x:c r="D55" s="23" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E55" s="17"/>
+      <x:c r="F55" s="24" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="G55" s="17"/>
+      <x:c r="H55" s="24" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I55" s="17"/>
+      <x:c r="J55" s="24" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K55" s="17"/>
+      <x:c r="L55" s="17"/>
+      <x:c r="M55" s="17"/>
+      <x:c r="N55" s="17"/>
+      <x:c r="O55" s="17"/>
     </x:row>
     <x:row r="56" ht="25" customHeight="1">
-      <x:c r="A56" s="2"/>
-      <x:c r="B56" s="2"/>
-      <x:c r="C56" s="2"/>
-      <x:c r="D56" s="2"/>
-      <x:c r="E56" s="2"/>
-      <x:c r="F56" s="2"/>
-      <x:c r="G56" s="2"/>
-      <x:c r="H56" s="2"/>
-      <x:c r="I56" s="2"/>
-      <x:c r="J56" s="2"/>
-      <x:c r="K56" s="2"/>
-      <x:c r="L56" s="2"/>
-      <x:c r="M56" s="2"/>
-    </x:row>
-    <x:row r="57" ht="25" customHeight="1">
-      <x:c r="A57" s="2"/>
-      <x:c r="B57" s="2"/>
-      <x:c r="C57" s="2"/>
-      <x:c r="D57" s="2"/>
-      <x:c r="E57" s="2"/>
-      <x:c r="F57" s="2"/>
-      <x:c r="G57" s="2"/>
-      <x:c r="H57" s="2"/>
-      <x:c r="I57" s="2"/>
-      <x:c r="J57" s="2"/>
-      <x:c r="K57" s="2"/>
-      <x:c r="L57" s="2"/>
-      <x:c r="M57" s="2"/>
+      <x:c r="A56" s="17"/>
+      <x:c r="B56" s="17"/>
+      <x:c r="C56" s="17"/>
+      <x:c r="D56" s="17"/>
+      <x:c r="E56" s="17"/>
+      <x:c r="F56" s="17"/>
+      <x:c r="G56" s="17"/>
+      <x:c r="H56" s="17"/>
+      <x:c r="I56" s="17"/>
+      <x:c r="J56" s="17"/>
+      <x:c r="K56" s="17"/>
+      <x:c r="L56" s="17"/>
+      <x:c r="M56" s="17"/>
+      <x:c r="N56" s="17"/>
+      <x:c r="O56" s="17"/>
+    </x:row>
+    <x:row r="57" ht="38" customHeight="1">
+      <x:c r="A57" s="22" t="str">
+        <x:v>模型</x:v>
+      </x:c>
+      <x:c r="B57" s="22" t="str">
+        <x:v>EP</x:v>
+      </x:c>
+      <x:c r="C57" s="22" t="str">
+        <x:v>P基线通信 ms</x:v>
+      </x:c>
+      <x:c r="D57" s="22" t="str">
+        <x:v>P争用后 ms</x:v>
+      </x:c>
+      <x:c r="E57" s="22" t="str">
+        <x:v>P forward增量</x:v>
+      </x:c>
+      <x:c r="F57" s="22" t="str">
+        <x:v>D基线通信 ms</x:v>
+      </x:c>
+      <x:c r="G57" s="22" t="str">
+        <x:v>D争用后 ms</x:v>
+      </x:c>
+      <x:c r="H57" s="22" t="str">
+        <x:v>D forward增量</x:v>
+      </x:c>
+      <x:c r="I57" s="22" t="str">
+        <x:v>P基线FW ms输入</x:v>
+      </x:c>
+      <x:c r="J57" s="22" t="str">
+        <x:v>P forward增幅</x:v>
+      </x:c>
+      <x:c r="K57" s="22" t="str">
+        <x:v>D基线FW ms输入</x:v>
+      </x:c>
+      <x:c r="L57" s="22" t="str">
+        <x:v>D forward增幅</x:v>
+      </x:c>
+      <x:c r="M57" s="22" t="str">
+        <x:v>P带宽 GB/s 输入</x:v>
+      </x:c>
+      <x:c r="N57" s="22" t="str">
+        <x:v>D带宽 GB/s 输入</x:v>
+      </x:c>
+      <x:c r="O57" s="22" t="str">
+        <x:v>评估范围</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="25" customHeight="1">
-      <x:c r="A58" s="2"/>
-      <x:c r="B58" s="2"/>
-      <x:c r="C58" s="2"/>
-      <x:c r="D58" s="2"/>
-      <x:c r="E58" s="2"/>
-      <x:c r="F58" s="2"/>
-      <x:c r="G58" s="2"/>
-      <x:c r="H58" s="2"/>
-      <x:c r="I58" s="2"/>
-      <x:c r="J58" s="2"/>
-      <x:c r="K58" s="2"/>
-      <x:c r="L58" s="2"/>
-      <x:c r="M58" s="2"/>
+      <x:c r="A58" s="17" t="str">
+        <x:f>A6</x:f>
+        <x:v>DS V4 10T</x:v>
+      </x:c>
+      <x:c r="B58" s="17" t="n">
+        <x:f>B6</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C58" s="25" t="n">
+        <x:f>IF(AND(ISNUMBER(M58),M58&gt;0,ISNUMBER(N58),N58&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),I6*2^30/B6/(M58*1e6),NA())</x:f>
+        <x:v>208.22905344</x:v>
+      </x:c>
+      <x:c r="D58" s="25" t="n">
+        <x:f>C58*(1+$H$55*$F$55/(1-$F$55))</x:f>
+        <x:v>231.36561493333335</x:v>
+      </x:c>
+      <x:c r="E58" s="25" t="n">
+        <x:f>(D58-C58)*$J$55</x:f>
+        <x:v>23.136561493333346</x:v>
+      </x:c>
+      <x:c r="F58" s="25" t="n">
+        <x:f>IF(AND(ISNUMBER(M58),M58&gt;0,ISNUMBER(N58),N58&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),J6*2^30/B6/(N58*1e6),NA())</x:f>
+        <x:v>13.49901696</x:v>
+      </x:c>
+      <x:c r="G58" s="25" t="n">
+        <x:f>F58*(1+$H$55*$F$55/(1-$F$55))</x:f>
+        <x:v>14.998907733333334</x:v>
+      </x:c>
+      <x:c r="H58" s="25" t="n">
+        <x:f>(G58-F58)*$J$55</x:f>
+        <x:v>1.499890773333334</x:v>
+      </x:c>
+      <x:c r="I58" s="27"/>
+      <x:c r="J58" s="26" t="str">
+        <x:f>IF(AND(ISNUMBER(I58),I58&gt;0,I58&gt;=C58*$J$55),E58/I58,"")</x:f>
+      </x:c>
+      <x:c r="K58" s="27"/>
+      <x:c r="L58" s="26" t="str">
+        <x:f>IF(AND(ISNUMBER(K58),K58&gt;0,K58&gt;=F58*$J$55),H58/K58,"")</x:f>
+      </x:c>
+      <x:c r="M58" s="28" t="n">
+        <x:f>$B$55</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="N58" s="28" t="n">
+        <x:f>$D$55</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="O58" s="17" t="str">
+        <x:v>仅EP；总耗时需实测基线</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="25" customHeight="1">
-      <x:c r="A59" s="2"/>
-      <x:c r="B59" s="2"/>
-      <x:c r="C59" s="2"/>
-      <x:c r="D59" s="2"/>
-      <x:c r="E59" s="2"/>
-      <x:c r="F59" s="2"/>
-      <x:c r="G59" s="2"/>
-      <x:c r="H59" s="2"/>
-      <x:c r="I59" s="2"/>
-      <x:c r="J59" s="2"/>
-      <x:c r="K59" s="2"/>
-      <x:c r="L59" s="2"/>
-      <x:c r="M59" s="2"/>
+      <x:c r="A59" s="17" t="str">
+        <x:f>A7</x:f>
+        <x:v>DS V4 10T</x:v>
+      </x:c>
+      <x:c r="B59" s="17" t="n">
+        <x:f>B7</x:f>
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="C59" s="25" t="n">
+        <x:f>IF(AND(ISNUMBER(M59),M59&gt;0,ISNUMBER(N59),N59&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),I7*2^30/B7/(M59*1e6),NA())</x:f>
+        <x:v>214.3951872</x:v>
+      </x:c>
+      <x:c r="D59" s="25" t="n">
+        <x:f>C59*(1+$H$55*$F$55/(1-$F$55))</x:f>
+        <x:v>238.21687466666668</x:v>
+      </x:c>
+      <x:c r="E59" s="25" t="n">
+        <x:f>(D59-C59)*$J$55</x:f>
+        <x:v>23.821687466666674</x:v>
+      </x:c>
+      <x:c r="F59" s="25" t="n">
+        <x:f>IF(AND(ISNUMBER(M59),M59&gt;0,ISNUMBER(N59),N59&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),J7*2^30/B7/(N59*1e6),NA())</x:f>
+        <x:v>13.8825264</x:v>
+      </x:c>
+      <x:c r="G59" s="25" t="n">
+        <x:f>F59*(1+$H$55*$F$55/(1-$F$55))</x:f>
+        <x:v>15.425029333333333</x:v>
+      </x:c>
+      <x:c r="H59" s="25" t="n">
+        <x:f>(G59-F59)*$J$55</x:f>
+        <x:v>1.542502933333333</x:v>
+      </x:c>
+      <x:c r="I59" s="27"/>
+      <x:c r="J59" s="26" t="str">
+        <x:f>IF(AND(ISNUMBER(I59),I59&gt;0,I59&gt;=C59*$J$55),E59/I59,"")</x:f>
+      </x:c>
+      <x:c r="K59" s="27"/>
+      <x:c r="L59" s="26" t="str">
+        <x:f>IF(AND(ISNUMBER(K59),K59&gt;0,K59&gt;=F59*$J$55),H59/K59,"")</x:f>
+      </x:c>
+      <x:c r="M59" s="28" t="n">
+        <x:f>$B$55</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="N59" s="28" t="n">
+        <x:f>$D$55</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="O59" s="17" t="str">
+        <x:v>仅EP；总耗时需实测基线</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="25" customHeight="1">
-      <x:c r="A60" s="2"/>
-      <x:c r="B60" s="2"/>
-      <x:c r="C60" s="2"/>
-      <x:c r="D60" s="2"/>
-      <x:c r="E60" s="2"/>
-      <x:c r="F60" s="2"/>
-      <x:c r="G60" s="2"/>
-      <x:c r="H60" s="2"/>
-      <x:c r="I60" s="2"/>
-      <x:c r="J60" s="2"/>
-      <x:c r="K60" s="2"/>
-      <x:c r="L60" s="2"/>
-      <x:c r="M60" s="2"/>
+      <x:c r="A60" s="17" t="str">
+        <x:f>A8</x:f>
+        <x:v>DS V4 Pro</x:v>
+      </x:c>
+      <x:c r="B60" s="17" t="n">
+        <x:f>B8</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C60" s="25" t="n">
+        <x:f>IF(AND(ISNUMBER(M60),M60&gt;0,ISNUMBER(N60),N60&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),I8*2^30/B8/(M60*1e6),NA())</x:f>
+        <x:v>208.22905344</x:v>
+      </x:c>
+      <x:c r="D60" s="25" t="n">
+        <x:f>C60*(1+$H$55*$F$55/(1-$F$55))</x:f>
+        <x:v>231.36561493333335</x:v>
+      </x:c>
+      <x:c r="E60" s="25" t="n">
+        <x:f>(D60-C60)*$J$55</x:f>
+        <x:v>23.136561493333346</x:v>
+      </x:c>
+      <x:c r="F60" s="25" t="n">
+        <x:f>IF(AND(ISNUMBER(M60),M60&gt;0,ISNUMBER(N60),N60&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),J8*2^30/B8/(N60*1e6),NA())</x:f>
+        <x:v>13.49901696</x:v>
+      </x:c>
+      <x:c r="G60" s="25" t="n">
+        <x:f>F60*(1+$H$55*$F$55/(1-$F$55))</x:f>
+        <x:v>14.998907733333334</x:v>
+      </x:c>
+      <x:c r="H60" s="25" t="n">
+        <x:f>(G60-F60)*$J$55</x:f>
+        <x:v>1.499890773333334</x:v>
+      </x:c>
+      <x:c r="I60" s="27"/>
+      <x:c r="J60" s="26" t="str">
+        <x:f>IF(AND(ISNUMBER(I60),I60&gt;0,I60&gt;=C60*$J$55),E60/I60,"")</x:f>
+      </x:c>
+      <x:c r="K60" s="27"/>
+      <x:c r="L60" s="26" t="str">
+        <x:f>IF(AND(ISNUMBER(K60),K60&gt;0,K60&gt;=F60*$J$55),H60/K60,"")</x:f>
+      </x:c>
+      <x:c r="M60" s="28" t="n">
+        <x:f>$B$55</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="N60" s="28" t="n">
+        <x:f>$D$55</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="O60" s="17" t="str">
+        <x:v>仅EP；总耗时需实测基线</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="25" customHeight="1">
-      <x:c r="A61" s="2"/>
-      <x:c r="B61" s="2"/>
-      <x:c r="C61" s="2"/>
-      <x:c r="D61" s="2"/>
-      <x:c r="E61" s="2"/>
-      <x:c r="F61" s="2"/>
-      <x:c r="G61" s="2"/>
-      <x:c r="H61" s="2"/>
-      <x:c r="I61" s="2"/>
-      <x:c r="J61" s="2"/>
-      <x:c r="K61" s="2"/>
-      <x:c r="L61" s="2"/>
-      <x:c r="M61" s="2"/>
+      <x:c r="A61" s="17" t="str">
+        <x:f>A9</x:f>
+        <x:v>DS V4 Pro</x:v>
+      </x:c>
+      <x:c r="B61" s="17" t="n">
+        <x:f>B9</x:f>
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="C61" s="25" t="n">
+        <x:f>IF(AND(ISNUMBER(M61),M61&gt;0,ISNUMBER(N61),N61&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),I9*2^30/B9/(M61*1e6),NA())</x:f>
+        <x:v>214.3951872</x:v>
+      </x:c>
+      <x:c r="D61" s="25" t="n">
+        <x:f>C61*(1+$H$55*$F$55/(1-$F$55))</x:f>
+        <x:v>238.21687466666668</x:v>
+      </x:c>
+      <x:c r="E61" s="25" t="n">
+        <x:f>(D61-C61)*$J$55</x:f>
+        <x:v>23.821687466666674</x:v>
+      </x:c>
+      <x:c r="F61" s="25" t="n">
+        <x:f>IF(AND(ISNUMBER(M61),M61&gt;0,ISNUMBER(N61),N61&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),J9*2^30/B9/(N61*1e6),NA())</x:f>
+        <x:v>13.8825264</x:v>
+      </x:c>
+      <x:c r="G61" s="25" t="n">
+        <x:f>F61*(1+$H$55*$F$55/(1-$F$55))</x:f>
+        <x:v>15.425029333333333</x:v>
+      </x:c>
+      <x:c r="H61" s="25" t="n">
+        <x:f>(G61-F61)*$J$55</x:f>
+        <x:v>1.542502933333333</x:v>
+      </x:c>
+      <x:c r="I61" s="27"/>
+      <x:c r="J61" s="26" t="str">
+        <x:f>IF(AND(ISNUMBER(I61),I61&gt;0,I61&gt;=C61*$J$55),E61/I61,"")</x:f>
+      </x:c>
+      <x:c r="K61" s="27"/>
+      <x:c r="L61" s="26" t="str">
+        <x:f>IF(AND(ISNUMBER(K61),K61&gt;0,K61&gt;=F61*$J$55),H61/K61,"")</x:f>
+      </x:c>
+      <x:c r="M61" s="28" t="n">
+        <x:f>$B$55</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="N61" s="28" t="n">
+        <x:f>$D$55</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="O61" s="17" t="str">
+        <x:v>仅EP；总耗时需实测基线</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="25" customHeight="1">
-      <x:c r="A62" s="2"/>
-      <x:c r="B62" s="2"/>
-      <x:c r="C62" s="2"/>
-      <x:c r="D62" s="2"/>
-      <x:c r="E62" s="2"/>
-      <x:c r="F62" s="2"/>
-      <x:c r="G62" s="2"/>
-      <x:c r="H62" s="2"/>
-      <x:c r="I62" s="2"/>
-      <x:c r="J62" s="2"/>
-      <x:c r="K62" s="2"/>
-      <x:c r="L62" s="2"/>
-      <x:c r="M62" s="2"/>
+      <x:c r="A62" s="17" t="str">
+        <x:f>A10</x:f>
+        <x:v>GLM5.3</x:v>
+      </x:c>
+      <x:c r="B62" s="17" t="n">
+        <x:f>B10</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C62" s="25" t="n">
+        <x:f>IF(AND(ISNUMBER(M62),M62&gt;0,ISNUMBER(N62),N62&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),I10*2^30/B10/(M62*1e6),NA())</x:f>
+        <x:v>292.576512</x:v>
+      </x:c>
+      <x:c r="D62" s="25" t="n">
+        <x:f>C62*(1+$H$55*$F$55/(1-$F$55))</x:f>
+        <x:v>325.08501333333334</x:v>
+      </x:c>
+      <x:c r="E62" s="25" t="n">
+        <x:f>(D62-C62)*$J$55</x:f>
+        <x:v>32.508501333333356</x:v>
+      </x:c>
+      <x:c r="F62" s="25" t="n">
+        <x:f>IF(AND(ISNUMBER(M62),M62&gt;0,ISNUMBER(N62),N62&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),J10*2^30/B10/(N62*1e6),NA())</x:f>
+        <x:v>19.07616</x:v>
+      </x:c>
+      <x:c r="G62" s="25" t="n">
+        <x:f>F62*(1+$H$55*$F$55/(1-$F$55))</x:f>
+        <x:v>21.195733333333337</x:v>
+      </x:c>
+      <x:c r="H62" s="25" t="n">
+        <x:f>(G62-F62)*$J$55</x:f>
+        <x:v>2.119573333333335</x:v>
+      </x:c>
+      <x:c r="I62" s="27"/>
+      <x:c r="J62" s="26" t="str">
+        <x:f>IF(AND(ISNUMBER(I62),I62&gt;0,I62&gt;=C62*$J$55),E62/I62,"")</x:f>
+      </x:c>
+      <x:c r="K62" s="27"/>
+      <x:c r="L62" s="26" t="str">
+        <x:f>IF(AND(ISNUMBER(K62),K62&gt;0,K62&gt;=F62*$J$55),H62/K62,"")</x:f>
+      </x:c>
+      <x:c r="M62" s="28" t="n">
+        <x:f>$B$55</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="N62" s="28" t="n">
+        <x:f>$D$55</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="O62" s="17" t="str">
+        <x:v>仅EP；总耗时需实测基线</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="25" customHeight="1">
-      <x:c r="A63" s="2"/>
-      <x:c r="B63" s="2"/>
-      <x:c r="C63" s="2"/>
-      <x:c r="D63" s="2"/>
-      <x:c r="E63" s="2"/>
-      <x:c r="F63" s="2"/>
-      <x:c r="G63" s="2"/>
-      <x:c r="H63" s="2"/>
-      <x:c r="I63" s="2"/>
-      <x:c r="J63" s="2"/>
-      <x:c r="K63" s="2"/>
-      <x:c r="L63" s="2"/>
-      <x:c r="M63" s="2"/>
+      <x:c r="A63" s="17" t="str">
+        <x:f>A11</x:f>
+        <x:v>GLM5.3</x:v>
+      </x:c>
+      <x:c r="B63" s="17" t="n">
+        <x:f>B11</x:f>
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="C63" s="25" t="n">
+        <x:f>IF(AND(ISNUMBER(M63),M63&gt;0,ISNUMBER(N63),N63&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),I11*2^30/B11/(M63*1e6),NA())</x:f>
+        <x:v>301.00608</x:v>
+      </x:c>
+      <x:c r="D63" s="25" t="n">
+        <x:f>C63*(1+$H$55*$F$55/(1-$F$55))</x:f>
+        <x:v>334.45120000000003</x:v>
+      </x:c>
+      <x:c r="E63" s="25" t="n">
+        <x:f>(D63-C63)*$J$55</x:f>
+        <x:v>33.44512000000003</x:v>
+      </x:c>
+      <x:c r="F63" s="25" t="n">
+        <x:f>IF(AND(ISNUMBER(M63),M63&gt;0,ISNUMBER(N63),N63&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),J11*2^30/B11/(N63*1e6),NA())</x:f>
+        <x:v>19.6146</x:v>
+      </x:c>
+      <x:c r="G63" s="25" t="n">
+        <x:f>F63*(1+$H$55*$F$55/(1-$F$55))</x:f>
+        <x:v>21.794</x:v>
+      </x:c>
+      <x:c r="H63" s="25" t="n">
+        <x:f>(G63-F63)*$J$55</x:f>
+        <x:v>2.179400000000001</x:v>
+      </x:c>
+      <x:c r="I63" s="27"/>
+      <x:c r="J63" s="26" t="str">
+        <x:f>IF(AND(ISNUMBER(I63),I63&gt;0,I63&gt;=C63*$J$55),E63/I63,"")</x:f>
+      </x:c>
+      <x:c r="K63" s="27"/>
+      <x:c r="L63" s="26" t="str">
+        <x:f>IF(AND(ISNUMBER(K63),K63&gt;0,K63&gt;=F63*$J$55),H63/K63,"")</x:f>
+      </x:c>
+      <x:c r="M63" s="28" t="n">
+        <x:f>$B$55</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="N63" s="28" t="n">
+        <x:f>$D$55</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="O63" s="17" t="str">
+        <x:v>仅EP；总耗时需实测基线</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="25" customHeight="1">
-      <x:c r="A64" s="2"/>
-      <x:c r="B64" s="2"/>
-      <x:c r="C64" s="2"/>
-      <x:c r="D64" s="2"/>
-      <x:c r="E64" s="2"/>
-      <x:c r="F64" s="2"/>
-      <x:c r="G64" s="2"/>
-      <x:c r="H64" s="2"/>
-      <x:c r="I64" s="2"/>
-      <x:c r="J64" s="2"/>
-      <x:c r="K64" s="2"/>
-      <x:c r="L64" s="2"/>
-      <x:c r="M64" s="2"/>
+      <x:c r="A64" s="17" t="str">
+        <x:f>A12</x:f>
+        <x:v>KimiK3</x:v>
+      </x:c>
+      <x:c r="B64" s="17" t="n">
+        <x:f>B12</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C64" s="25" t="n">
+        <x:f>IF(AND(ISNUMBER(M64),M64&gt;0,ISNUMBER(N64),N64&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),I12*2^30/B12/(M64*1e6),NA())</x:f>
+        <x:v>837.45306624</x:v>
+      </x:c>
+      <x:c r="D64" s="25" t="n">
+        <x:f>C64*(1+$H$55*$F$55/(1-$F$55))</x:f>
+        <x:v>930.5034069333334</x:v>
+      </x:c>
+      <x:c r="E64" s="25" t="n">
+        <x:f>(D64-C64)*$J$55</x:f>
+        <x:v>93.0503406933334</x:v>
+      </x:c>
+      <x:c r="F64" s="25" t="n">
+        <x:f>IF(AND(ISNUMBER(M64),M64&gt;0,ISNUMBER(N64),N64&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),J12*2^30/B12/(N64*1e6),NA())</x:f>
+        <x:v>6.8082944</x:v>
+      </x:c>
+      <x:c r="G64" s="25" t="n">
+        <x:f>F64*(1+$H$55*$F$55/(1-$F$55))</x:f>
+        <x:v>7.564771555555557</x:v>
+      </x:c>
+      <x:c r="H64" s="25" t="n">
+        <x:f>(G64-F64)*$J$55</x:f>
+        <x:v>0.7564771555555563</x:v>
+      </x:c>
+      <x:c r="I64" s="27"/>
+      <x:c r="J64" s="26" t="str">
+        <x:f>IF(AND(ISNUMBER(I64),I64&gt;0,I64&gt;=C64*$J$55),E64/I64,"")</x:f>
+      </x:c>
+      <x:c r="K64" s="27"/>
+      <x:c r="L64" s="26" t="str">
+        <x:f>IF(AND(ISNUMBER(K64),K64&gt;0,K64&gt;=F64*$J$55),H64/K64,"")</x:f>
+      </x:c>
+      <x:c r="M64" s="28" t="n">
+        <x:f>$B$55</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="N64" s="28" t="n">
+        <x:f>$D$55</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="O64" s="17" t="str">
+        <x:v>仅EP；总耗时需实测基线</x:v>
+      </x:c>
     </x:row>
     <x:row r="65" ht="25" customHeight="1">
-      <x:c r="A65" s="2"/>
-      <x:c r="B65" s="2"/>
-      <x:c r="C65" s="2"/>
-      <x:c r="D65" s="2"/>
-      <x:c r="E65" s="2"/>
-      <x:c r="F65" s="2"/>
-      <x:c r="G65" s="2"/>
-      <x:c r="H65" s="2"/>
-      <x:c r="I65" s="2"/>
-      <x:c r="J65" s="2"/>
-      <x:c r="K65" s="2"/>
-      <x:c r="L65" s="2"/>
-      <x:c r="M65" s="2"/>
+      <x:c r="A65" s="17" t="str">
+        <x:f>A13</x:f>
+        <x:v>KimiK3</x:v>
+      </x:c>
+      <x:c r="B65" s="17" t="n">
+        <x:f>B13</x:f>
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="C65" s="25" t="n">
+        <x:f>IF(AND(ISNUMBER(M65),M65&gt;0,ISNUMBER(N65),N65&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),I13*2^30/B13/(M65*1e6),NA())</x:f>
+        <x:v>861.9466752</x:v>
+      </x:c>
+      <x:c r="D65" s="25" t="n">
+        <x:f>C65*(1+$H$55*$F$55/(1-$F$55))</x:f>
+        <x:v>957.718528</x:v>
+      </x:c>
+      <x:c r="E65" s="25" t="n">
+        <x:f>(D65-C65)*$J$55</x:f>
+        <x:v>95.77185280000003</x:v>
+      </x:c>
+      <x:c r="F65" s="25" t="n">
+        <x:f>IF(AND(ISNUMBER(M65),M65&gt;0,ISNUMBER(N65),N65&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),J13*2^30/B13/(N65*1e6),NA())</x:f>
+        <x:v>7.0042176</x:v>
+      </x:c>
+      <x:c r="G65" s="25" t="n">
+        <x:f>F65*(1+$H$55*$F$55/(1-$F$55))</x:f>
+        <x:v>7.782464</x:v>
+      </x:c>
+      <x:c r="H65" s="25" t="n">
+        <x:f>(G65-F65)*$J$55</x:f>
+        <x:v>0.7782464000000004</x:v>
+      </x:c>
+      <x:c r="I65" s="27"/>
+      <x:c r="J65" s="26" t="str">
+        <x:f>IF(AND(ISNUMBER(I65),I65&gt;0,I65&gt;=C65*$J$55),E65/I65,"")</x:f>
+      </x:c>
+      <x:c r="K65" s="27"/>
+      <x:c r="L65" s="26" t="str">
+        <x:f>IF(AND(ISNUMBER(K65),K65&gt;0,K65&gt;=F65*$J$55),H65/K65,"")</x:f>
+      </x:c>
+      <x:c r="M65" s="28" t="n">
+        <x:f>$B$55</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="N65" s="28" t="n">
+        <x:f>$D$55</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="O65" s="17" t="str">
+        <x:v>仅EP；总耗时需实测基线</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="25" customHeight="1">
+      <x:c r="A66" s="17" t="str">
+        <x:f>A14</x:f>
+        <x:v>Qwen3.8 2.4T</x:v>
+      </x:c>
+      <x:c r="B66" s="17" t="n">
+        <x:f>B14</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C66" s="25" t="n">
+        <x:f>IF(AND(ISNUMBER(M66),M66&gt;0,ISNUMBER(N66),N66&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),I14*2^30/B14/(M66*1e6),NA())</x:f>
+        <x:v>598.16615936</x:v>
+      </x:c>
+      <x:c r="D66" s="25" t="n">
+        <x:f>C66*(1+$H$55*$F$55/(1-$F$55))</x:f>
+        <x:v>664.6290659555557</x:v>
+      </x:c>
+      <x:c r="E66" s="25" t="n">
+        <x:f>(D66-C66)*$J$55</x:f>
+        <x:v>66.46290659555564</x:v>
+      </x:c>
+      <x:c r="F66" s="25" t="n">
+        <x:f>IF(AND(ISNUMBER(M66),M66&gt;0,ISNUMBER(N66),N66&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),J14*2^30/B14/(N66*1e6),NA())</x:f>
+        <x:v>4.91091584</x:v>
+      </x:c>
+      <x:c r="G66" s="25" t="n">
+        <x:f>F66*(1+$H$55*$F$55/(1-$F$55))</x:f>
+        <x:v>5.4565731555555566</x:v>
+      </x:c>
+      <x:c r="H66" s="25" t="n">
+        <x:f>(G66-F66)*$J$55</x:f>
+        <x:v>0.5456573155555562</x:v>
+      </x:c>
+      <x:c r="I66" s="27"/>
+      <x:c r="J66" s="26" t="str">
+        <x:f>IF(AND(ISNUMBER(I66),I66&gt;0,I66&gt;=C66*$J$55),E66/I66,"")</x:f>
+      </x:c>
+      <x:c r="K66" s="27"/>
+      <x:c r="L66" s="26" t="str">
+        <x:f>IF(AND(ISNUMBER(K66),K66&gt;0,K66&gt;=F66*$J$55),H66/K66,"")</x:f>
+      </x:c>
+      <x:c r="M66" s="28" t="n">
+        <x:f>$B$55</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="N66" s="28" t="n">
+        <x:f>$D$55</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="O66" s="17" t="str">
+        <x:v>仅EP；总耗时需实测基线</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="25" customHeight="1">
+      <x:c r="A67" s="17" t="str">
+        <x:f>A15</x:f>
+        <x:v>Qwen3.8 2.4T</x:v>
+      </x:c>
+      <x:c r="B67" s="17" t="n">
+        <x:f>B15</x:f>
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="C67" s="25" t="n">
+        <x:f>IF(AND(ISNUMBER(M67),M67&gt;0,ISNUMBER(N67),N67&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),I15*2^30/B15/(M67*1e6),NA())</x:f>
+        <x:v>615.4702848</x:v>
+      </x:c>
+      <x:c r="D67" s="25" t="n">
+        <x:f>C67*(1+$H$55*$F$55/(1-$F$55))</x:f>
+        <x:v>683.855872</x:v>
+      </x:c>
+      <x:c r="E67" s="25" t="n">
+        <x:f>(D67-C67)*$J$55</x:f>
+        <x:v>68.38558720000003</x:v>
+      </x:c>
+      <x:c r="F67" s="25" t="n">
+        <x:f>IF(AND(ISNUMBER(M67),M67&gt;0,ISNUMBER(N67),N67&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),J15*2^30/B15/(N67*1e6),NA())</x:f>
+        <x:v>5.0495304</x:v>
+      </x:c>
+      <x:c r="G67" s="25" t="n">
+        <x:f>F67*(1+$H$55*$F$55/(1-$F$55))</x:f>
+        <x:v>5.610589333333333</x:v>
+      </x:c>
+      <x:c r="H67" s="25" t="n">
+        <x:f>(G67-F67)*$J$55</x:f>
+        <x:v>0.5610589333333333</x:v>
+      </x:c>
+      <x:c r="I67" s="27"/>
+      <x:c r="J67" s="26" t="str">
+        <x:f>IF(AND(ISNUMBER(I67),I67&gt;0,I67&gt;=C67*$J$55),E67/I67,"")</x:f>
+      </x:c>
+      <x:c r="K67" s="27"/>
+      <x:c r="L67" s="26" t="str">
+        <x:f>IF(AND(ISNUMBER(K67),K67&gt;0,K67&gt;=F67*$J$55),H67/K67,"")</x:f>
+      </x:c>
+      <x:c r="M67" s="28" t="n">
+        <x:f>$B$55</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="N67" s="28" t="n">
+        <x:f>$D$55</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="O67" s="17" t="str">
+        <x:v>仅EP；总耗时需实测基线</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="25" customHeight="1">
+      <x:c r="A68" s="17" t="str">
+        <x:f>A16</x:f>
+        <x:v>DS V4.1 Flash</x:v>
+      </x:c>
+      <x:c r="B68" s="17" t="n">
+        <x:f>B16</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C68" s="25" t="n">
+        <x:f>IF(AND(ISNUMBER(M68),M68&gt;0,ISNUMBER(N68),N68&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),I16*2^30/B16/(M68*1e6),NA())</x:f>
+        <x:v>97.5366144</x:v>
+      </x:c>
+      <x:c r="D68" s="25" t="n">
+        <x:f>C68*(1+$H$55*$F$55/(1-$F$55))</x:f>
+        <x:v>108.37401600000001</x:v>
+      </x:c>
+      <x:c r="E68" s="25" t="n">
+        <x:f>(D68-C68)*$J$55</x:f>
+        <x:v>10.837401600000007</x:v>
+      </x:c>
+      <x:c r="F68" s="25" t="n">
+        <x:f>IF(AND(ISNUMBER(M68),M68&gt;0,ISNUMBER(N68),N68&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),J16*2^30/B16/(N68*1e6),NA())</x:f>
+        <x:v>6.4138752</x:v>
+      </x:c>
+      <x:c r="G68" s="25" t="n">
+        <x:f>F68*(1+$H$55*$F$55/(1-$F$55))</x:f>
+        <x:v>7.1265279999999995</x:v>
+      </x:c>
+      <x:c r="H68" s="25" t="n">
+        <x:f>(G68-F68)*$J$55</x:f>
+        <x:v>0.7126527999999999</x:v>
+      </x:c>
+      <x:c r="I68" s="27"/>
+      <x:c r="J68" s="26" t="str">
+        <x:f>IF(AND(ISNUMBER(I68),I68&gt;0,I68&gt;=C68*$J$55),E68/I68,"")</x:f>
+      </x:c>
+      <x:c r="K68" s="27"/>
+      <x:c r="L68" s="26" t="str">
+        <x:f>IF(AND(ISNUMBER(K68),K68&gt;0,K68&gt;=F68*$J$55),H68/K68,"")</x:f>
+      </x:c>
+      <x:c r="M68" s="28" t="n">
+        <x:f>$B$55</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="N68" s="28" t="n">
+        <x:f>$D$55</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="O68" s="17" t="str">
+        <x:v>仅EP；V4.1 PD条件评估</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="25" customHeight="1">
+      <x:c r="A69" s="17" t="str">
+        <x:f>A17</x:f>
+        <x:v>DS V4.1 Flash</x:v>
+      </x:c>
+      <x:c r="B69" s="17" t="n">
+        <x:f>B17</x:f>
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="C69" s="25" t="n">
+        <x:f>IF(AND(ISNUMBER(M69),M69&gt;0,ISNUMBER(N69),N69&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),I17*2^30/B17/(M69*1e6),NA())</x:f>
+        <x:v>100.478976</x:v>
+      </x:c>
+      <x:c r="D69" s="25" t="n">
+        <x:f>C69*(1+$H$55*$F$55/(1-$F$55))</x:f>
+        <x:v>111.64330666666667</x:v>
+      </x:c>
+      <x:c r="E69" s="25" t="n">
+        <x:f>(D69-C69)*$J$55</x:f>
+        <x:v>11.164330666666672</x:v>
+      </x:c>
+      <x:c r="F69" s="25" t="n">
+        <x:f>IF(AND(ISNUMBER(M69),M69&gt;0,ISNUMBER(N69),N69&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),J17*2^30/B17/(N69*1e6),NA())</x:f>
+        <x:v>6.596544</x:v>
+      </x:c>
+      <x:c r="G69" s="25" t="n">
+        <x:f>F69*(1+$H$55*$F$55/(1-$F$55))</x:f>
+        <x:v>7.329493333333334</x:v>
+      </x:c>
+      <x:c r="H69" s="25" t="n">
+        <x:f>(G69-F69)*$J$55</x:f>
+        <x:v>0.7329493333333339</x:v>
+      </x:c>
+      <x:c r="I69" s="27"/>
+      <x:c r="J69" s="26" t="str">
+        <x:f>IF(AND(ISNUMBER(I69),I69&gt;0,I69&gt;=C69*$J$55),E69/I69,"")</x:f>
+      </x:c>
+      <x:c r="K69" s="27"/>
+      <x:c r="L69" s="26" t="str">
+        <x:f>IF(AND(ISNUMBER(K69),K69&gt;0,K69&gt;=F69*$J$55),H69/K69,"")</x:f>
+      </x:c>
+      <x:c r="M69" s="28" t="n">
+        <x:f>$B$55</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="N69" s="28" t="n">
+        <x:f>$D$55</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="O69" s="17" t="str">
+        <x:v>仅EP；V4.1 PD条件评估</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="25" customHeight="1">
+      <x:c r="A70" s="17"/>
+      <x:c r="B70" s="17"/>
+      <x:c r="C70" s="17"/>
+      <x:c r="D70" s="17"/>
+      <x:c r="E70" s="17"/>
+      <x:c r="F70" s="17"/>
+      <x:c r="G70" s="17"/>
+      <x:c r="H70" s="17"/>
+      <x:c r="I70" s="17"/>
+      <x:c r="J70" s="17"/>
+      <x:c r="K70" s="17"/>
+      <x:c r="L70" s="17"/>
+      <x:c r="M70" s="17"/>
+      <x:c r="N70" s="17"/>
+      <x:c r="O70" s="17"/>
+    </x:row>
+    <x:row r="71" ht="25" customHeight="1">
+      <x:c r="A71" s="17" t="str">
+        <x:v>带宽下降 10% 对受影响带宽项增加 11.11%。forward 增幅还需真实基线；不把 KV 交接等待再加到每个 Decode Step。</x:v>
+      </x:c>
+      <x:c r="B71" s="17"/>
+      <x:c r="C71" s="17"/>
+      <x:c r="D71" s="17"/>
+      <x:c r="E71" s="17"/>
+      <x:c r="F71" s="17"/>
+      <x:c r="G71" s="17"/>
+      <x:c r="H71" s="17"/>
+      <x:c r="I71" s="17"/>
+      <x:c r="J71" s="17"/>
+      <x:c r="K71" s="17"/>
+      <x:c r="L71" s="17"/>
+      <x:c r="M71" s="17"/>
+      <x:c r="N71" s="17"/>
+      <x:c r="O71" s="17"/>
+    </x:row>
+    <x:row r="72" ht="25" customHeight="1">
+      <x:c r="A72" s="17"/>
+      <x:c r="B72" s="17"/>
+      <x:c r="C72" s="17"/>
+      <x:c r="D72" s="17"/>
+      <x:c r="E72" s="17"/>
+      <x:c r="F72" s="17"/>
+      <x:c r="G72" s="17"/>
+      <x:c r="H72" s="17"/>
+      <x:c r="I72" s="17"/>
+      <x:c r="J72" s="17"/>
+      <x:c r="K72" s="17"/>
+      <x:c r="L72" s="17"/>
+      <x:c r="M72" s="17"/>
+      <x:c r="N72" s="17"/>
+      <x:c r="O72" s="17"/>
+    </x:row>
+    <x:row r="73" ht="25" customHeight="1">
+      <x:c r="A73" s="17" t="str">
+        <x:v>黄色 M/N 列可填各模型、各 EP 的无争用有效带宽，GB/s=10⁹ B/s。默认共享比例为 1；逐模型表可按事件调整。</x:v>
+      </x:c>
+      <x:c r="B73" s="17"/>
+      <x:c r="C73" s="17"/>
+      <x:c r="D73" s="17"/>
+      <x:c r="E73" s="17"/>
+      <x:c r="F73" s="17"/>
+      <x:c r="G73" s="17"/>
+      <x:c r="H73" s="17"/>
+      <x:c r="I73" s="17"/>
+      <x:c r="J73" s="17"/>
+      <x:c r="K73" s="17"/>
+      <x:c r="L73" s="17"/>
+      <x:c r="M73" s="17"/>
+      <x:c r="N73" s="17"/>
+      <x:c r="O73" s="17"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Match PD timing sections to existing workbook styles
</commit_message>
<xml_diff>
--- a/examples/kv-ep-sweep/kv-ep32-ep256.xlsx
+++ b/examples/kv-ep-sweep/kv-ep32-ep256.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规格汇总" sheetId="1" r:id="Raa03d22eb82f43e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KV明细" sheetId="2" r:id="R09003c5bc9c24f3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EP通信" sheetId="3" r:id="R039f1c84f86f4f2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规格汇总" sheetId="1" r:id="R01c86217981149a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KV明细" sheetId="2" r:id="Rae1d944e3d8e44ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EP通信" sheetId="3" r:id="Rda010fe3171d4ec8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -24,7 +24,7 @@
     <x:numFmt numFmtId="205" formatCode="0.00%"/>
     <x:numFmt numFmtId="206" formatCode="0.00"/>
   </x:numFmts>
-  <x:fonts count="9">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -74,8 +74,14 @@
       <x:color rgb="FF000000"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF202C3B"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -107,6 +113,16 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF253D5B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF0C2"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -114,7 +130,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="29">
+  <x:cellXfs count="45">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -194,6 +210,54 @@
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="206" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
@@ -2202,895 +2266,895 @@
       <x:c r="M50" s="2"/>
     </x:row>
     <x:row r="51" ht="25" customHeight="1">
-      <x:c r="A51" s="19" t="str">
+      <x:c r="A51" s="10" t="str">
         <x:v>PD 带宽争用：EP32 / EP256</x:v>
       </x:c>
-      <x:c r="B51" s="17"/>
-      <x:c r="C51" s="17"/>
-      <x:c r="D51" s="17"/>
-      <x:c r="E51" s="17"/>
-      <x:c r="F51" s="17"/>
-      <x:c r="G51" s="17"/>
-      <x:c r="H51" s="17"/>
-      <x:c r="I51" s="17"/>
-      <x:c r="J51" s="17"/>
-      <x:c r="K51" s="17"/>
-      <x:c r="L51" s="17"/>
-      <x:c r="M51" s="17"/>
-      <x:c r="N51" s="17"/>
-      <x:c r="O51" s="17"/>
+      <x:c r="B51" s="2"/>
+      <x:c r="C51" s="2"/>
+      <x:c r="D51" s="2"/>
+      <x:c r="E51" s="2"/>
+      <x:c r="F51" s="2"/>
+      <x:c r="G51" s="2"/>
+      <x:c r="H51" s="2"/>
+      <x:c r="I51" s="2"/>
+      <x:c r="J51" s="2"/>
+      <x:c r="K51" s="2"/>
+      <x:c r="L51" s="2"/>
+      <x:c r="M51" s="2"/>
+      <x:c r="N51" s="2"/>
+      <x:c r="O51" s="2"/>
     </x:row>
     <x:row r="52" ht="25" customHeight="1">
-      <x:c r="A52" s="17" t="str">
+      <x:c r="A52" s="2" t="str">
         <x:v>只计 MoE EP 带宽项，单位 ms/Step/Rank。100 GB/s 是归一化示例；全组字节先除 EP，不能直接除单卡带宽。</x:v>
       </x:c>
-      <x:c r="B52" s="17"/>
-      <x:c r="C52" s="17"/>
-      <x:c r="D52" s="17"/>
-      <x:c r="E52" s="17"/>
-      <x:c r="F52" s="17"/>
-      <x:c r="G52" s="17"/>
-      <x:c r="H52" s="17"/>
-      <x:c r="I52" s="17"/>
-      <x:c r="J52" s="17"/>
-      <x:c r="K52" s="17"/>
-      <x:c r="L52" s="17"/>
-      <x:c r="M52" s="17"/>
-      <x:c r="N52" s="17"/>
-      <x:c r="O52" s="17"/>
+      <x:c r="B52" s="2"/>
+      <x:c r="C52" s="2"/>
+      <x:c r="D52" s="2"/>
+      <x:c r="E52" s="2"/>
+      <x:c r="F52" s="2"/>
+      <x:c r="G52" s="2"/>
+      <x:c r="H52" s="2"/>
+      <x:c r="I52" s="2"/>
+      <x:c r="J52" s="2"/>
+      <x:c r="K52" s="2"/>
+      <x:c r="L52" s="2"/>
+      <x:c r="M52" s="2"/>
+      <x:c r="N52" s="2"/>
+      <x:c r="O52" s="2"/>
     </x:row>
     <x:row r="53" ht="25" customHeight="1">
-      <x:c r="A53" s="17"/>
-      <x:c r="B53" s="17"/>
-      <x:c r="C53" s="17"/>
-      <x:c r="D53" s="17"/>
-      <x:c r="E53" s="17"/>
-      <x:c r="F53" s="17"/>
-      <x:c r="G53" s="17"/>
-      <x:c r="H53" s="17"/>
-      <x:c r="I53" s="17"/>
-      <x:c r="J53" s="17"/>
-      <x:c r="K53" s="17"/>
-      <x:c r="L53" s="17"/>
-      <x:c r="M53" s="17"/>
-      <x:c r="N53" s="17"/>
-      <x:c r="O53" s="17"/>
-    </x:row>
-    <x:row r="54" ht="38" customHeight="1">
-      <x:c r="A54" s="22" t="str">
+      <x:c r="A53" s="2"/>
+      <x:c r="B53" s="2"/>
+      <x:c r="C53" s="2"/>
+      <x:c r="D53" s="2"/>
+      <x:c r="E53" s="2"/>
+      <x:c r="F53" s="2"/>
+      <x:c r="G53" s="2"/>
+      <x:c r="H53" s="2"/>
+      <x:c r="I53" s="2"/>
+      <x:c r="J53" s="2"/>
+      <x:c r="K53" s="2"/>
+      <x:c r="L53" s="2"/>
+      <x:c r="M53" s="2"/>
+      <x:c r="N53" s="2"/>
+      <x:c r="O53" s="2"/>
+    </x:row>
+    <x:row r="54" ht="40" customHeight="1">
+      <x:c r="A54" s="39" t="str">
         <x:v>P GB/s</x:v>
       </x:c>
-      <x:c r="B54" s="22" t="str">
+      <x:c r="B54" s="39" t="str">
         <x:v>输入</x:v>
       </x:c>
-      <x:c r="C54" s="22" t="str">
+      <x:c r="C54" s="39" t="str">
         <x:v>D GB/s</x:v>
       </x:c>
-      <x:c r="D54" s="22" t="str">
+      <x:c r="D54" s="39" t="str">
         <x:v>输入</x:v>
       </x:c>
-      <x:c r="E54" s="22" t="str">
+      <x:c r="E54" s="39" t="str">
         <x:v>带宽降幅</x:v>
       </x:c>
-      <x:c r="F54" s="22" t="str">
+      <x:c r="F54" s="39" t="str">
         <x:v>输入</x:v>
       </x:c>
-      <x:c r="G54" s="22" t="str">
+      <x:c r="G54" s="39" t="str">
         <x:v>争用覆盖率</x:v>
       </x:c>
-      <x:c r="H54" s="22" t="str">
+      <x:c r="H54" s="39" t="str">
         <x:v>输入</x:v>
       </x:c>
-      <x:c r="I54" s="22" t="str">
+      <x:c r="I54" s="39" t="str">
         <x:v>暴露系数</x:v>
       </x:c>
-      <x:c r="J54" s="22" t="str">
+      <x:c r="J54" s="39" t="str">
         <x:v>输入</x:v>
       </x:c>
-      <x:c r="K54" s="17"/>
-      <x:c r="L54" s="17"/>
-      <x:c r="M54" s="17"/>
-      <x:c r="N54" s="17"/>
-      <x:c r="O54" s="17"/>
+      <x:c r="K54" s="2"/>
+      <x:c r="L54" s="2"/>
+      <x:c r="M54" s="2"/>
+      <x:c r="N54" s="2"/>
+      <x:c r="O54" s="2"/>
     </x:row>
     <x:row r="55" ht="25" customHeight="1">
-      <x:c r="A55" s="17"/>
-      <x:c r="B55" s="23" t="n">
+      <x:c r="A55" s="2"/>
+      <x:c r="B55" s="40" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="C55" s="17"/>
-      <x:c r="D55" s="23" t="n">
+      <x:c r="C55" s="2"/>
+      <x:c r="D55" s="40" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="E55" s="17"/>
-      <x:c r="F55" s="24" t="n">
+      <x:c r="E55" s="2"/>
+      <x:c r="F55" s="41" t="n">
         <x:v>0.1</x:v>
       </x:c>
-      <x:c r="G55" s="17"/>
-      <x:c r="H55" s="24" t="n">
+      <x:c r="G55" s="2"/>
+      <x:c r="H55" s="41" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I55" s="17"/>
-      <x:c r="J55" s="24" t="n">
+      <x:c r="I55" s="2"/>
+      <x:c r="J55" s="41" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K55" s="17"/>
-      <x:c r="L55" s="17"/>
-      <x:c r="M55" s="17"/>
-      <x:c r="N55" s="17"/>
-      <x:c r="O55" s="17"/>
+      <x:c r="K55" s="2"/>
+      <x:c r="L55" s="2"/>
+      <x:c r="M55" s="2"/>
+      <x:c r="N55" s="2"/>
+      <x:c r="O55" s="2"/>
     </x:row>
     <x:row r="56" ht="25" customHeight="1">
-      <x:c r="A56" s="17"/>
-      <x:c r="B56" s="17"/>
-      <x:c r="C56" s="17"/>
-      <x:c r="D56" s="17"/>
-      <x:c r="E56" s="17"/>
-      <x:c r="F56" s="17"/>
-      <x:c r="G56" s="17"/>
-      <x:c r="H56" s="17"/>
-      <x:c r="I56" s="17"/>
-      <x:c r="J56" s="17"/>
-      <x:c r="K56" s="17"/>
-      <x:c r="L56" s="17"/>
-      <x:c r="M56" s="17"/>
-      <x:c r="N56" s="17"/>
-      <x:c r="O56" s="17"/>
-    </x:row>
-    <x:row r="57" ht="38" customHeight="1">
-      <x:c r="A57" s="22" t="str">
+      <x:c r="A56" s="2"/>
+      <x:c r="B56" s="2"/>
+      <x:c r="C56" s="2"/>
+      <x:c r="D56" s="2"/>
+      <x:c r="E56" s="2"/>
+      <x:c r="F56" s="2"/>
+      <x:c r="G56" s="2"/>
+      <x:c r="H56" s="2"/>
+      <x:c r="I56" s="2"/>
+      <x:c r="J56" s="2"/>
+      <x:c r="K56" s="2"/>
+      <x:c r="L56" s="2"/>
+      <x:c r="M56" s="2"/>
+      <x:c r="N56" s="2"/>
+      <x:c r="O56" s="2"/>
+    </x:row>
+    <x:row r="57" ht="40" customHeight="1">
+      <x:c r="A57" s="39" t="str">
         <x:v>模型</x:v>
       </x:c>
-      <x:c r="B57" s="22" t="str">
+      <x:c r="B57" s="39" t="str">
         <x:v>EP</x:v>
       </x:c>
-      <x:c r="C57" s="22" t="str">
+      <x:c r="C57" s="39" t="str">
         <x:v>P基线通信 ms</x:v>
       </x:c>
-      <x:c r="D57" s="22" t="str">
+      <x:c r="D57" s="39" t="str">
         <x:v>P争用后 ms</x:v>
       </x:c>
-      <x:c r="E57" s="22" t="str">
+      <x:c r="E57" s="39" t="str">
         <x:v>P forward增量</x:v>
       </x:c>
-      <x:c r="F57" s="22" t="str">
+      <x:c r="F57" s="39" t="str">
         <x:v>D基线通信 ms</x:v>
       </x:c>
-      <x:c r="G57" s="22" t="str">
+      <x:c r="G57" s="39" t="str">
         <x:v>D争用后 ms</x:v>
       </x:c>
-      <x:c r="H57" s="22" t="str">
+      <x:c r="H57" s="39" t="str">
         <x:v>D forward增量</x:v>
       </x:c>
-      <x:c r="I57" s="22" t="str">
+      <x:c r="I57" s="39" t="str">
         <x:v>P基线FW ms输入</x:v>
       </x:c>
-      <x:c r="J57" s="22" t="str">
+      <x:c r="J57" s="39" t="str">
         <x:v>P forward增幅</x:v>
       </x:c>
-      <x:c r="K57" s="22" t="str">
+      <x:c r="K57" s="39" t="str">
         <x:v>D基线FW ms输入</x:v>
       </x:c>
-      <x:c r="L57" s="22" t="str">
+      <x:c r="L57" s="39" t="str">
         <x:v>D forward增幅</x:v>
       </x:c>
-      <x:c r="M57" s="22" t="str">
+      <x:c r="M57" s="39" t="str">
         <x:v>P带宽 GB/s 输入</x:v>
       </x:c>
-      <x:c r="N57" s="22" t="str">
+      <x:c r="N57" s="39" t="str">
         <x:v>D带宽 GB/s 输入</x:v>
       </x:c>
-      <x:c r="O57" s="22" t="str">
+      <x:c r="O57" s="39" t="str">
         <x:v>评估范围</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="25" customHeight="1">
-      <x:c r="A58" s="17" t="str">
+      <x:c r="A58" s="2" t="str">
         <x:f>A6</x:f>
         <x:v>DS V4 10T</x:v>
       </x:c>
-      <x:c r="B58" s="17" t="n">
+      <x:c r="B58" s="2" t="n">
         <x:f>B6</x:f>
         <x:v>32</x:v>
       </x:c>
-      <x:c r="C58" s="25" t="n">
+      <x:c r="C58" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(M58),M58&gt;0,ISNUMBER(N58),N58&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),I6*2^30/B6/(M58*1e6),NA())</x:f>
         <x:v>208.22905344</x:v>
       </x:c>
-      <x:c r="D58" s="25" t="n">
+      <x:c r="D58" s="9" t="n">
         <x:f>C58*(1+$H$55*$F$55/(1-$F$55))</x:f>
         <x:v>231.36561493333335</x:v>
       </x:c>
-      <x:c r="E58" s="25" t="n">
+      <x:c r="E58" s="9" t="n">
         <x:f>(D58-C58)*$J$55</x:f>
         <x:v>23.136561493333346</x:v>
       </x:c>
-      <x:c r="F58" s="25" t="n">
+      <x:c r="F58" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(M58),M58&gt;0,ISNUMBER(N58),N58&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),J6*2^30/B6/(N58*1e6),NA())</x:f>
         <x:v>13.49901696</x:v>
       </x:c>
-      <x:c r="G58" s="25" t="n">
+      <x:c r="G58" s="9" t="n">
         <x:f>F58*(1+$H$55*$F$55/(1-$F$55))</x:f>
         <x:v>14.998907733333334</x:v>
       </x:c>
-      <x:c r="H58" s="25" t="n">
+      <x:c r="H58" s="9" t="n">
         <x:f>(G58-F58)*$J$55</x:f>
         <x:v>1.499890773333334</x:v>
       </x:c>
-      <x:c r="I58" s="27"/>
-      <x:c r="J58" s="26" t="str">
+      <x:c r="I58" s="44"/>
+      <x:c r="J58" s="35" t="str">
         <x:f>IF(AND(ISNUMBER(I58),I58&gt;0,I58&gt;=C58*$J$55),E58/I58,"")</x:f>
       </x:c>
-      <x:c r="K58" s="27"/>
-      <x:c r="L58" s="26" t="str">
+      <x:c r="K58" s="44"/>
+      <x:c r="L58" s="35" t="str">
         <x:f>IF(AND(ISNUMBER(K58),K58&gt;0,K58&gt;=F58*$J$55),H58/K58,"")</x:f>
       </x:c>
-      <x:c r="M58" s="28" t="n">
+      <x:c r="M58" s="43" t="n">
         <x:f>$B$55</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="N58" s="28" t="n">
+      <x:c r="N58" s="43" t="n">
         <x:f>$D$55</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="O58" s="17" t="str">
+      <x:c r="O58" s="2" t="str">
         <x:v>仅EP；总耗时需实测基线</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="25" customHeight="1">
-      <x:c r="A59" s="17" t="str">
+      <x:c r="A59" s="2" t="str">
         <x:f>A7</x:f>
         <x:v>DS V4 10T</x:v>
       </x:c>
-      <x:c r="B59" s="17" t="n">
+      <x:c r="B59" s="2" t="n">
         <x:f>B7</x:f>
         <x:v>256</x:v>
       </x:c>
-      <x:c r="C59" s="25" t="n">
+      <x:c r="C59" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(M59),M59&gt;0,ISNUMBER(N59),N59&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),I7*2^30/B7/(M59*1e6),NA())</x:f>
         <x:v>214.3951872</x:v>
       </x:c>
-      <x:c r="D59" s="25" t="n">
+      <x:c r="D59" s="9" t="n">
         <x:f>C59*(1+$H$55*$F$55/(1-$F$55))</x:f>
         <x:v>238.21687466666668</x:v>
       </x:c>
-      <x:c r="E59" s="25" t="n">
+      <x:c r="E59" s="9" t="n">
         <x:f>(D59-C59)*$J$55</x:f>
         <x:v>23.821687466666674</x:v>
       </x:c>
-      <x:c r="F59" s="25" t="n">
+      <x:c r="F59" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(M59),M59&gt;0,ISNUMBER(N59),N59&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),J7*2^30/B7/(N59*1e6),NA())</x:f>
         <x:v>13.8825264</x:v>
       </x:c>
-      <x:c r="G59" s="25" t="n">
+      <x:c r="G59" s="9" t="n">
         <x:f>F59*(1+$H$55*$F$55/(1-$F$55))</x:f>
         <x:v>15.425029333333333</x:v>
       </x:c>
-      <x:c r="H59" s="25" t="n">
+      <x:c r="H59" s="9" t="n">
         <x:f>(G59-F59)*$J$55</x:f>
         <x:v>1.542502933333333</x:v>
       </x:c>
-      <x:c r="I59" s="27"/>
-      <x:c r="J59" s="26" t="str">
+      <x:c r="I59" s="44"/>
+      <x:c r="J59" s="35" t="str">
         <x:f>IF(AND(ISNUMBER(I59),I59&gt;0,I59&gt;=C59*$J$55),E59/I59,"")</x:f>
       </x:c>
-      <x:c r="K59" s="27"/>
-      <x:c r="L59" s="26" t="str">
+      <x:c r="K59" s="44"/>
+      <x:c r="L59" s="35" t="str">
         <x:f>IF(AND(ISNUMBER(K59),K59&gt;0,K59&gt;=F59*$J$55),H59/K59,"")</x:f>
       </x:c>
-      <x:c r="M59" s="28" t="n">
+      <x:c r="M59" s="43" t="n">
         <x:f>$B$55</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="N59" s="28" t="n">
+      <x:c r="N59" s="43" t="n">
         <x:f>$D$55</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="O59" s="17" t="str">
+      <x:c r="O59" s="2" t="str">
         <x:v>仅EP；总耗时需实测基线</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="25" customHeight="1">
-      <x:c r="A60" s="17" t="str">
+      <x:c r="A60" s="2" t="str">
         <x:f>A8</x:f>
         <x:v>DS V4 Pro</x:v>
       </x:c>
-      <x:c r="B60" s="17" t="n">
+      <x:c r="B60" s="2" t="n">
         <x:f>B8</x:f>
         <x:v>32</x:v>
       </x:c>
-      <x:c r="C60" s="25" t="n">
+      <x:c r="C60" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(M60),M60&gt;0,ISNUMBER(N60),N60&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),I8*2^30/B8/(M60*1e6),NA())</x:f>
         <x:v>208.22905344</x:v>
       </x:c>
-      <x:c r="D60" s="25" t="n">
+      <x:c r="D60" s="9" t="n">
         <x:f>C60*(1+$H$55*$F$55/(1-$F$55))</x:f>
         <x:v>231.36561493333335</x:v>
       </x:c>
-      <x:c r="E60" s="25" t="n">
+      <x:c r="E60" s="9" t="n">
         <x:f>(D60-C60)*$J$55</x:f>
         <x:v>23.136561493333346</x:v>
       </x:c>
-      <x:c r="F60" s="25" t="n">
+      <x:c r="F60" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(M60),M60&gt;0,ISNUMBER(N60),N60&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),J8*2^30/B8/(N60*1e6),NA())</x:f>
         <x:v>13.49901696</x:v>
       </x:c>
-      <x:c r="G60" s="25" t="n">
+      <x:c r="G60" s="9" t="n">
         <x:f>F60*(1+$H$55*$F$55/(1-$F$55))</x:f>
         <x:v>14.998907733333334</x:v>
       </x:c>
-      <x:c r="H60" s="25" t="n">
+      <x:c r="H60" s="9" t="n">
         <x:f>(G60-F60)*$J$55</x:f>
         <x:v>1.499890773333334</x:v>
       </x:c>
-      <x:c r="I60" s="27"/>
-      <x:c r="J60" s="26" t="str">
+      <x:c r="I60" s="44"/>
+      <x:c r="J60" s="35" t="str">
         <x:f>IF(AND(ISNUMBER(I60),I60&gt;0,I60&gt;=C60*$J$55),E60/I60,"")</x:f>
       </x:c>
-      <x:c r="K60" s="27"/>
-      <x:c r="L60" s="26" t="str">
+      <x:c r="K60" s="44"/>
+      <x:c r="L60" s="35" t="str">
         <x:f>IF(AND(ISNUMBER(K60),K60&gt;0,K60&gt;=F60*$J$55),H60/K60,"")</x:f>
       </x:c>
-      <x:c r="M60" s="28" t="n">
+      <x:c r="M60" s="43" t="n">
         <x:f>$B$55</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="N60" s="28" t="n">
+      <x:c r="N60" s="43" t="n">
         <x:f>$D$55</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="O60" s="17" t="str">
+      <x:c r="O60" s="2" t="str">
         <x:v>仅EP；总耗时需实测基线</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="25" customHeight="1">
-      <x:c r="A61" s="17" t="str">
+      <x:c r="A61" s="2" t="str">
         <x:f>A9</x:f>
         <x:v>DS V4 Pro</x:v>
       </x:c>
-      <x:c r="B61" s="17" t="n">
+      <x:c r="B61" s="2" t="n">
         <x:f>B9</x:f>
         <x:v>256</x:v>
       </x:c>
-      <x:c r="C61" s="25" t="n">
+      <x:c r="C61" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(M61),M61&gt;0,ISNUMBER(N61),N61&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),I9*2^30/B9/(M61*1e6),NA())</x:f>
         <x:v>214.3951872</x:v>
       </x:c>
-      <x:c r="D61" s="25" t="n">
+      <x:c r="D61" s="9" t="n">
         <x:f>C61*(1+$H$55*$F$55/(1-$F$55))</x:f>
         <x:v>238.21687466666668</x:v>
       </x:c>
-      <x:c r="E61" s="25" t="n">
+      <x:c r="E61" s="9" t="n">
         <x:f>(D61-C61)*$J$55</x:f>
         <x:v>23.821687466666674</x:v>
       </x:c>
-      <x:c r="F61" s="25" t="n">
+      <x:c r="F61" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(M61),M61&gt;0,ISNUMBER(N61),N61&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),J9*2^30/B9/(N61*1e6),NA())</x:f>
         <x:v>13.8825264</x:v>
       </x:c>
-      <x:c r="G61" s="25" t="n">
+      <x:c r="G61" s="9" t="n">
         <x:f>F61*(1+$H$55*$F$55/(1-$F$55))</x:f>
         <x:v>15.425029333333333</x:v>
       </x:c>
-      <x:c r="H61" s="25" t="n">
+      <x:c r="H61" s="9" t="n">
         <x:f>(G61-F61)*$J$55</x:f>
         <x:v>1.542502933333333</x:v>
       </x:c>
-      <x:c r="I61" s="27"/>
-      <x:c r="J61" s="26" t="str">
+      <x:c r="I61" s="44"/>
+      <x:c r="J61" s="35" t="str">
         <x:f>IF(AND(ISNUMBER(I61),I61&gt;0,I61&gt;=C61*$J$55),E61/I61,"")</x:f>
       </x:c>
-      <x:c r="K61" s="27"/>
-      <x:c r="L61" s="26" t="str">
+      <x:c r="K61" s="44"/>
+      <x:c r="L61" s="35" t="str">
         <x:f>IF(AND(ISNUMBER(K61),K61&gt;0,K61&gt;=F61*$J$55),H61/K61,"")</x:f>
       </x:c>
-      <x:c r="M61" s="28" t="n">
+      <x:c r="M61" s="43" t="n">
         <x:f>$B$55</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="N61" s="28" t="n">
+      <x:c r="N61" s="43" t="n">
         <x:f>$D$55</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="O61" s="17" t="str">
+      <x:c r="O61" s="2" t="str">
         <x:v>仅EP；总耗时需实测基线</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="25" customHeight="1">
-      <x:c r="A62" s="17" t="str">
+      <x:c r="A62" s="2" t="str">
         <x:f>A10</x:f>
         <x:v>GLM5.3</x:v>
       </x:c>
-      <x:c r="B62" s="17" t="n">
+      <x:c r="B62" s="2" t="n">
         <x:f>B10</x:f>
         <x:v>32</x:v>
       </x:c>
-      <x:c r="C62" s="25" t="n">
+      <x:c r="C62" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(M62),M62&gt;0,ISNUMBER(N62),N62&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),I10*2^30/B10/(M62*1e6),NA())</x:f>
         <x:v>292.576512</x:v>
       </x:c>
-      <x:c r="D62" s="25" t="n">
+      <x:c r="D62" s="9" t="n">
         <x:f>C62*(1+$H$55*$F$55/(1-$F$55))</x:f>
         <x:v>325.08501333333334</x:v>
       </x:c>
-      <x:c r="E62" s="25" t="n">
+      <x:c r="E62" s="9" t="n">
         <x:f>(D62-C62)*$J$55</x:f>
         <x:v>32.508501333333356</x:v>
       </x:c>
-      <x:c r="F62" s="25" t="n">
+      <x:c r="F62" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(M62),M62&gt;0,ISNUMBER(N62),N62&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),J10*2^30/B10/(N62*1e6),NA())</x:f>
         <x:v>19.07616</x:v>
       </x:c>
-      <x:c r="G62" s="25" t="n">
+      <x:c r="G62" s="9" t="n">
         <x:f>F62*(1+$H$55*$F$55/(1-$F$55))</x:f>
         <x:v>21.195733333333337</x:v>
       </x:c>
-      <x:c r="H62" s="25" t="n">
+      <x:c r="H62" s="9" t="n">
         <x:f>(G62-F62)*$J$55</x:f>
         <x:v>2.119573333333335</x:v>
       </x:c>
-      <x:c r="I62" s="27"/>
-      <x:c r="J62" s="26" t="str">
+      <x:c r="I62" s="44"/>
+      <x:c r="J62" s="35" t="str">
         <x:f>IF(AND(ISNUMBER(I62),I62&gt;0,I62&gt;=C62*$J$55),E62/I62,"")</x:f>
       </x:c>
-      <x:c r="K62" s="27"/>
-      <x:c r="L62" s="26" t="str">
+      <x:c r="K62" s="44"/>
+      <x:c r="L62" s="35" t="str">
         <x:f>IF(AND(ISNUMBER(K62),K62&gt;0,K62&gt;=F62*$J$55),H62/K62,"")</x:f>
       </x:c>
-      <x:c r="M62" s="28" t="n">
+      <x:c r="M62" s="43" t="n">
         <x:f>$B$55</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="N62" s="28" t="n">
+      <x:c r="N62" s="43" t="n">
         <x:f>$D$55</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="O62" s="17" t="str">
+      <x:c r="O62" s="2" t="str">
         <x:v>仅EP；总耗时需实测基线</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="25" customHeight="1">
-      <x:c r="A63" s="17" t="str">
+      <x:c r="A63" s="2" t="str">
         <x:f>A11</x:f>
         <x:v>GLM5.3</x:v>
       </x:c>
-      <x:c r="B63" s="17" t="n">
+      <x:c r="B63" s="2" t="n">
         <x:f>B11</x:f>
         <x:v>256</x:v>
       </x:c>
-      <x:c r="C63" s="25" t="n">
+      <x:c r="C63" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(M63),M63&gt;0,ISNUMBER(N63),N63&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),I11*2^30/B11/(M63*1e6),NA())</x:f>
         <x:v>301.00608</x:v>
       </x:c>
-      <x:c r="D63" s="25" t="n">
+      <x:c r="D63" s="9" t="n">
         <x:f>C63*(1+$H$55*$F$55/(1-$F$55))</x:f>
         <x:v>334.45120000000003</x:v>
       </x:c>
-      <x:c r="E63" s="25" t="n">
+      <x:c r="E63" s="9" t="n">
         <x:f>(D63-C63)*$J$55</x:f>
         <x:v>33.44512000000003</x:v>
       </x:c>
-      <x:c r="F63" s="25" t="n">
+      <x:c r="F63" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(M63),M63&gt;0,ISNUMBER(N63),N63&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),J11*2^30/B11/(N63*1e6),NA())</x:f>
         <x:v>19.6146</x:v>
       </x:c>
-      <x:c r="G63" s="25" t="n">
+      <x:c r="G63" s="9" t="n">
         <x:f>F63*(1+$H$55*$F$55/(1-$F$55))</x:f>
         <x:v>21.794</x:v>
       </x:c>
-      <x:c r="H63" s="25" t="n">
+      <x:c r="H63" s="9" t="n">
         <x:f>(G63-F63)*$J$55</x:f>
         <x:v>2.179400000000001</x:v>
       </x:c>
-      <x:c r="I63" s="27"/>
-      <x:c r="J63" s="26" t="str">
+      <x:c r="I63" s="44"/>
+      <x:c r="J63" s="35" t="str">
         <x:f>IF(AND(ISNUMBER(I63),I63&gt;0,I63&gt;=C63*$J$55),E63/I63,"")</x:f>
       </x:c>
-      <x:c r="K63" s="27"/>
-      <x:c r="L63" s="26" t="str">
+      <x:c r="K63" s="44"/>
+      <x:c r="L63" s="35" t="str">
         <x:f>IF(AND(ISNUMBER(K63),K63&gt;0,K63&gt;=F63*$J$55),H63/K63,"")</x:f>
       </x:c>
-      <x:c r="M63" s="28" t="n">
+      <x:c r="M63" s="43" t="n">
         <x:f>$B$55</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="N63" s="28" t="n">
+      <x:c r="N63" s="43" t="n">
         <x:f>$D$55</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="O63" s="17" t="str">
+      <x:c r="O63" s="2" t="str">
         <x:v>仅EP；总耗时需实测基线</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="25" customHeight="1">
-      <x:c r="A64" s="17" t="str">
+      <x:c r="A64" s="2" t="str">
         <x:f>A12</x:f>
         <x:v>KimiK3</x:v>
       </x:c>
-      <x:c r="B64" s="17" t="n">
+      <x:c r="B64" s="2" t="n">
         <x:f>B12</x:f>
         <x:v>32</x:v>
       </x:c>
-      <x:c r="C64" s="25" t="n">
+      <x:c r="C64" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(M64),M64&gt;0,ISNUMBER(N64),N64&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),I12*2^30/B12/(M64*1e6),NA())</x:f>
         <x:v>837.45306624</x:v>
       </x:c>
-      <x:c r="D64" s="25" t="n">
+      <x:c r="D64" s="9" t="n">
         <x:f>C64*(1+$H$55*$F$55/(1-$F$55))</x:f>
         <x:v>930.5034069333334</x:v>
       </x:c>
-      <x:c r="E64" s="25" t="n">
+      <x:c r="E64" s="9" t="n">
         <x:f>(D64-C64)*$J$55</x:f>
         <x:v>93.0503406933334</x:v>
       </x:c>
-      <x:c r="F64" s="25" t="n">
+      <x:c r="F64" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(M64),M64&gt;0,ISNUMBER(N64),N64&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),J12*2^30/B12/(N64*1e6),NA())</x:f>
         <x:v>6.8082944</x:v>
       </x:c>
-      <x:c r="G64" s="25" t="n">
+      <x:c r="G64" s="9" t="n">
         <x:f>F64*(1+$H$55*$F$55/(1-$F$55))</x:f>
         <x:v>7.564771555555557</x:v>
       </x:c>
-      <x:c r="H64" s="25" t="n">
+      <x:c r="H64" s="9" t="n">
         <x:f>(G64-F64)*$J$55</x:f>
         <x:v>0.7564771555555563</x:v>
       </x:c>
-      <x:c r="I64" s="27"/>
-      <x:c r="J64" s="26" t="str">
+      <x:c r="I64" s="44"/>
+      <x:c r="J64" s="35" t="str">
         <x:f>IF(AND(ISNUMBER(I64),I64&gt;0,I64&gt;=C64*$J$55),E64/I64,"")</x:f>
       </x:c>
-      <x:c r="K64" s="27"/>
-      <x:c r="L64" s="26" t="str">
+      <x:c r="K64" s="44"/>
+      <x:c r="L64" s="35" t="str">
         <x:f>IF(AND(ISNUMBER(K64),K64&gt;0,K64&gt;=F64*$J$55),H64/K64,"")</x:f>
       </x:c>
-      <x:c r="M64" s="28" t="n">
+      <x:c r="M64" s="43" t="n">
         <x:f>$B$55</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="N64" s="28" t="n">
+      <x:c r="N64" s="43" t="n">
         <x:f>$D$55</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="O64" s="17" t="str">
+      <x:c r="O64" s="2" t="str">
         <x:v>仅EP；总耗时需实测基线</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="25" customHeight="1">
-      <x:c r="A65" s="17" t="str">
+      <x:c r="A65" s="2" t="str">
         <x:f>A13</x:f>
         <x:v>KimiK3</x:v>
       </x:c>
-      <x:c r="B65" s="17" t="n">
+      <x:c r="B65" s="2" t="n">
         <x:f>B13</x:f>
         <x:v>256</x:v>
       </x:c>
-      <x:c r="C65" s="25" t="n">
+      <x:c r="C65" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(M65),M65&gt;0,ISNUMBER(N65),N65&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),I13*2^30/B13/(M65*1e6),NA())</x:f>
         <x:v>861.9466752</x:v>
       </x:c>
-      <x:c r="D65" s="25" t="n">
+      <x:c r="D65" s="9" t="n">
         <x:f>C65*(1+$H$55*$F$55/(1-$F$55))</x:f>
         <x:v>957.718528</x:v>
       </x:c>
-      <x:c r="E65" s="25" t="n">
+      <x:c r="E65" s="9" t="n">
         <x:f>(D65-C65)*$J$55</x:f>
         <x:v>95.77185280000003</x:v>
       </x:c>
-      <x:c r="F65" s="25" t="n">
+      <x:c r="F65" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(M65),M65&gt;0,ISNUMBER(N65),N65&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),J13*2^30/B13/(N65*1e6),NA())</x:f>
         <x:v>7.0042176</x:v>
       </x:c>
-      <x:c r="G65" s="25" t="n">
+      <x:c r="G65" s="9" t="n">
         <x:f>F65*(1+$H$55*$F$55/(1-$F$55))</x:f>
         <x:v>7.782464</x:v>
       </x:c>
-      <x:c r="H65" s="25" t="n">
+      <x:c r="H65" s="9" t="n">
         <x:f>(G65-F65)*$J$55</x:f>
         <x:v>0.7782464000000004</x:v>
       </x:c>
-      <x:c r="I65" s="27"/>
-      <x:c r="J65" s="26" t="str">
+      <x:c r="I65" s="44"/>
+      <x:c r="J65" s="35" t="str">
         <x:f>IF(AND(ISNUMBER(I65),I65&gt;0,I65&gt;=C65*$J$55),E65/I65,"")</x:f>
       </x:c>
-      <x:c r="K65" s="27"/>
-      <x:c r="L65" s="26" t="str">
+      <x:c r="K65" s="44"/>
+      <x:c r="L65" s="35" t="str">
         <x:f>IF(AND(ISNUMBER(K65),K65&gt;0,K65&gt;=F65*$J$55),H65/K65,"")</x:f>
       </x:c>
-      <x:c r="M65" s="28" t="n">
+      <x:c r="M65" s="43" t="n">
         <x:f>$B$55</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="N65" s="28" t="n">
+      <x:c r="N65" s="43" t="n">
         <x:f>$D$55</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="O65" s="17" t="str">
+      <x:c r="O65" s="2" t="str">
         <x:v>仅EP；总耗时需实测基线</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="25" customHeight="1">
-      <x:c r="A66" s="17" t="str">
+      <x:c r="A66" s="2" t="str">
         <x:f>A14</x:f>
         <x:v>Qwen3.8 2.4T</x:v>
       </x:c>
-      <x:c r="B66" s="17" t="n">
+      <x:c r="B66" s="2" t="n">
         <x:f>B14</x:f>
         <x:v>32</x:v>
       </x:c>
-      <x:c r="C66" s="25" t="n">
+      <x:c r="C66" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(M66),M66&gt;0,ISNUMBER(N66),N66&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),I14*2^30/B14/(M66*1e6),NA())</x:f>
         <x:v>598.16615936</x:v>
       </x:c>
-      <x:c r="D66" s="25" t="n">
+      <x:c r="D66" s="9" t="n">
         <x:f>C66*(1+$H$55*$F$55/(1-$F$55))</x:f>
         <x:v>664.6290659555557</x:v>
       </x:c>
-      <x:c r="E66" s="25" t="n">
+      <x:c r="E66" s="9" t="n">
         <x:f>(D66-C66)*$J$55</x:f>
         <x:v>66.46290659555564</x:v>
       </x:c>
-      <x:c r="F66" s="25" t="n">
+      <x:c r="F66" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(M66),M66&gt;0,ISNUMBER(N66),N66&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),J14*2^30/B14/(N66*1e6),NA())</x:f>
         <x:v>4.91091584</x:v>
       </x:c>
-      <x:c r="G66" s="25" t="n">
+      <x:c r="G66" s="9" t="n">
         <x:f>F66*(1+$H$55*$F$55/(1-$F$55))</x:f>
         <x:v>5.4565731555555566</x:v>
       </x:c>
-      <x:c r="H66" s="25" t="n">
+      <x:c r="H66" s="9" t="n">
         <x:f>(G66-F66)*$J$55</x:f>
         <x:v>0.5456573155555562</x:v>
       </x:c>
-      <x:c r="I66" s="27"/>
-      <x:c r="J66" s="26" t="str">
+      <x:c r="I66" s="44"/>
+      <x:c r="J66" s="35" t="str">
         <x:f>IF(AND(ISNUMBER(I66),I66&gt;0,I66&gt;=C66*$J$55),E66/I66,"")</x:f>
       </x:c>
-      <x:c r="K66" s="27"/>
-      <x:c r="L66" s="26" t="str">
+      <x:c r="K66" s="44"/>
+      <x:c r="L66" s="35" t="str">
         <x:f>IF(AND(ISNUMBER(K66),K66&gt;0,K66&gt;=F66*$J$55),H66/K66,"")</x:f>
       </x:c>
-      <x:c r="M66" s="28" t="n">
+      <x:c r="M66" s="43" t="n">
         <x:f>$B$55</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="N66" s="28" t="n">
+      <x:c r="N66" s="43" t="n">
         <x:f>$D$55</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="O66" s="17" t="str">
+      <x:c r="O66" s="2" t="str">
         <x:v>仅EP；总耗时需实测基线</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="25" customHeight="1">
-      <x:c r="A67" s="17" t="str">
+      <x:c r="A67" s="2" t="str">
         <x:f>A15</x:f>
         <x:v>Qwen3.8 2.4T</x:v>
       </x:c>
-      <x:c r="B67" s="17" t="n">
+      <x:c r="B67" s="2" t="n">
         <x:f>B15</x:f>
         <x:v>256</x:v>
       </x:c>
-      <x:c r="C67" s="25" t="n">
+      <x:c r="C67" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(M67),M67&gt;0,ISNUMBER(N67),N67&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),I15*2^30/B15/(M67*1e6),NA())</x:f>
         <x:v>615.4702848</x:v>
       </x:c>
-      <x:c r="D67" s="25" t="n">
+      <x:c r="D67" s="9" t="n">
         <x:f>C67*(1+$H$55*$F$55/(1-$F$55))</x:f>
         <x:v>683.855872</x:v>
       </x:c>
-      <x:c r="E67" s="25" t="n">
+      <x:c r="E67" s="9" t="n">
         <x:f>(D67-C67)*$J$55</x:f>
         <x:v>68.38558720000003</x:v>
       </x:c>
-      <x:c r="F67" s="25" t="n">
+      <x:c r="F67" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(M67),M67&gt;0,ISNUMBER(N67),N67&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),J15*2^30/B15/(N67*1e6),NA())</x:f>
         <x:v>5.0495304</x:v>
       </x:c>
-      <x:c r="G67" s="25" t="n">
+      <x:c r="G67" s="9" t="n">
         <x:f>F67*(1+$H$55*$F$55/(1-$F$55))</x:f>
         <x:v>5.610589333333333</x:v>
       </x:c>
-      <x:c r="H67" s="25" t="n">
+      <x:c r="H67" s="9" t="n">
         <x:f>(G67-F67)*$J$55</x:f>
         <x:v>0.5610589333333333</x:v>
       </x:c>
-      <x:c r="I67" s="27"/>
-      <x:c r="J67" s="26" t="str">
+      <x:c r="I67" s="44"/>
+      <x:c r="J67" s="35" t="str">
         <x:f>IF(AND(ISNUMBER(I67),I67&gt;0,I67&gt;=C67*$J$55),E67/I67,"")</x:f>
       </x:c>
-      <x:c r="K67" s="27"/>
-      <x:c r="L67" s="26" t="str">
+      <x:c r="K67" s="44"/>
+      <x:c r="L67" s="35" t="str">
         <x:f>IF(AND(ISNUMBER(K67),K67&gt;0,K67&gt;=F67*$J$55),H67/K67,"")</x:f>
       </x:c>
-      <x:c r="M67" s="28" t="n">
+      <x:c r="M67" s="43" t="n">
         <x:f>$B$55</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="N67" s="28" t="n">
+      <x:c r="N67" s="43" t="n">
         <x:f>$D$55</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="O67" s="17" t="str">
+      <x:c r="O67" s="2" t="str">
         <x:v>仅EP；总耗时需实测基线</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="25" customHeight="1">
-      <x:c r="A68" s="17" t="str">
+      <x:c r="A68" s="2" t="str">
         <x:f>A16</x:f>
         <x:v>DS V4.1 Flash</x:v>
       </x:c>
-      <x:c r="B68" s="17" t="n">
+      <x:c r="B68" s="2" t="n">
         <x:f>B16</x:f>
         <x:v>32</x:v>
       </x:c>
-      <x:c r="C68" s="25" t="n">
+      <x:c r="C68" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(M68),M68&gt;0,ISNUMBER(N68),N68&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),I16*2^30/B16/(M68*1e6),NA())</x:f>
         <x:v>97.5366144</x:v>
       </x:c>
-      <x:c r="D68" s="25" t="n">
+      <x:c r="D68" s="9" t="n">
         <x:f>C68*(1+$H$55*$F$55/(1-$F$55))</x:f>
         <x:v>108.37401600000001</x:v>
       </x:c>
-      <x:c r="E68" s="25" t="n">
+      <x:c r="E68" s="9" t="n">
         <x:f>(D68-C68)*$J$55</x:f>
         <x:v>10.837401600000007</x:v>
       </x:c>
-      <x:c r="F68" s="25" t="n">
+      <x:c r="F68" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(M68),M68&gt;0,ISNUMBER(N68),N68&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),J16*2^30/B16/(N68*1e6),NA())</x:f>
         <x:v>6.4138752</x:v>
       </x:c>
-      <x:c r="G68" s="25" t="n">
+      <x:c r="G68" s="9" t="n">
         <x:f>F68*(1+$H$55*$F$55/(1-$F$55))</x:f>
         <x:v>7.1265279999999995</x:v>
       </x:c>
-      <x:c r="H68" s="25" t="n">
+      <x:c r="H68" s="9" t="n">
         <x:f>(G68-F68)*$J$55</x:f>
         <x:v>0.7126527999999999</x:v>
       </x:c>
-      <x:c r="I68" s="27"/>
-      <x:c r="J68" s="26" t="str">
+      <x:c r="I68" s="44"/>
+      <x:c r="J68" s="35" t="str">
         <x:f>IF(AND(ISNUMBER(I68),I68&gt;0,I68&gt;=C68*$J$55),E68/I68,"")</x:f>
       </x:c>
-      <x:c r="K68" s="27"/>
-      <x:c r="L68" s="26" t="str">
+      <x:c r="K68" s="44"/>
+      <x:c r="L68" s="35" t="str">
         <x:f>IF(AND(ISNUMBER(K68),K68&gt;0,K68&gt;=F68*$J$55),H68/K68,"")</x:f>
       </x:c>
-      <x:c r="M68" s="28" t="n">
+      <x:c r="M68" s="43" t="n">
         <x:f>$B$55</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="N68" s="28" t="n">
+      <x:c r="N68" s="43" t="n">
         <x:f>$D$55</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="O68" s="17" t="str">
+      <x:c r="O68" s="2" t="str">
         <x:v>仅EP；V4.1 PD条件评估</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="25" customHeight="1">
-      <x:c r="A69" s="17" t="str">
+      <x:c r="A69" s="2" t="str">
         <x:f>A17</x:f>
         <x:v>DS V4.1 Flash</x:v>
       </x:c>
-      <x:c r="B69" s="17" t="n">
+      <x:c r="B69" s="2" t="n">
         <x:f>B17</x:f>
         <x:v>256</x:v>
       </x:c>
-      <x:c r="C69" s="25" t="n">
+      <x:c r="C69" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(M69),M69&gt;0,ISNUMBER(N69),N69&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),I17*2^30/B17/(M69*1e6),NA())</x:f>
         <x:v>100.478976</x:v>
       </x:c>
-      <x:c r="D69" s="25" t="n">
+      <x:c r="D69" s="9" t="n">
         <x:f>C69*(1+$H$55*$F$55/(1-$F$55))</x:f>
         <x:v>111.64330666666667</x:v>
       </x:c>
-      <x:c r="E69" s="25" t="n">
+      <x:c r="E69" s="9" t="n">
         <x:f>(D69-C69)*$J$55</x:f>
         <x:v>11.164330666666672</x:v>
       </x:c>
-      <x:c r="F69" s="25" t="n">
+      <x:c r="F69" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(M69),M69&gt;0,ISNUMBER(N69),N69&gt;0,ISNUMBER($F$55),$F$55&gt;=0,$F$55&lt;1,ISNUMBER($H$55),$H$55&gt;=0,$H$55&lt;=1,ISNUMBER($J$55),$J$55&gt;=0,$J$55&lt;=1),J17*2^30/B17/(N69*1e6),NA())</x:f>
         <x:v>6.596544</x:v>
       </x:c>
-      <x:c r="G69" s="25" t="n">
+      <x:c r="G69" s="9" t="n">
         <x:f>F69*(1+$H$55*$F$55/(1-$F$55))</x:f>
         <x:v>7.329493333333334</x:v>
       </x:c>
-      <x:c r="H69" s="25" t="n">
+      <x:c r="H69" s="9" t="n">
         <x:f>(G69-F69)*$J$55</x:f>
         <x:v>0.7329493333333339</x:v>
       </x:c>
-      <x:c r="I69" s="27"/>
-      <x:c r="J69" s="26" t="str">
+      <x:c r="I69" s="44"/>
+      <x:c r="J69" s="35" t="str">
         <x:f>IF(AND(ISNUMBER(I69),I69&gt;0,I69&gt;=C69*$J$55),E69/I69,"")</x:f>
       </x:c>
-      <x:c r="K69" s="27"/>
-      <x:c r="L69" s="26" t="str">
+      <x:c r="K69" s="44"/>
+      <x:c r="L69" s="35" t="str">
         <x:f>IF(AND(ISNUMBER(K69),K69&gt;0,K69&gt;=F69*$J$55),H69/K69,"")</x:f>
       </x:c>
-      <x:c r="M69" s="28" t="n">
+      <x:c r="M69" s="43" t="n">
         <x:f>$B$55</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="N69" s="28" t="n">
+      <x:c r="N69" s="43" t="n">
         <x:f>$D$55</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="O69" s="17" t="str">
+      <x:c r="O69" s="2" t="str">
         <x:v>仅EP；V4.1 PD条件评估</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="25" customHeight="1">
-      <x:c r="A70" s="17"/>
-      <x:c r="B70" s="17"/>
-      <x:c r="C70" s="17"/>
-      <x:c r="D70" s="17"/>
-      <x:c r="E70" s="17"/>
-      <x:c r="F70" s="17"/>
-      <x:c r="G70" s="17"/>
-      <x:c r="H70" s="17"/>
-      <x:c r="I70" s="17"/>
-      <x:c r="J70" s="17"/>
-      <x:c r="K70" s="17"/>
-      <x:c r="L70" s="17"/>
-      <x:c r="M70" s="17"/>
-      <x:c r="N70" s="17"/>
-      <x:c r="O70" s="17"/>
+      <x:c r="A70" s="2"/>
+      <x:c r="B70" s="2"/>
+      <x:c r="C70" s="2"/>
+      <x:c r="D70" s="2"/>
+      <x:c r="E70" s="2"/>
+      <x:c r="F70" s="2"/>
+      <x:c r="G70" s="2"/>
+      <x:c r="H70" s="2"/>
+      <x:c r="I70" s="2"/>
+      <x:c r="J70" s="2"/>
+      <x:c r="K70" s="2"/>
+      <x:c r="L70" s="2"/>
+      <x:c r="M70" s="2"/>
+      <x:c r="N70" s="2"/>
+      <x:c r="O70" s="2"/>
     </x:row>
     <x:row r="71" ht="25" customHeight="1">
-      <x:c r="A71" s="17" t="str">
+      <x:c r="A71" s="2" t="str">
         <x:v>带宽下降 10% 对受影响带宽项增加 11.11%。forward 增幅还需真实基线；不把 KV 交接等待再加到每个 Decode Step。</x:v>
       </x:c>
-      <x:c r="B71" s="17"/>
-      <x:c r="C71" s="17"/>
-      <x:c r="D71" s="17"/>
-      <x:c r="E71" s="17"/>
-      <x:c r="F71" s="17"/>
-      <x:c r="G71" s="17"/>
-      <x:c r="H71" s="17"/>
-      <x:c r="I71" s="17"/>
-      <x:c r="J71" s="17"/>
-      <x:c r="K71" s="17"/>
-      <x:c r="L71" s="17"/>
-      <x:c r="M71" s="17"/>
-      <x:c r="N71" s="17"/>
-      <x:c r="O71" s="17"/>
+      <x:c r="B71" s="2"/>
+      <x:c r="C71" s="2"/>
+      <x:c r="D71" s="2"/>
+      <x:c r="E71" s="2"/>
+      <x:c r="F71" s="2"/>
+      <x:c r="G71" s="2"/>
+      <x:c r="H71" s="2"/>
+      <x:c r="I71" s="2"/>
+      <x:c r="J71" s="2"/>
+      <x:c r="K71" s="2"/>
+      <x:c r="L71" s="2"/>
+      <x:c r="M71" s="2"/>
+      <x:c r="N71" s="2"/>
+      <x:c r="O71" s="2"/>
     </x:row>
     <x:row r="72" ht="25" customHeight="1">
-      <x:c r="A72" s="17"/>
-      <x:c r="B72" s="17"/>
-      <x:c r="C72" s="17"/>
-      <x:c r="D72" s="17"/>
-      <x:c r="E72" s="17"/>
-      <x:c r="F72" s="17"/>
-      <x:c r="G72" s="17"/>
-      <x:c r="H72" s="17"/>
-      <x:c r="I72" s="17"/>
-      <x:c r="J72" s="17"/>
-      <x:c r="K72" s="17"/>
-      <x:c r="L72" s="17"/>
-      <x:c r="M72" s="17"/>
-      <x:c r="N72" s="17"/>
-      <x:c r="O72" s="17"/>
+      <x:c r="A72" s="2"/>
+      <x:c r="B72" s="2"/>
+      <x:c r="C72" s="2"/>
+      <x:c r="D72" s="2"/>
+      <x:c r="E72" s="2"/>
+      <x:c r="F72" s="2"/>
+      <x:c r="G72" s="2"/>
+      <x:c r="H72" s="2"/>
+      <x:c r="I72" s="2"/>
+      <x:c r="J72" s="2"/>
+      <x:c r="K72" s="2"/>
+      <x:c r="L72" s="2"/>
+      <x:c r="M72" s="2"/>
+      <x:c r="N72" s="2"/>
+      <x:c r="O72" s="2"/>
     </x:row>
     <x:row r="73" ht="25" customHeight="1">
-      <x:c r="A73" s="17" t="str">
+      <x:c r="A73" s="2" t="str">
         <x:v>黄色 M/N 列可填各模型、各 EP 的无争用有效带宽，GB/s=10⁹ B/s。默认共享比例为 1；逐模型表可按事件调整。</x:v>
       </x:c>
-      <x:c r="B73" s="17"/>
-      <x:c r="C73" s="17"/>
-      <x:c r="D73" s="17"/>
-      <x:c r="E73" s="17"/>
-      <x:c r="F73" s="17"/>
-      <x:c r="G73" s="17"/>
-      <x:c r="H73" s="17"/>
-      <x:c r="I73" s="17"/>
-      <x:c r="J73" s="17"/>
-      <x:c r="K73" s="17"/>
-      <x:c r="L73" s="17"/>
-      <x:c r="M73" s="17"/>
-      <x:c r="N73" s="17"/>
-      <x:c r="O73" s="17"/>
+      <x:c r="B73" s="2"/>
+      <x:c r="C73" s="2"/>
+      <x:c r="D73" s="2"/>
+      <x:c r="E73" s="2"/>
+      <x:c r="F73" s="2"/>
+      <x:c r="G73" s="2"/>
+      <x:c r="H73" s="2"/>
+      <x:c r="I73" s="2"/>
+      <x:c r="J73" s="2"/>
+      <x:c r="K73" s="2"/>
+      <x:c r="L73" s="2"/>
+      <x:c r="M73" s="2"/>
+      <x:c r="N73" s="2"/>
+      <x:c r="O73" s="2"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Remove V4.1 planning labels from editable workbooks
</commit_message>
<xml_diff>
--- a/examples/kv-ep-sweep/kv-ep32-ep256.xlsx
+++ b/examples/kv-ep-sweep/kv-ep32-ep256.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规格汇总" sheetId="1" r:id="R0b06d05ee9d5473e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KV明细" sheetId="2" r:id="R6ec9d229fbce4d72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EP通信" sheetId="3" r:id="Rccfded5c9169426d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分钟场景" sheetId="4" r:id="Rf80536f8dfe34d1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规格汇总" sheetId="1" r:id="R1d47e198ab0e4634"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KV明细" sheetId="2" r:id="R7d640cce8b1f4a4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EP通信" sheetId="3" r:id="R40d4b3d93e004840"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分钟场景" sheetId="4" r:id="R7e6ad5c18ec84a60"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1561,7 +1561,7 @@
       </x:c>
       <x:c r="M16" s="58" t="str">
         <x:f>M34</x:f>
-        <x:v>取为规划值；迁移未支持</x:v>
+        <x:v>专家数整除</x:v>
       </x:c>
       <x:c r="N16" s="59"/>
       <x:c r="O16" s="59"/>
@@ -1617,7 +1617,7 @@
       </x:c>
       <x:c r="M17" s="58" t="str">
         <x:f>M35</x:f>
-        <x:v>补128槽并验证；取为规划值</x:v>
+        <x:v>需补齐128槽并验证EPLB</x:v>
       </x:c>
       <x:c r="N17" s="59"/>
       <x:c r="O17" s="59"/>
@@ -1677,7 +1677,7 @@
     </x:row>
     <x:row r="21" ht="18" customHeight="1">
       <x:c r="A21" s="58" t="str">
-        <x:v>单位 GiB。存＝生成 KV 行＋最终辅助状态；取＝P→D 张量字节。V4.1 的取仅为规划值，main 未支持迁移。</x:v>
+        <x:v>单位 GiB。存＝生成 KV 行＋最终辅助状态；取＝P→D 张量字节。</x:v>
       </x:c>
       <x:c r="B21" s="58"/>
       <x:c r="C21" s="58"/>
@@ -1734,19 +1734,19 @@
         <x:v>存/请求</x:v>
       </x:c>
       <x:c r="H23" s="70" t="str">
-        <x:v>取或规划取/请求</x:v>
+        <x:v>取/请求</x:v>
       </x:c>
       <x:c r="I23" s="70" t="str">
         <x:v>存/P DP批</x:v>
       </x:c>
       <x:c r="J23" s="70" t="str">
-        <x:v>取或规划取/批</x:v>
+        <x:v>取/批</x:v>
       </x:c>
       <x:c r="K23" s="70" t="str">
         <x:v>存/P整组</x:v>
       </x:c>
       <x:c r="L23" s="70" t="str">
-        <x:v>取或规划取/整组</x:v>
+        <x:v>取/整组</x:v>
       </x:c>
       <x:c r="M23" s="70" t="str">
         <x:v>部署 / 迁移条件</x:v>
@@ -2364,8 +2364,8 @@
         <x:v>45.7265625</x:v>
       </x:c>
       <x:c r="M34" s="58" t="str">
-        <x:f>IF('EP通信'!H20&gt;0,"补128槽并验证；取为规划值","取为规划值；迁移未支持")</x:f>
-        <x:v>取为规划值；迁移未支持</x:v>
+        <x:f>IF('EP通信'!H20&gt;0,"需补齐128槽并验证EPLB","专家数整除")</x:f>
+        <x:v>专家数整除</x:v>
       </x:c>
       <x:c r="N34" s="59"/>
       <x:c r="O34" s="59"/>
@@ -2420,8 +2420,8 @@
         <x:v>365.8125</x:v>
       </x:c>
       <x:c r="M35" s="58" t="str">
-        <x:f>IF('EP通信'!H21&gt;0,"补128槽并验证；取为规划值","取为规划值；迁移未支持")</x:f>
-        <x:v>补128槽并验证；取为规划值</x:v>
+        <x:f>IF('EP通信'!H21&gt;0,"需补齐128槽并验证EPLB","专家数整除")</x:f>
+        <x:v>需补齐128槽并验证EPLB</x:v>
       </x:c>
       <x:c r="N35" s="59"/>
       <x:c r="O35" s="59"/>
@@ -2571,7 +2571,7 @@
     </x:row>
     <x:row r="44" ht="18" customHeight="1">
       <x:c r="A44" s="58" t="str">
-        <x:v>V4.1：完成 S tokens 后交接；长 KV / Indexer 只计 4 个源层，SWA 尾块和 32 行环形页按规划传输。</x:v>
+        <x:v>V4.1：完成 S tokens 后交接；长 KV / Indexer 只计 4 个源层，SWA 尾块和 32 行环形页按完整块传输。</x:v>
       </x:c>
       <x:c r="B44" s="58"/>
       <x:c r="C44" s="58"/>
@@ -3754,7 +3754,7 @@
         <x:v>P 保留行</x:v>
       </x:c>
       <x:c r="G8" s="70" t="str">
-        <x:v>D 取/规划行</x:v>
+        <x:v>D 取行</x:v>
       </x:c>
       <x:c r="H8" s="70" t="str">
         <x:v>P 副本/分片</x:v>
@@ -3769,7 +3769,7 @@
         <x:v>保留 GiB</x:v>
       </x:c>
       <x:c r="L8" s="70" t="str">
-        <x:v>取/规划 GiB</x:v>
+        <x:v>取 GiB</x:v>
       </x:c>
       <x:c r="M8" s="58"/>
     </x:row>
@@ -5021,9 +5021,7 @@
         <x:f>C41*D41*G41*I41/2^30</x:f>
         <x:v>0.009765625</x:v>
       </x:c>
-      <x:c r="M41" s="58" t="str">
-        <x:v>迁移未支持；取为规划值</x:v>
-      </x:c>
+      <x:c r="M41" s="58" t="str"/>
     </x:row>
     <x:row r="42" ht="22" customHeight="1">
       <x:c r="A42" s="58" t="str">
@@ -5068,9 +5066,7 @@
         <x:f>C42*D42*G42*I42/2^30</x:f>
         <x:v>0.375</x:v>
       </x:c>
-      <x:c r="M42" s="58" t="str">
-        <x:v>迁移未支持；取为规划值</x:v>
-      </x:c>
+      <x:c r="M42" s="58" t="str"/>
     </x:row>
     <x:row r="43" ht="22" customHeight="1">
       <x:c r="A43" s="58" t="str">
@@ -5115,9 +5111,7 @@
         <x:f>C43*D43*G43*I43/2^30</x:f>
         <x:v>0.047607421875</x:v>
       </x:c>
-      <x:c r="M43" s="58" t="str">
-        <x:v>迁移未支持；取为规划值</x:v>
-      </x:c>
+      <x:c r="M43" s="58" t="str"/>
     </x:row>
     <x:row r="44" ht="22" customHeight="1">
       <x:c r="A44" s="58" t="str">
@@ -5162,9 +5156,7 @@
         <x:f>C44*D44*G44*I44/2^30</x:f>
         <x:v>0.25</x:v>
       </x:c>
-      <x:c r="M44" s="58" t="str">
-        <x:v>迁移未支持；取为规划值</x:v>
-      </x:c>
+      <x:c r="M44" s="58" t="str"/>
     </x:row>
     <x:row r="45" ht="22" customHeight="1">
       <x:c r="A45" s="58" t="str">
@@ -5209,9 +5201,7 @@
         <x:f>C45*D45*G45*I45/2^30</x:f>
         <x:v>0.03173828125</x:v>
       </x:c>
-      <x:c r="M45" s="58" t="str">
-        <x:v>迁移未支持；取为规划值</x:v>
-      </x:c>
+      <x:c r="M45" s="58" t="str"/>
     </x:row>
     <x:row r="46" ht="22" customHeight="1">
       <x:c r="A46" s="58" t="str">
@@ -5256,9 +5246,7 @@
         <x:f>C46*D46*G46*I46/2^30</x:f>
         <x:v>0.0003662109375</x:v>
       </x:c>
-      <x:c r="M46" s="58" t="str">
-        <x:v>迁移未支持；取为规划值</x:v>
-      </x:c>
+      <x:c r="M46" s="58" t="str"/>
     </x:row>
     <x:row r="47" ht="22" customHeight="1">
       <x:c r="A47" s="81" t="str">
@@ -5384,7 +5372,7 @@
     </x:row>
     <x:row r="54" ht="22" customHeight="1">
       <x:c r="A54" s="58" t="str">
-        <x:v>V4.1：S tokens 快照；C2 物理页 B/2 行，只计完成的压缩对；环形 state 规划传完整 32 行页。</x:v>
+        <x:v>V4.1：S tokens 快照；C2 物理页 B/2 行，只计完成的压缩对；环形 state 传完整 32 行页。</x:v>
       </x:c>
       <x:c r="B54" s="58"/>
       <x:c r="C54" s="62"/>
@@ -9088,9 +9076,7 @@
         <x:f>$J$9</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="O33" s="58" t="str">
-        <x:v>V4.1 KV 规划</x:v>
-      </x:c>
+      <x:c r="O33" s="58" t="str"/>
       <x:c r="P33" s="101" t="n">
         <x:f>$F$11</x:f>
         <x:v>4800</x:v>
@@ -9166,7 +9152,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O34" s="58" t="str">
-        <x:v>V4.1 KV 规划；需 128 个冗余专家槽</x:v>
+        <x:v>需 128 个冗余专家槽</x:v>
       </x:c>
       <x:c r="P34" s="101" t="n">
         <x:f>$F$11</x:f>
@@ -19623,8 +19609,7 @@
         <x:v>0.01784768662115556</x:v>
       </x:c>
       <x:c r="O160" s="58" t="str">
-        <x:f>IF(W310="","V4.1 规划",W310)</x:f>
-        <x:v>V4.1 规划</x:v>
+        <x:f>IF(W310="","",W310)</x:f>
       </x:c>
       <x:c r="P160" s="88" t="n">
         <x:f>Q310</x:f>
@@ -19709,8 +19694,7 @@
         <x:v>0.00892384331057778</x:v>
       </x:c>
       <x:c r="O161" s="58" t="str">
-        <x:f>IF(W311="","V4.1 规划",W311)</x:f>
-        <x:v>V4.1 规划</x:v>
+        <x:f>IF(W311="","",W311)</x:f>
       </x:c>
       <x:c r="P161" s="88" t="n">
         <x:f>Q311</x:f>
@@ -19795,8 +19779,7 @@
         <x:v>0.00446192165528889</x:v>
       </x:c>
       <x:c r="O162" s="58" t="str">
-        <x:f>IF(W312="","V4.1 规划",W312)</x:f>
-        <x:v>V4.1 规划</x:v>
+        <x:f>IF(W312="","",W312)</x:f>
       </x:c>
       <x:c r="P162" s="88" t="n">
         <x:f>Q312</x:f>
@@ -19881,8 +19864,7 @@
         <x:v>0.0029746144368592593</x:v>
       </x:c>
       <x:c r="O163" s="58" t="str">
-        <x:f>IF(W313="","V4.1 规划",W313)</x:f>
-        <x:v>V4.1 规划</x:v>
+        <x:f>IF(W313="","",W313)</x:f>
       </x:c>
       <x:c r="P163" s="88" t="n">
         <x:f>Q313</x:f>
@@ -19967,8 +19949,7 @@
         <x:v>0.04743094165489779</x:v>
       </x:c>
       <x:c r="O164" s="58" t="str">
-        <x:f>IF(W314="","V4.1 规划",W314)</x:f>
-        <x:v>V4.1 规划</x:v>
+        <x:f>IF(W314="","",W314)</x:f>
       </x:c>
       <x:c r="P164" s="88" t="n">
         <x:f>Q314</x:f>
@@ -20053,8 +20034,7 @@
         <x:v>0.023715470827448897</x:v>
       </x:c>
       <x:c r="O165" s="58" t="str">
-        <x:f>IF(W315="","V4.1 规划",W315)</x:f>
-        <x:v>V4.1 规划</x:v>
+        <x:f>IF(W315="","",W315)</x:f>
       </x:c>
       <x:c r="P165" s="88" t="n">
         <x:f>Q315</x:f>
@@ -20139,8 +20119,7 @@
         <x:v>0.011857735413724448</x:v>
       </x:c>
       <x:c r="O166" s="58" t="str">
-        <x:f>IF(W316="","V4.1 规划",W316)</x:f>
-        <x:v>V4.1 规划</x:v>
+        <x:f>IF(W316="","",W316)</x:f>
       </x:c>
       <x:c r="P166" s="88" t="n">
         <x:f>Q316</x:f>
@@ -20225,8 +20204,7 @@
         <x:v>0.007905156942482965</x:v>
       </x:c>
       <x:c r="O167" s="58" t="str">
-        <x:f>IF(W317="","V4.1 规划",W317)</x:f>
-        <x:v>V4.1 规划</x:v>
+        <x:f>IF(W317="","",W317)</x:f>
       </x:c>
       <x:c r="P167" s="88" t="n">
         <x:f>Q317</x:f>
@@ -20311,8 +20289,7 @@
         <x:v>0.06259581183767705</x:v>
       </x:c>
       <x:c r="O168" s="58" t="str">
-        <x:f>IF(W318="","V4.1 规划",W318)</x:f>
-        <x:v>V4.1 规划</x:v>
+        <x:f>IF(W318="","",W318)</x:f>
       </x:c>
       <x:c r="P168" s="88" t="n">
         <x:f>Q318</x:f>
@@ -20397,8 +20374,7 @@
         <x:v>0.03129790591883853</x:v>
       </x:c>
       <x:c r="O169" s="58" t="str">
-        <x:f>IF(W319="","V4.1 规划",W319)</x:f>
-        <x:v>V4.1 规划</x:v>
+        <x:f>IF(W319="","",W319)</x:f>
       </x:c>
       <x:c r="P169" s="88" t="n">
         <x:f>Q319</x:f>
@@ -20483,8 +20459,7 @@
         <x:v>0.015648952959419263</x:v>
       </x:c>
       <x:c r="O170" s="58" t="str">
-        <x:f>IF(W320="","V4.1 规划",W320)</x:f>
-        <x:v>V4.1 规划</x:v>
+        <x:f>IF(W320="","",W320)</x:f>
       </x:c>
       <x:c r="P170" s="88" t="n">
         <x:f>Q320</x:f>
@@ -20569,8 +20544,7 @@
         <x:v>0.010432635306279508</x:v>
       </x:c>
       <x:c r="O171" s="58" t="str">
-        <x:f>IF(W321="","V4.1 规划",W321)</x:f>
-        <x:v>V4.1 规划</x:v>
+        <x:f>IF(W321="","",W321)</x:f>
       </x:c>
       <x:c r="P171" s="88" t="n">
         <x:f>Q321</x:f>
@@ -20655,8 +20629,7 @@
         <x:v>0.018351957820913582</x:v>
       </x:c>
       <x:c r="O172" s="58" t="str">
-        <x:f>IF(W322="","V4.1 规划",W322)</x:f>
-        <x:v>V4.1 规划</x:v>
+        <x:f>IF(W322="","",W322)</x:f>
       </x:c>
       <x:c r="P172" s="88" t="n">
         <x:f>Q322</x:f>
@@ -20741,8 +20714,7 @@
         <x:v>0.009175978910456791</x:v>
       </x:c>
       <x:c r="O173" s="58" t="str">
-        <x:f>IF(W323="","V4.1 规划",W323)</x:f>
-        <x:v>V4.1 规划</x:v>
+        <x:f>IF(W323="","",W323)</x:f>
       </x:c>
       <x:c r="P173" s="88" t="n">
         <x:f>Q323</x:f>
@@ -20827,8 +20799,7 @@
         <x:v>0.0045879894552283956</x:v>
       </x:c>
       <x:c r="O174" s="58" t="str">
-        <x:f>IF(W324="","V4.1 规划",W324)</x:f>
-        <x:v>V4.1 规划</x:v>
+        <x:f>IF(W324="","",W324)</x:f>
       </x:c>
       <x:c r="P174" s="88" t="n">
         <x:f>Q324</x:f>
@@ -20913,8 +20884,7 @@
         <x:v>0.00305865963681893</x:v>
       </x:c>
       <x:c r="O175" s="58" t="str">
-        <x:f>IF(W325="","V4.1 规划",W325)</x:f>
-        <x:v>V4.1 规划</x:v>
+        <x:f>IF(W325="","",W325)</x:f>
       </x:c>
       <x:c r="P175" s="88" t="n">
         <x:f>Q325</x:f>
@@ -20999,8 +20969,7 @@
         <x:v>0.04878097986640494</x:v>
       </x:c>
       <x:c r="O176" s="58" t="str">
-        <x:f>IF(W326="","V4.1 规划",W326)</x:f>
-        <x:v>V4.1 规划</x:v>
+        <x:f>IF(W326="","",W326)</x:f>
       </x:c>
       <x:c r="P176" s="88" t="n">
         <x:f>Q326</x:f>
@@ -21085,8 +21054,7 @@
         <x:v>0.02439048993320247</x:v>
       </x:c>
       <x:c r="O177" s="58" t="str">
-        <x:f>IF(W327="","V4.1 规划",W327)</x:f>
-        <x:v>V4.1 规划</x:v>
+        <x:f>IF(W327="","",W327)</x:f>
       </x:c>
       <x:c r="P177" s="88" t="n">
         <x:f>Q327</x:f>
@@ -21171,8 +21139,7 @@
         <x:v>0.012195244966601236</x:v>
       </x:c>
       <x:c r="O178" s="58" t="str">
-        <x:f>IF(W328="","V4.1 规划",W328)</x:f>
-        <x:v>V4.1 规划</x:v>
+        <x:f>IF(W328="","",W328)</x:f>
       </x:c>
       <x:c r="P178" s="88" t="n">
         <x:f>Q328</x:f>
@@ -21257,8 +21224,7 @@
         <x:v>0.008130163311067489</x:v>
       </x:c>
       <x:c r="O179" s="58" t="str">
-        <x:f>IF(W329="","V4.1 规划",W329)</x:f>
-        <x:v>V4.1 规划</x:v>
+        <x:f>IF(W329="","",W329)</x:f>
       </x:c>
       <x:c r="P179" s="88" t="n">
         <x:f>Q329</x:f>
@@ -21343,8 +21309,7 @@
         <x:v>0.06437828747783869</x:v>
       </x:c>
       <x:c r="O180" s="58" t="str">
-        <x:f>IF(W330="","V4.1 规划",W330)</x:f>
-        <x:v>V4.1 规划</x:v>
+        <x:f>IF(W330="","",W330)</x:f>
       </x:c>
       <x:c r="P180" s="88" t="n">
         <x:f>Q330</x:f>
@@ -21429,8 +21394,7 @@
         <x:v>0.032189143738919346</x:v>
       </x:c>
       <x:c r="O181" s="58" t="str">
-        <x:f>IF(W331="","V4.1 规划",W331)</x:f>
-        <x:v>V4.1 规划</x:v>
+        <x:f>IF(W331="","",W331)</x:f>
       </x:c>
       <x:c r="P181" s="88" t="n">
         <x:f>Q331</x:f>
@@ -21515,8 +21479,7 @@
         <x:v>0.016094571869459673</x:v>
       </x:c>
       <x:c r="O182" s="58" t="str">
-        <x:f>IF(W332="","V4.1 规划",W332)</x:f>
-        <x:v>V4.1 规划</x:v>
+        <x:f>IF(W332="","",W332)</x:f>
       </x:c>
       <x:c r="P182" s="88" t="n">
         <x:f>Q332</x:f>
@@ -21601,8 +21564,7 @@
         <x:v>0.01072971457963978</x:v>
       </x:c>
       <x:c r="O183" s="58" t="str">
-        <x:f>IF(W333="","V4.1 规划",W333)</x:f>
-        <x:v>V4.1 规划</x:v>
+        <x:f>IF(W333="","",W333)</x:f>
       </x:c>
       <x:c r="P183" s="88" t="n">
         <x:f>Q333</x:f>
@@ -44072,7 +44034,7 @@
         <x:v>保留行</x:v>
       </x:c>
       <x:c r="J339" s="70" t="str">
-        <x:v>取/规划行</x:v>
+        <x:v>取行</x:v>
       </x:c>
       <x:c r="K339" s="70" t="str">
         <x:v>生成 GiB</x:v>
@@ -44081,7 +44043,7 @@
         <x:v>保留 GiB</x:v>
       </x:c>
       <x:c r="M339" s="70" t="str">
-        <x:v>取/规划 GiB</x:v>
+        <x:v>取 GiB</x:v>
       </x:c>
       <x:c r="N339" s="58"/>
       <x:c r="O339" s="58"/>
@@ -49887,7 +49849,7 @@
     </x:row>
     <x:row r="445" ht="45" customHeight="1">
       <x:c r="A445" s="58" t="str">
-        <x:v>来源：库内 config.json、analysis/KV-EP-SPECS.md、analysis/PD-MINUTE.md；V4.1 为既有 KV 规划量。</x:v>
+        <x:v>来源：库内 config.json、analysis/KV-EP-SPECS.md、analysis/PD-MINUTE.md。</x:v>
       </x:c>
       <x:c r="B445" s="58"/>
       <x:c r="C445" s="58"/>

</xml_diff>

<commit_message>
Clarify PD contention inputs with English terms and inline explanations
</commit_message>
<xml_diff>
--- a/examples/kv-ep-sweep/kv-ep32-ep256.xlsx
+++ b/examples/kv-ep-sweep/kv-ep32-ep256.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规格汇总" sheetId="1" r:id="R1d47e198ab0e4634"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KV明细" sheetId="2" r:id="R7d640cce8b1f4a4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EP通信" sheetId="3" r:id="R40d4b3d93e004840"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分钟场景" sheetId="4" r:id="R7e6ad5c18ec84a60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规格汇总" sheetId="1" r:id="Rb60a63b8d3854e8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KV明细" sheetId="2" r:id="Rf8e0d8f6b8eb4b78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EP通信" sheetId="3" r:id="R38883d9a1a5f40bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分钟场景" sheetId="4" r:id="R395764b5e5a6414c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -210,7 +210,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="118">
+  <x:cellXfs count="119">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -549,6 +549,9 @@
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="209" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -7643,7 +7646,7 @@
       <x:c r="W4" s="58"/>
       <x:c r="X4" s="58"/>
     </x:row>
-    <x:row r="5" ht="18" customHeight="1">
+    <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="58" t="str">
         <x:v>每 P DP 请求数</x:v>
       </x:c>
@@ -7652,16 +7655,18 @@
       </x:c>
       <x:c r="C5" s="58"/>
       <x:c r="D5" s="58"/>
-      <x:c r="E5" s="58" t="str">
-        <x:v>P EP 组数</x:v>
+      <x:c r="E5" s="90" t="str">
+        <x:v>P deployment
+count</x:v>
       </x:c>
       <x:c r="F5" s="94" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G5" s="58"/>
       <x:c r="H5" s="58"/>
-      <x:c r="I5" s="58" t="str">
-        <x:v>D EP 组数</x:v>
+      <x:c r="I5" s="90" t="str">
+        <x:v>D deployment
+count</x:v>
       </x:c>
       <x:c r="J5" s="94" t="n">
         <x:v>1</x:v>
@@ -7779,25 +7784,28 @@
       <x:c r="W8" s="58"/>
       <x:c r="X8" s="58"/>
     </x:row>
-    <x:row r="9" ht="18" customHeight="1">
-      <x:c r="A9" s="58" t="str">
-        <x:v>每周期错峰批数</x:v>
+    <x:row r="9" ht="34" customHeight="1">
+      <x:c r="A9" s="90" t="str">
+        <x:v>KV bursts
+per interval</x:v>
       </x:c>
       <x:c r="B9" s="94" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C9" s="58"/>
       <x:c r="D9" s="58"/>
-      <x:c r="E9" s="58" t="str">
-        <x:v>EP 共享比例</x:v>
+      <x:c r="E9" s="90" t="str">
+        <x:v>EP shared
+resource fraction</x:v>
       </x:c>
       <x:c r="F9" s="98" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G9" s="58"/>
       <x:c r="H9" s="58"/>
-      <x:c r="I9" s="58" t="str">
-        <x:v>EP 暴露率</x:v>
+      <x:c r="I9" s="90" t="str">
+        <x:v>EP exposed
+comm fraction</x:v>
       </x:c>
       <x:c r="J9" s="98" t="n">
         <x:v>1</x:v>
@@ -7847,7 +7855,7 @@
       <x:c r="W10" s="58"/>
       <x:c r="X10" s="58"/>
     </x:row>
-    <x:row r="11" ht="18" customHeight="1">
+    <x:row r="11" ht="34" customHeight="1">
       <x:c r="A11" s="58" t="str">
         <x:v>Conv 额外 slots</x:v>
       </x:c>
@@ -7864,16 +7872,18 @@
       </x:c>
       <x:c r="G11" s="58"/>
       <x:c r="H11" s="58"/>
-      <x:c r="I11" s="58" t="str">
-        <x:v>TP 共享比例</x:v>
+      <x:c r="I11" s="90" t="str">
+        <x:v>TP shared
+resource fraction</x:v>
       </x:c>
       <x:c r="J11" s="104" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="K11" s="58"/>
       <x:c r="L11" s="58"/>
-      <x:c r="M11" s="58" t="str">
-        <x:v>TP 暴露率</x:v>
+      <x:c r="M11" s="90" t="str">
+        <x:v>TP exposed
+comm fraction</x:v>
       </x:c>
       <x:c r="N11" s="104" t="n">
         <x:v>1</x:v>
@@ -7891,7 +7901,7 @@
     </x:row>
     <x:row r="12" ht="18" customHeight="1">
       <x:c r="A12" s="58" t="str">
-        <x:v>TTFT 作为批次周期；EP 与 TP 带宽分别填写。TP 不与 KV 共用链路时，将 TP 共享比例设为 0。</x:v>
+        <x:v>P = Prefill，D = Decode。通常只需修改带宽、请求数和 TTFT/TPOT；附加假设可保持默认。</x:v>
       </x:c>
       <x:c r="B12" s="58"/>
       <x:c r="C12" s="58"/>
@@ -7918,7 +7928,9 @@
       <x:c r="X12" s="58"/>
     </x:row>
     <x:row r="13" ht="18" customHeight="1">
-      <x:c r="A13" s="58"/>
+      <x:c r="A13" s="58" t="str">
+        <x:v>Total overhead 表示基线 60 秒工作量的额外耗时；TTFT 在这里作为 KV 批次到达间隔。</x:v>
+      </x:c>
       <x:c r="B13" s="58"/>
       <x:c r="C13" s="58"/>
       <x:c r="D13" s="58"/>
@@ -7997,22 +8009,22 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G15" s="58"/>
-      <x:c r="H15" s="58" t="str">
-        <x:v>黄色为输入；模型 / EP 带宽可在下表逐项覆盖。</x:v>
-      </x:c>
-      <x:c r="I15" s="58"/>
-      <x:c r="J15" s="58"/>
-      <x:c r="K15" s="58"/>
-      <x:c r="L15" s="58"/>
-      <x:c r="M15" s="58"/>
-      <x:c r="N15" s="58"/>
-      <x:c r="O15" s="58"/>
-      <x:c r="P15" s="58"/>
-      <x:c r="Q15" s="58"/>
-      <x:c r="R15" s="58"/>
-      <x:c r="S15" s="58"/>
-      <x:c r="T15" s="58"/>
-      <x:c r="U15" s="58"/>
+      <x:c r="H15" s="118" t="str">
+        <x:v>Default: P = D = 1; KV bursts = 1; shared / exposed fractions = 100%.</x:v>
+      </x:c>
+      <x:c r="I15" s="118"/>
+      <x:c r="J15" s="118"/>
+      <x:c r="K15" s="118"/>
+      <x:c r="L15" s="118"/>
+      <x:c r="M15" s="118"/>
+      <x:c r="N15" s="118"/>
+      <x:c r="O15" s="118"/>
+      <x:c r="P15" s="118"/>
+      <x:c r="Q15" s="118"/>
+      <x:c r="R15" s="118"/>
+      <x:c r="S15" s="118"/>
+      <x:c r="T15" s="118"/>
+      <x:c r="U15" s="118"/>
       <x:c r="V15" s="58"/>
       <x:c r="W15" s="58"/>
       <x:c r="X15" s="58"/>
@@ -8035,22 +8047,22 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="G16" s="58"/>
-      <x:c r="H16" s="58" t="str">
-        <x:v>时间增量针对基线 60 秒工作量；不表示实测吞吐或 P99。</x:v>
-      </x:c>
-      <x:c r="I16" s="58"/>
-      <x:c r="J16" s="58"/>
-      <x:c r="K16" s="58"/>
-      <x:c r="L16" s="58"/>
-      <x:c r="M16" s="58"/>
-      <x:c r="N16" s="58"/>
-      <x:c r="O16" s="58"/>
-      <x:c r="P16" s="58"/>
-      <x:c r="Q16" s="58"/>
-      <x:c r="R16" s="58"/>
-      <x:c r="S16" s="58"/>
-      <x:c r="T16" s="58"/>
-      <x:c r="U16" s="58"/>
+      <x:c r="H16" s="118" t="str">
+        <x:v>Deployment count：完整 EP 部署的套数；EP32 每套 32 卡，EP256 每套 256 卡。</x:v>
+      </x:c>
+      <x:c r="I16" s="118"/>
+      <x:c r="J16" s="118"/>
+      <x:c r="K16" s="118"/>
+      <x:c r="L16" s="118"/>
+      <x:c r="M16" s="118"/>
+      <x:c r="N16" s="118"/>
+      <x:c r="O16" s="118"/>
+      <x:c r="P16" s="118"/>
+      <x:c r="Q16" s="118"/>
+      <x:c r="R16" s="118"/>
+      <x:c r="S16" s="118"/>
+      <x:c r="T16" s="118"/>
+      <x:c r="U16" s="118"/>
       <x:c r="V16" s="58"/>
       <x:c r="W16" s="58"/>
       <x:c r="X16" s="58"/>
@@ -8073,22 +8085,22 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="G17" s="58"/>
-      <x:c r="H17" s="58" t="str">
-        <x:v>TTFT 只用于到达节奏，本页计算 D 侧 TPOT；P 耗时仍见原表。</x:v>
-      </x:c>
-      <x:c r="I17" s="58"/>
-      <x:c r="J17" s="58"/>
-      <x:c r="K17" s="58"/>
-      <x:c r="L17" s="58"/>
-      <x:c r="M17" s="58"/>
-      <x:c r="N17" s="58"/>
-      <x:c r="O17" s="58"/>
-      <x:c r="P17" s="58"/>
-      <x:c r="Q17" s="58"/>
-      <x:c r="R17" s="58"/>
-      <x:c r="S17" s="58"/>
-      <x:c r="T17" s="58"/>
-      <x:c r="U17" s="58"/>
+      <x:c r="H17" s="118" t="str">
+        <x:v>Shared resource fraction：通信中与 KV 竞争同一资源的比例。100% = 全部；0% = 资源独立。</x:v>
+      </x:c>
+      <x:c r="I17" s="118"/>
+      <x:c r="J17" s="118"/>
+      <x:c r="K17" s="118"/>
+      <x:c r="L17" s="118"/>
+      <x:c r="M17" s="118"/>
+      <x:c r="N17" s="118"/>
+      <x:c r="O17" s="118"/>
+      <x:c r="P17" s="118"/>
+      <x:c r="Q17" s="118"/>
+      <x:c r="R17" s="118"/>
+      <x:c r="S17" s="118"/>
+      <x:c r="T17" s="118"/>
+      <x:c r="U17" s="118"/>
       <x:c r="V17" s="58"/>
       <x:c r="W17" s="58"/>
       <x:c r="X17" s="58"/>
@@ -8105,22 +8117,22 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="G18" s="58"/>
-      <x:c r="H18" s="58" t="str">
-        <x:v>全通信＝该步所有等效 EP＋TP 段都在 KV 窗口内；TP 首尾通信均摊到层段。</x:v>
-      </x:c>
-      <x:c r="I18" s="58"/>
-      <x:c r="J18" s="58"/>
-      <x:c r="K18" s="58"/>
-      <x:c r="L18" s="58"/>
-      <x:c r="M18" s="58"/>
-      <x:c r="N18" s="58"/>
-      <x:c r="O18" s="58"/>
-      <x:c r="P18" s="58"/>
-      <x:c r="Q18" s="58"/>
-      <x:c r="R18" s="58"/>
-      <x:c r="S18" s="58"/>
-      <x:c r="T18" s="58"/>
-      <x:c r="U18" s="58"/>
+      <x:c r="H18" s="118" t="str">
+        <x:v>Exposed communication fraction：通信增时最终计入 forward 的比例；被计算遮住的部分不计入。</x:v>
+      </x:c>
+      <x:c r="I18" s="118"/>
+      <x:c r="J18" s="118"/>
+      <x:c r="K18" s="118"/>
+      <x:c r="L18" s="118"/>
+      <x:c r="M18" s="118"/>
+      <x:c r="N18" s="118"/>
+      <x:c r="O18" s="118"/>
+      <x:c r="P18" s="118"/>
+      <x:c r="Q18" s="118"/>
+      <x:c r="R18" s="118"/>
+      <x:c r="S18" s="118"/>
+      <x:c r="T18" s="118"/>
+      <x:c r="U18" s="118"/>
       <x:c r="V18" s="58"/>
       <x:c r="W18" s="58"/>
       <x:c r="X18" s="58"/>
@@ -8133,20 +8145,22 @@
       <x:c r="E19" s="58"/>
       <x:c r="F19" s="58"/>
       <x:c r="G19" s="58"/>
-      <x:c r="H19" s="58"/>
-      <x:c r="I19" s="58"/>
-      <x:c r="J19" s="58"/>
-      <x:c r="K19" s="58"/>
-      <x:c r="L19" s="58"/>
-      <x:c r="M19" s="58"/>
-      <x:c r="N19" s="58"/>
-      <x:c r="O19" s="58"/>
-      <x:c r="P19" s="58"/>
-      <x:c r="Q19" s="58"/>
-      <x:c r="R19" s="58"/>
-      <x:c r="S19" s="58"/>
-      <x:c r="T19" s="58"/>
-      <x:c r="U19" s="58"/>
+      <x:c r="H19" s="118" t="str">
+        <x:v>KV bursts per interval：一批 KV 均分成 m 次、等间隔发送；m = 2 时每次一半，总量不变。</x:v>
+      </x:c>
+      <x:c r="I19" s="118"/>
+      <x:c r="J19" s="118"/>
+      <x:c r="K19" s="118"/>
+      <x:c r="L19" s="118"/>
+      <x:c r="M19" s="118"/>
+      <x:c r="N19" s="118"/>
+      <x:c r="O19" s="118"/>
+      <x:c r="P19" s="118"/>
+      <x:c r="Q19" s="118"/>
+      <x:c r="R19" s="118"/>
+      <x:c r="S19" s="118"/>
+      <x:c r="T19" s="118"/>
+      <x:c r="U19" s="118"/>
       <x:c r="V19" s="58"/>
       <x:c r="W19" s="58"/>
       <x:c r="X19" s="58"/>
@@ -8159,20 +8173,22 @@
       <x:c r="E20" s="58"/>
       <x:c r="F20" s="58"/>
       <x:c r="G20" s="58"/>
-      <x:c r="H20" s="58"/>
-      <x:c r="I20" s="58"/>
-      <x:c r="J20" s="58"/>
-      <x:c r="K20" s="58"/>
-      <x:c r="L20" s="58"/>
-      <x:c r="M20" s="58"/>
-      <x:c r="N20" s="58"/>
-      <x:c r="O20" s="58"/>
-      <x:c r="P20" s="58"/>
-      <x:c r="Q20" s="58"/>
-      <x:c r="R20" s="58"/>
-      <x:c r="S20" s="58"/>
-      <x:c r="T20" s="58"/>
-      <x:c r="U20" s="58"/>
+      <x:c r="H20" s="118" t="str">
+        <x:v>Temporal overlap 由 KV 窗口自动计算；没有 profiling 时，不必另猜 shared / exposed 两个比例。</x:v>
+      </x:c>
+      <x:c r="I20" s="118"/>
+      <x:c r="J20" s="118"/>
+      <x:c r="K20" s="118"/>
+      <x:c r="L20" s="118"/>
+      <x:c r="M20" s="118"/>
+      <x:c r="N20" s="118"/>
+      <x:c r="O20" s="118"/>
+      <x:c r="P20" s="118"/>
+      <x:c r="Q20" s="118"/>
+      <x:c r="R20" s="118"/>
+      <x:c r="S20" s="118"/>
+      <x:c r="T20" s="118"/>
+      <x:c r="U20" s="118"/>
       <x:c r="V20" s="58"/>
       <x:c r="W20" s="58"/>
       <x:c r="X20" s="58"/>
@@ -8241,10 +8257,12 @@
         <x:v>产出 tokens/步</x:v>
       </x:c>
       <x:c r="M22" s="70" t="str">
-        <x:v>共享比例</x:v>
+        <x:v>EP shared
+resource fraction</x:v>
       </x:c>
       <x:c r="N22" s="70" t="str">
-        <x:v>暴露率</x:v>
+        <x:v>EP exposed
+comm fraction</x:v>
       </x:c>
       <x:c r="O22" s="70" t="str">
         <x:v>配置条件</x:v>
@@ -8252,11 +8270,13 @@
       <x:c r="P22" s="109" t="str">
         <x:v>TP GB/s 输入</x:v>
       </x:c>
-      <x:c r="Q22" s="109" t="str">
-        <x:v>TP 共享比例</x:v>
-      </x:c>
-      <x:c r="R22" s="109" t="str">
-        <x:v>TP 暴露率</x:v>
+      <x:c r="Q22" s="70" t="str">
+        <x:v>TP shared
+resource fraction</x:v>
+      </x:c>
+      <x:c r="R22" s="70" t="str">
+        <x:v>TP exposed
+comm fraction</x:v>
       </x:c>
       <x:c r="S22" s="109" t="str">
         <x:v>Attention 层数</x:v>
@@ -9320,7 +9340,8 @@
         <x:v>重叠层段 次/min</x:v>
       </x:c>
       <x:c r="L39" s="70" t="str">
-        <x:v>60s 工作增时 ms</x:v>
+        <x:v>Total overhead
+ms/60s</x:v>
       </x:c>
       <x:c r="M39" s="70" t="str">
         <x:v>平均 TPOT 增量 μs</x:v>
@@ -9340,11 +9361,13 @@
       <x:c r="R39" s="109" t="str">
         <x:v>TP 带宽项 ms</x:v>
       </x:c>
-      <x:c r="S39" s="109" t="str">
-        <x:v>EP 增时 ms/60s</x:v>
-      </x:c>
-      <x:c r="T39" s="109" t="str">
-        <x:v>TP 增时 ms/60s</x:v>
+      <x:c r="S39" s="70" t="str">
+        <x:v>EP overhead
+ms/60s</x:v>
+      </x:c>
+      <x:c r="T39" s="70" t="str">
+        <x:v>TP overhead
+ms/60s</x:v>
       </x:c>
       <x:c r="U39" s="58"/>
       <x:c r="V39" s="58"/>
@@ -21790,7 +21813,8 @@
         <x:v>基线 FW/min</x:v>
       </x:c>
       <x:c r="V189" s="70" t="str">
-        <x:v>60s 工作增时 ms</x:v>
+        <x:v>Total overhead
+ms/60s</x:v>
       </x:c>
       <x:c r="W189" s="70" t="str">
         <x:v>输入 / 调度状态</x:v>

</xml_diff>

<commit_message>
Add decode throughput loss percentages to PD minute scenarios
</commit_message>
<xml_diff>
--- a/examples/kv-ep-sweep/kv-ep32-ep256.xlsx
+++ b/examples/kv-ep-sweep/kv-ep32-ep256.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规格汇总" sheetId="1" r:id="Rb60a63b8d3854e8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KV明细" sheetId="2" r:id="Rf8e0d8f6b8eb4b78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EP通信" sheetId="3" r:id="R38883d9a1a5f40bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分钟场景" sheetId="4" r:id="R395764b5e5a6414c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规格汇总" sheetId="1" r:id="R0447516498bc4879"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KV明细" sheetId="2" r:id="R7e3bbdeddf8a45e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EP通信" sheetId="3" r:id="R8044e445d1cc4947"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分钟场景" sheetId="4" r:id="Rbb66981a8a264253"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,7 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="11">
+  <x:numFmts count="12">
     <x:numFmt numFmtId="200" formatCode="#,##0"/>
     <x:numFmt numFmtId="201" formatCode="#,##0.000"/>
     <x:numFmt numFmtId="202" formatCode="#,##0.000000"/>
@@ -28,6 +28,7 @@
     <x:numFmt numFmtId="208" formatCode="0.0%"/>
     <x:numFmt numFmtId="209" formatCode="0.000000"/>
     <x:numFmt numFmtId="210" formatCode="0.000000%"/>
+    <x:numFmt numFmtId="211" formatCode="[=0]0.000000%;[&lt;0.00000001]&quot;&lt;0.000001%&quot;;0.000000%"/>
   </x:numFmts>
   <x:fonts count="13">
     <x:font>
@@ -103,7 +104,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="15">
+  <x:fills count="16">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -175,6 +176,11 @@
         <x:fgColor rgb="FFD9E1F2"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9E1F2"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="3">
     <x:border/>
@@ -210,7 +216,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="119">
+  <x:cellXfs count="125">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -552,6 +558,24 @@
     <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -7518,7 +7542,7 @@
     <x:col min="18" max="18" width="19" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="19" hidden="0" customWidth="1"/>
     <x:col min="20" max="20" width="19" hidden="0" customWidth="1"/>
-    <x:col min="21" max="21" width="19" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="21" hidden="0" customWidth="1"/>
     <x:col min="22" max="22" width="19" hidden="0" customWidth="1"/>
     <x:col min="23" max="23" width="19" hidden="0" customWidth="1"/>
     <x:col min="24" max="24" width="19" hidden="0" customWidth="1"/>
@@ -9369,7 +9393,10 @@
         <x:v>TP overhead
 ms/60s</x:v>
       </x:c>
-      <x:c r="U39" s="58"/>
+      <x:c r="U39" s="123" t="str">
+        <x:v>Decode throughput
+loss (%)</x:v>
+      </x:c>
       <x:c r="V39" s="58"/>
       <x:c r="W39" s="58"/>
       <x:c r="X39" s="58"/>
@@ -9454,7 +9481,10 @@
         <x:f>IF(W190="",AJ190,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U40" s="58"/>
+      <x:c r="U40" s="124" t="n">
+        <x:f>IF(ISNUMBER(L40),L40/(60000+L40),IF(L40="","",L40))</x:f>
+        <x:v>1.213936102836291e-7</x:v>
+      </x:c>
       <x:c r="V40" s="58"/>
       <x:c r="W40" s="58"/>
       <x:c r="X40" s="58"/>
@@ -9539,7 +9569,10 @@
         <x:f>IF(W191="",AJ191,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U41" s="58"/>
+      <x:c r="U41" s="124" t="n">
+        <x:f>IF(ISNUMBER(L41),L41/(60000+L41),IF(L41="","",L41))</x:f>
+        <x:v>6.069680882591694e-8</x:v>
+      </x:c>
       <x:c r="V41" s="58"/>
       <x:c r="W41" s="58"/>
       <x:c r="X41" s="58"/>
@@ -9624,7 +9657,10 @@
         <x:f>IF(W192="",AJ192,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U42" s="58"/>
+      <x:c r="U42" s="124" t="n">
+        <x:f>IF(ISNUMBER(L42),L42/(60000+L42),IF(L42="","",L42))</x:f>
+        <x:v>3.0348405333984146e-8</x:v>
+      </x:c>
       <x:c r="V42" s="58"/>
       <x:c r="W42" s="58"/>
       <x:c r="X42" s="58"/>
@@ -9709,7 +9745,10 @@
         <x:f>IF(W193="",AJ193,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U43" s="58"/>
+      <x:c r="U43" s="124" t="n">
+        <x:f>IF(ISNUMBER(L43),L43/(60000+L43),IF(L43="","",L43))</x:f>
+        <x:v>2.0232270427328478e-8</x:v>
+      </x:c>
       <x:c r="V43" s="58"/>
       <x:c r="W43" s="58"/>
       <x:c r="X43" s="58"/>
@@ -9794,7 +9833,10 @@
         <x:f>IF(W194="",AJ194,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U44" s="58"/>
+      <x:c r="U44" s="124" t="n">
+        <x:f>IF(ISNUMBER(L44),L44/(60000+L44),IF(L44="","",L44))</x:f>
+        <x:v>3.091538839342367e-7</x:v>
+      </x:c>
       <x:c r="V44" s="58"/>
       <x:c r="W44" s="58"/>
       <x:c r="X44" s="58"/>
@@ -9879,7 +9921,10 @@
         <x:f>IF(W195="",AJ195,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U45" s="58"/>
+      <x:c r="U45" s="124" t="n">
+        <x:f>IF(ISNUMBER(L45),L45/(60000+L45),IF(L45="","",L45))</x:f>
+        <x:v>1.5457696586115304e-7</x:v>
+      </x:c>
       <x:c r="V45" s="58"/>
       <x:c r="W45" s="58"/>
       <x:c r="X45" s="58"/>
@@ -9964,7 +10009,10 @@
         <x:f>IF(W196="",AJ196,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U46" s="58"/>
+      <x:c r="U46" s="124" t="n">
+        <x:f>IF(ISNUMBER(L46),L46/(60000+L46),IF(L46="","",L46))</x:f>
+        <x:v>7.728848890408657e-8</x:v>
+      </x:c>
       <x:c r="V46" s="58"/>
       <x:c r="W46" s="58"/>
       <x:c r="X46" s="58"/>
@@ -10049,7 +10097,10 @@
         <x:f>IF(W197="",AJ197,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U47" s="58"/>
+      <x:c r="U47" s="124" t="n">
+        <x:f>IF(ISNUMBER(L47),L47/(60000+L47),IF(L47="","",L47))</x:f>
+        <x:v>5.1525660596837856e-8</x:v>
+      </x:c>
       <x:c r="V47" s="58"/>
       <x:c r="W47" s="58"/>
       <x:c r="X47" s="58"/>
@@ -10134,7 +10185,10 @@
         <x:f>IF(W198="",AJ198,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U48" s="58"/>
+      <x:c r="U48" s="124" t="n">
+        <x:f>IF(ISNUMBER(L48),L48/(60000+L48),IF(L48="","",L48))</x:f>
+        <x:v>4.0691809906119785e-7</x:v>
+      </x:c>
       <x:c r="V48" s="58"/>
       <x:c r="W48" s="58"/>
       <x:c r="X48" s="58"/>
@@ -10219,7 +10273,10 @@
         <x:f>IF(W199="",AJ199,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U49" s="58"/>
+      <x:c r="U49" s="124" t="n">
+        <x:f>IF(ISNUMBER(L49),L49/(60000+L49),IF(L49="","",L49))</x:f>
+        <x:v>2.0345909092619215e-7</x:v>
+      </x:c>
       <x:c r="V49" s="58"/>
       <x:c r="W49" s="58"/>
       <x:c r="X49" s="58"/>
@@ -10304,7 +10361,10 @@
         <x:f>IF(W200="",AJ200,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U50" s="58"/>
+      <x:c r="U50" s="124" t="n">
+        <x:f>IF(ISNUMBER(L50),L50/(60000+L50),IF(L50="","",L50))</x:f>
+        <x:v>1.0172955581199755e-7</x:v>
+      </x:c>
       <x:c r="V50" s="58"/>
       <x:c r="W50" s="58"/>
       <x:c r="X50" s="58"/>
@@ -10389,7 +10449,10 @@
         <x:f>IF(W201="",AJ201,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U51" s="58"/>
+      <x:c r="U51" s="124" t="n">
+        <x:f>IF(ISNUMBER(L51),L51/(60000+L51),IF(L51="","",L51))</x:f>
+        <x:v>6.781970617442124e-8</x:v>
+      </x:c>
       <x:c r="V51" s="58"/>
       <x:c r="W51" s="58"/>
       <x:c r="X51" s="58"/>
@@ -10474,7 +10537,10 @@
         <x:f>IF(W202="",AJ202,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U52" s="58"/>
+      <x:c r="U52" s="124" t="n">
+        <x:f>IF(ISNUMBER(L52),L52/(60000+L52),IF(L52="","",L52))</x:f>
+        <x:v>1.2483073166253527e-7</x:v>
+      </x:c>
       <x:c r="V52" s="58"/>
       <x:c r="W52" s="58"/>
       <x:c r="X52" s="58"/>
@@ -10559,7 +10625,10 @@
         <x:f>IF(W203="",AJ203,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U53" s="58"/>
+      <x:c r="U53" s="124" t="n">
+        <x:f>IF(ISNUMBER(L53),L53/(60000+L53),IF(L53="","",L53))</x:f>
+        <x:v>6.241536972694577e-8</x:v>
+      </x:c>
       <x:c r="V53" s="58"/>
       <x:c r="W53" s="58"/>
       <x:c r="X53" s="58"/>
@@ -10644,7 +10713,10 @@
         <x:f>IF(W204="",AJ204,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U54" s="58"/>
+      <x:c r="U54" s="124" t="n">
+        <x:f>IF(ISNUMBER(L54),L54/(60000+L54),IF(L54="","",L54))</x:f>
+        <x:v>3.1207685837392514e-8</x:v>
+      </x:c>
       <x:c r="V54" s="58"/>
       <x:c r="W54" s="58"/>
       <x:c r="X54" s="58"/>
@@ -10729,7 +10801,10 @@
         <x:f>IF(W205="",AJ205,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U55" s="58"/>
+      <x:c r="U55" s="124" t="n">
+        <x:f>IF(ISNUMBER(L55),L55/(60000+L55),IF(L55="","",L55))</x:f>
+        <x:v>2.08051241080216e-8</x:v>
+      </x:c>
       <x:c r="V55" s="58"/>
       <x:c r="W55" s="58"/>
       <x:c r="X55" s="58"/>
@@ -10814,7 +10889,10 @@
         <x:f>IF(W206="",AJ206,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U56" s="58"/>
+      <x:c r="U56" s="124" t="n">
+        <x:f>IF(ISNUMBER(L56),L56/(60000+L56),IF(L56="","",L56))</x:f>
+        <x:v>3.179346588298593e-7</x:v>
+      </x:c>
       <x:c r="V56" s="58"/>
       <x:c r="W56" s="58"/>
       <x:c r="X56" s="58"/>
@@ -10899,7 +10977,10 @@
         <x:f>IF(W207="",AJ207,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U57" s="58"/>
+      <x:c r="U57" s="124" t="n">
+        <x:f>IF(ISNUMBER(L57),L57/(60000+L57),IF(L57="","",L57))</x:f>
+        <x:v>1.589673546855455e-7</x:v>
+      </x:c>
       <x:c r="V57" s="58"/>
       <x:c r="W57" s="58"/>
       <x:c r="X57" s="58"/>
@@ -10984,7 +11065,10 @@
         <x:f>IF(W208="",AJ208,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U58" s="58"/>
+      <x:c r="U58" s="124" t="n">
+        <x:f>IF(ISNUMBER(L58),L58/(60000+L58),IF(L58="","",L58))</x:f>
+        <x:v>7.948368366042821e-8</x:v>
+      </x:c>
       <x:c r="V58" s="58"/>
       <x:c r="W58" s="58"/>
       <x:c r="X58" s="58"/>
@@ -11069,7 +11153,10 @@
         <x:f>IF(W209="",AJ209,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U59" s="58"/>
+      <x:c r="U59" s="124" t="n">
+        <x:f>IF(ISNUMBER(L59),L59/(60000+L59),IF(L59="","",L59))</x:f>
+        <x:v>5.2989123844209054e-8</x:v>
+      </x:c>
       <x:c r="V59" s="58"/>
       <x:c r="W59" s="58"/>
       <x:c r="X59" s="58"/>
@@ -11154,7 +11241,10 @@
         <x:f>IF(W210="",AJ210,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U60" s="58"/>
+      <x:c r="U60" s="124" t="n">
+        <x:f>IF(ISNUMBER(L60),L60/(60000+L60),IF(L60="","",L60))</x:f>
+        <x:v>4.1847792934110385e-7</x:v>
+      </x:c>
       <x:c r="V60" s="58"/>
       <x:c r="W60" s="58"/>
       <x:c r="X60" s="58"/>
@@ -11239,7 +11329,10 @@
         <x:f>IF(W211="",AJ211,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U61" s="58"/>
+      <x:c r="U61" s="124" t="n">
+        <x:f>IF(ISNUMBER(L61),L61/(60000+L61),IF(L61="","",L61))</x:f>
+        <x:v>2.0923900845150542e-7</x:v>
+      </x:c>
       <x:c r="V61" s="58"/>
       <x:c r="W61" s="58"/>
       <x:c r="X61" s="58"/>
@@ -11324,7 +11417,10 @@
         <x:f>IF(W212="",AJ212,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U62" s="58"/>
+      <x:c r="U62" s="124" t="n">
+        <x:f>IF(ISNUMBER(L62),L62/(60000+L62),IF(L62="","",L62))</x:f>
+        <x:v>1.0461951517099452e-7</x:v>
+      </x:c>
       <x:c r="V62" s="58"/>
       <x:c r="W62" s="58"/>
       <x:c r="X62" s="58"/>
@@ -11409,7 +11505,10 @@
         <x:f>IF(W213="",AJ213,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U63" s="58"/>
+      <x:c r="U63" s="124" t="n">
+        <x:f>IF(ISNUMBER(L63),L63/(60000+L63),IF(L63="","",L63))</x:f>
+        <x:v>6.974634587960599e-8</x:v>
+      </x:c>
       <x:c r="V63" s="58"/>
       <x:c r="W63" s="58"/>
       <x:c r="X63" s="58"/>
@@ -11494,7 +11593,10 @@
         <x:f>IF(W214="",AJ214,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U64" s="58"/>
+      <x:c r="U64" s="124" t="n">
+        <x:f>IF(ISNUMBER(L64),L64/(60000+L64),IF(L64="","",L64))</x:f>
+        <x:v>1.213936102836291e-7</x:v>
+      </x:c>
       <x:c r="V64" s="58"/>
       <x:c r="W64" s="58"/>
       <x:c r="X64" s="58"/>
@@ -11579,7 +11681,10 @@
         <x:f>IF(W215="",AJ215,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U65" s="58"/>
+      <x:c r="U65" s="124" t="n">
+        <x:f>IF(ISNUMBER(L65),L65/(60000+L65),IF(L65="","",L65))</x:f>
+        <x:v>6.069680882591694e-8</x:v>
+      </x:c>
       <x:c r="V65" s="58"/>
       <x:c r="W65" s="58"/>
       <x:c r="X65" s="58"/>
@@ -11664,7 +11769,10 @@
         <x:f>IF(W216="",AJ216,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U66" s="58"/>
+      <x:c r="U66" s="124" t="n">
+        <x:f>IF(ISNUMBER(L66),L66/(60000+L66),IF(L66="","",L66))</x:f>
+        <x:v>3.0348405333984146e-8</x:v>
+      </x:c>
       <x:c r="V66" s="58"/>
       <x:c r="W66" s="58"/>
       <x:c r="X66" s="58"/>
@@ -11749,7 +11857,10 @@
         <x:f>IF(W217="",AJ217,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U67" s="58"/>
+      <x:c r="U67" s="124" t="n">
+        <x:f>IF(ISNUMBER(L67),L67/(60000+L67),IF(L67="","",L67))</x:f>
+        <x:v>2.0232270427328478e-8</x:v>
+      </x:c>
       <x:c r="V67" s="58"/>
       <x:c r="W67" s="58"/>
       <x:c r="X67" s="58"/>
@@ -11834,7 +11945,10 @@
         <x:f>IF(W218="",AJ218,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U68" s="58"/>
+      <x:c r="U68" s="124" t="n">
+        <x:f>IF(ISNUMBER(L68),L68/(60000+L68),IF(L68="","",L68))</x:f>
+        <x:v>3.091538839342367e-7</x:v>
+      </x:c>
       <x:c r="V68" s="58"/>
       <x:c r="W68" s="58"/>
       <x:c r="X68" s="58"/>
@@ -11919,7 +12033,10 @@
         <x:f>IF(W219="",AJ219,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U69" s="58"/>
+      <x:c r="U69" s="124" t="n">
+        <x:f>IF(ISNUMBER(L69),L69/(60000+L69),IF(L69="","",L69))</x:f>
+        <x:v>1.5457696586115304e-7</x:v>
+      </x:c>
       <x:c r="V69" s="58"/>
       <x:c r="W69" s="58"/>
       <x:c r="X69" s="58"/>
@@ -12004,7 +12121,10 @@
         <x:f>IF(W220="",AJ220,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U70" s="58"/>
+      <x:c r="U70" s="124" t="n">
+        <x:f>IF(ISNUMBER(L70),L70/(60000+L70),IF(L70="","",L70))</x:f>
+        <x:v>7.728848890408657e-8</x:v>
+      </x:c>
       <x:c r="V70" s="58"/>
       <x:c r="W70" s="58"/>
       <x:c r="X70" s="58"/>
@@ -12089,7 +12209,10 @@
         <x:f>IF(W221="",AJ221,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U71" s="58"/>
+      <x:c r="U71" s="124" t="n">
+        <x:f>IF(ISNUMBER(L71),L71/(60000+L71),IF(L71="","",L71))</x:f>
+        <x:v>5.1525660596837856e-8</x:v>
+      </x:c>
       <x:c r="V71" s="58"/>
       <x:c r="W71" s="58"/>
       <x:c r="X71" s="58"/>
@@ -12174,7 +12297,10 @@
         <x:f>IF(W222="",AJ222,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U72" s="58"/>
+      <x:c r="U72" s="124" t="n">
+        <x:f>IF(ISNUMBER(L72),L72/(60000+L72),IF(L72="","",L72))</x:f>
+        <x:v>4.0691809906119785e-7</x:v>
+      </x:c>
       <x:c r="V72" s="58"/>
       <x:c r="W72" s="58"/>
       <x:c r="X72" s="58"/>
@@ -12259,7 +12385,10 @@
         <x:f>IF(W223="",AJ223,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U73" s="58"/>
+      <x:c r="U73" s="124" t="n">
+        <x:f>IF(ISNUMBER(L73),L73/(60000+L73),IF(L73="","",L73))</x:f>
+        <x:v>2.0345909092619215e-7</x:v>
+      </x:c>
       <x:c r="V73" s="58"/>
       <x:c r="W73" s="58"/>
       <x:c r="X73" s="58"/>
@@ -12344,7 +12473,10 @@
         <x:f>IF(W224="",AJ224,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U74" s="58"/>
+      <x:c r="U74" s="124" t="n">
+        <x:f>IF(ISNUMBER(L74),L74/(60000+L74),IF(L74="","",L74))</x:f>
+        <x:v>1.0172955581199755e-7</x:v>
+      </x:c>
       <x:c r="V74" s="58"/>
       <x:c r="W74" s="58"/>
       <x:c r="X74" s="58"/>
@@ -12429,7 +12561,10 @@
         <x:f>IF(W225="",AJ225,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U75" s="58"/>
+      <x:c r="U75" s="124" t="n">
+        <x:f>IF(ISNUMBER(L75),L75/(60000+L75),IF(L75="","",L75))</x:f>
+        <x:v>6.781970617442124e-8</x:v>
+      </x:c>
       <x:c r="V75" s="58"/>
       <x:c r="W75" s="58"/>
       <x:c r="X75" s="58"/>
@@ -12514,7 +12649,10 @@
         <x:f>IF(W226="",AJ226,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U76" s="58"/>
+      <x:c r="U76" s="124" t="n">
+        <x:f>IF(ISNUMBER(L76),L76/(60000+L76),IF(L76="","",L76))</x:f>
+        <x:v>1.2483073166253527e-7</x:v>
+      </x:c>
       <x:c r="V76" s="58"/>
       <x:c r="W76" s="58"/>
       <x:c r="X76" s="58"/>
@@ -12599,7 +12737,10 @@
         <x:f>IF(W227="",AJ227,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U77" s="58"/>
+      <x:c r="U77" s="124" t="n">
+        <x:f>IF(ISNUMBER(L77),L77/(60000+L77),IF(L77="","",L77))</x:f>
+        <x:v>6.241536972694577e-8</x:v>
+      </x:c>
       <x:c r="V77" s="58"/>
       <x:c r="W77" s="58"/>
       <x:c r="X77" s="58"/>
@@ -12684,7 +12825,10 @@
         <x:f>IF(W228="",AJ228,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U78" s="58"/>
+      <x:c r="U78" s="124" t="n">
+        <x:f>IF(ISNUMBER(L78),L78/(60000+L78),IF(L78="","",L78))</x:f>
+        <x:v>3.1207685837392514e-8</x:v>
+      </x:c>
       <x:c r="V78" s="58"/>
       <x:c r="W78" s="58"/>
       <x:c r="X78" s="58"/>
@@ -12769,7 +12913,10 @@
         <x:f>IF(W229="",AJ229,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U79" s="58"/>
+      <x:c r="U79" s="124" t="n">
+        <x:f>IF(ISNUMBER(L79),L79/(60000+L79),IF(L79="","",L79))</x:f>
+        <x:v>2.08051241080216e-8</x:v>
+      </x:c>
       <x:c r="V79" s="58"/>
       <x:c r="W79" s="58"/>
       <x:c r="X79" s="58"/>
@@ -12854,7 +13001,10 @@
         <x:f>IF(W230="",AJ230,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U80" s="58"/>
+      <x:c r="U80" s="124" t="n">
+        <x:f>IF(ISNUMBER(L80),L80/(60000+L80),IF(L80="","",L80))</x:f>
+        <x:v>3.179346588298593e-7</x:v>
+      </x:c>
       <x:c r="V80" s="58"/>
       <x:c r="W80" s="58"/>
       <x:c r="X80" s="58"/>
@@ -12939,7 +13089,10 @@
         <x:f>IF(W231="",AJ231,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U81" s="58"/>
+      <x:c r="U81" s="124" t="n">
+        <x:f>IF(ISNUMBER(L81),L81/(60000+L81),IF(L81="","",L81))</x:f>
+        <x:v>1.589673546855455e-7</x:v>
+      </x:c>
       <x:c r="V81" s="58"/>
       <x:c r="W81" s="58"/>
       <x:c r="X81" s="58"/>
@@ -13024,7 +13177,10 @@
         <x:f>IF(W232="",AJ232,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U82" s="58"/>
+      <x:c r="U82" s="124" t="n">
+        <x:f>IF(ISNUMBER(L82),L82/(60000+L82),IF(L82="","",L82))</x:f>
+        <x:v>7.948368366042821e-8</x:v>
+      </x:c>
       <x:c r="V82" s="58"/>
       <x:c r="W82" s="58"/>
       <x:c r="X82" s="58"/>
@@ -13109,7 +13265,10 @@
         <x:f>IF(W233="",AJ233,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U83" s="58"/>
+      <x:c r="U83" s="124" t="n">
+        <x:f>IF(ISNUMBER(L83),L83/(60000+L83),IF(L83="","",L83))</x:f>
+        <x:v>5.2989123844209054e-8</x:v>
+      </x:c>
       <x:c r="V83" s="58"/>
       <x:c r="W83" s="58"/>
       <x:c r="X83" s="58"/>
@@ -13194,7 +13353,10 @@
         <x:f>IF(W234="",AJ234,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U84" s="58"/>
+      <x:c r="U84" s="124" t="n">
+        <x:f>IF(ISNUMBER(L84),L84/(60000+L84),IF(L84="","",L84))</x:f>
+        <x:v>4.1847792934110385e-7</x:v>
+      </x:c>
       <x:c r="V84" s="58"/>
       <x:c r="W84" s="58"/>
       <x:c r="X84" s="58"/>
@@ -13279,7 +13441,10 @@
         <x:f>IF(W235="",AJ235,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U85" s="58"/>
+      <x:c r="U85" s="124" t="n">
+        <x:f>IF(ISNUMBER(L85),L85/(60000+L85),IF(L85="","",L85))</x:f>
+        <x:v>2.0923900845150542e-7</x:v>
+      </x:c>
       <x:c r="V85" s="58"/>
       <x:c r="W85" s="58"/>
       <x:c r="X85" s="58"/>
@@ -13364,7 +13529,10 @@
         <x:f>IF(W236="",AJ236,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U86" s="58"/>
+      <x:c r="U86" s="124" t="n">
+        <x:f>IF(ISNUMBER(L86),L86/(60000+L86),IF(L86="","",L86))</x:f>
+        <x:v>1.0461951517099452e-7</x:v>
+      </x:c>
       <x:c r="V86" s="58"/>
       <x:c r="W86" s="58"/>
       <x:c r="X86" s="58"/>
@@ -13449,7 +13617,10 @@
         <x:f>IF(W237="",AJ237,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U87" s="58"/>
+      <x:c r="U87" s="124" t="n">
+        <x:f>IF(ISNUMBER(L87),L87/(60000+L87),IF(L87="","",L87))</x:f>
+        <x:v>6.974634587960599e-8</x:v>
+      </x:c>
       <x:c r="V87" s="58"/>
       <x:c r="W87" s="58"/>
       <x:c r="X87" s="58"/>
@@ -13534,7 +13705,10 @@
         <x:f>IF(W238="",AJ238,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U88" s="58"/>
+      <x:c r="U88" s="124" t="n">
+        <x:f>IF(ISNUMBER(L88),L88/(60000+L88),IF(L88="","",L88))</x:f>
+        <x:v>0.0000014347343374794483</x:v>
+      </x:c>
       <x:c r="V88" s="58"/>
       <x:c r="W88" s="58"/>
       <x:c r="X88" s="58"/>
@@ -13619,7 +13793,10 @@
         <x:f>IF(W239="",AJ239,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U89" s="58"/>
+      <x:c r="U89" s="124" t="n">
+        <x:f>IF(ISNUMBER(L89),L89/(60000+L89),IF(L89="","",L89))</x:f>
+        <x:v>7.173676833557481e-7</x:v>
+      </x:c>
       <x:c r="V89" s="58"/>
       <x:c r="W89" s="58"/>
       <x:c r="X89" s="58"/>
@@ -13704,7 +13881,10 @@
         <x:f>IF(W240="",AJ240,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U90" s="58"/>
+      <x:c r="U90" s="124" t="n">
+        <x:f>IF(ISNUMBER(L90),L90/(60000+L90),IF(L90="","",L90))</x:f>
+        <x:v>3.586839703320185e-7</x:v>
+      </x:c>
       <x:c r="V90" s="58"/>
       <x:c r="W90" s="58"/>
       <x:c r="X90" s="58"/>
@@ -13789,7 +13969,10 @@
         <x:f>IF(W241="",AJ241,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U91" s="58"/>
+      <x:c r="U91" s="124" t="n">
+        <x:f>IF(ISNUMBER(L91),L91/(60000+L91),IF(L91="","",L91))</x:f>
+        <x:v>2.3912267547783585e-7</x:v>
+      </x:c>
       <x:c r="V91" s="58"/>
       <x:c r="W91" s="58"/>
       <x:c r="X91" s="58"/>
@@ -13874,7 +14057,10 @@
         <x:f>IF(W242="",AJ242,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U92" s="58"/>
+      <x:c r="U92" s="124" t="n">
+        <x:f>IF(ISNUMBER(L92),L92/(60000+L92),IF(L92="","",L92))</x:f>
+        <x:v>0.0000045930852798330524</x:v>
+      </x:c>
       <x:c r="V92" s="58"/>
       <x:c r="W92" s="58"/>
       <x:c r="X92" s="58"/>
@@ -13959,7 +14145,10 @@
         <x:f>IF(W243="",AJ243,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U93" s="58"/>
+      <x:c r="U93" s="124" t="n">
+        <x:f>IF(ISNUMBER(L93),L93/(60000+L93),IF(L93="","",L93))</x:f>
+        <x:v>0.0000022965479140367353</x:v>
+      </x:c>
       <x:c r="V93" s="58"/>
       <x:c r="W93" s="58"/>
       <x:c r="X93" s="58"/>
@@ -14044,7 +14233,10 @@
         <x:f>IF(W244="",AJ244,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U94" s="58"/>
+      <x:c r="U94" s="124" t="n">
+        <x:f>IF(ISNUMBER(L94),L94/(60000+L94),IF(L94="","",L94))</x:f>
+        <x:v>0.000001148275275552962</x:v>
+      </x:c>
       <x:c r="V94" s="58"/>
       <x:c r="W94" s="58"/>
       <x:c r="X94" s="58"/>
@@ -14129,7 +14321,10 @@
         <x:f>IF(W245="",AJ245,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U95" s="58"/>
+      <x:c r="U95" s="124" t="n">
+        <x:f>IF(ISNUMBER(L95),L95/(60000+L95),IF(L95="","",L95))</x:f>
+        <x:v>7.655171433767776e-7</x:v>
+      </x:c>
       <x:c r="V95" s="58"/>
       <x:c r="W95" s="58"/>
       <x:c r="X95" s="58"/>
@@ -14214,7 +14409,10 @@
         <x:f>IF(W246="",AJ246,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U96" s="58"/>
+      <x:c r="U96" s="124" t="n">
+        <x:f>IF(ISNUMBER(L96),L96/(60000+L96),IF(L96="","",L96))</x:f>
+        <x:v>0.000006124234322629933</x:v>
+      </x:c>
       <x:c r="V96" s="58"/>
       <x:c r="W96" s="58"/>
       <x:c r="X96" s="58"/>
@@ -14299,7 +14497,10 @@
         <x:f>IF(W247="",AJ247,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U97" s="58"/>
+      <x:c r="U97" s="124" t="n">
+        <x:f>IF(ISNUMBER(L97),L97/(60000+L97),IF(L97="","",L97))</x:f>
+        <x:v>0.0000030621265379051884</x:v>
+      </x:c>
       <x:c r="V97" s="58"/>
       <x:c r="W97" s="58"/>
       <x:c r="X97" s="58"/>
@@ -14384,7 +14585,10 @@
         <x:f>IF(W248="",AJ248,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U98" s="58"/>
+      <x:c r="U98" s="124" t="n">
+        <x:f>IF(ISNUMBER(L98),L98/(60000+L98),IF(L98="","",L98))</x:f>
+        <x:v>0.0000015310656131109166</x:v>
+      </x:c>
       <x:c r="V98" s="58"/>
       <x:c r="W98" s="58"/>
       <x:c r="X98" s="58"/>
@@ -14469,7 +14673,10 @@
         <x:f>IF(W249="",AJ249,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U99" s="58"/>
+      <x:c r="U99" s="124" t="n">
+        <x:f>IF(ISNUMBER(L99),L99/(60000+L99),IF(L99="","",L99))</x:f>
+        <x:v>0.0000010207109296657463</x:v>
+      </x:c>
       <x:c r="V99" s="58"/>
       <x:c r="W99" s="58"/>
       <x:c r="X99" s="58"/>
@@ -14554,7 +14761,10 @@
         <x:f>IF(W250="",AJ250,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U100" s="58"/>
+      <x:c r="U100" s="124" t="n">
+        <x:f>IF(ISNUMBER(L100),L100/(60000+L100),IF(L100="","",L100))</x:f>
+        <x:v>0.000001475211947762934</x:v>
+      </x:c>
       <x:c r="V100" s="58"/>
       <x:c r="W100" s="58"/>
       <x:c r="X100" s="58"/>
@@ -14639,7 +14849,10 @@
         <x:f>IF(W251="",AJ251,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U101" s="58"/>
+      <x:c r="U101" s="124" t="n">
+        <x:f>IF(ISNUMBER(L101),L101/(60000+L101),IF(L101="","",L101))</x:f>
+        <x:v>7.37606517944441e-7</x:v>
+      </x:c>
       <x:c r="V101" s="58"/>
       <x:c r="W101" s="58"/>
       <x:c r="X101" s="58"/>
@@ -14724,7 +14937,10 @@
         <x:f>IF(W252="",AJ252,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U102" s="58"/>
+      <x:c r="U102" s="124" t="n">
+        <x:f>IF(ISNUMBER(L102),L102/(60000+L102),IF(L102="","",L102))</x:f>
+        <x:v>3.688033949881145e-7</x:v>
+      </x:c>
       <x:c r="V102" s="58"/>
       <x:c r="W102" s="58"/>
       <x:c r="X102" s="58"/>
@@ -14809,7 +15025,10 @@
         <x:f>IF(W253="",AJ253,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U103" s="58"/>
+      <x:c r="U103" s="124" t="n">
+        <x:f>IF(ISNUMBER(L103),L103/(60000+L103),IF(L103="","",L103))</x:f>
+        <x:v>2.4586896021784544e-7</x:v>
+      </x:c>
       <x:c r="V103" s="58"/>
       <x:c r="W103" s="58"/>
       <x:c r="X103" s="58"/>
@@ -14894,7 +15113,10 @@
         <x:f>IF(W254="",AJ254,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U104" s="58"/>
+      <x:c r="U104" s="124" t="n">
+        <x:f>IF(ISNUMBER(L104),L104/(60000+L104),IF(L104="","",L104))</x:f>
+        <x:v>0.0000047227244309719</x:v>
+      </x:c>
       <x:c r="V104" s="58"/>
       <x:c r="W104" s="58"/>
       <x:c r="X104" s="58"/>
@@ -14979,7 +15201,10 @@
         <x:f>IF(W255="",AJ255,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U105" s="58"/>
+      <x:c r="U105" s="124" t="n">
+        <x:f>IF(ISNUMBER(L105),L105/(60000+L105),IF(L105="","",L105))</x:f>
+        <x:v>0.0000023613677915306294</x:v>
+      </x:c>
       <x:c r="V105" s="58"/>
       <x:c r="W105" s="58"/>
       <x:c r="X105" s="58"/>
@@ -15064,7 +15289,10 @@
         <x:f>IF(W256="",AJ256,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U106" s="58"/>
+      <x:c r="U106" s="124" t="n">
+        <x:f>IF(ISNUMBER(L106),L106/(60000+L106),IF(L106="","",L106))</x:f>
+        <x:v>0.0000011806852897814223</x:v>
+      </x:c>
       <x:c r="V106" s="58"/>
       <x:c r="W106" s="58"/>
       <x:c r="X106" s="58"/>
@@ -15149,7 +15377,10 @@
         <x:f>IF(W257="",AJ257,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U107" s="58"/>
+      <x:c r="U107" s="124" t="n">
+        <x:f>IF(ISNUMBER(L107),L107/(60000+L107),IF(L107="","",L107))</x:f>
+        <x:v>7.871238363027931e-7</x:v>
+      </x:c>
       <x:c r="V107" s="58"/>
       <x:c r="W107" s="58"/>
       <x:c r="X107" s="58"/>
@@ -15234,7 +15465,10 @@
         <x:f>IF(W258="",AJ258,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U108" s="58"/>
+      <x:c r="U108" s="124" t="n">
+        <x:f>IF(ISNUMBER(L108),L108/(60000+L108),IF(L108="","",L108))</x:f>
+        <x:v>0.000006297093429192404</x:v>
+      </x:c>
       <x:c r="V108" s="58"/>
       <x:c r="W108" s="58"/>
       <x:c r="X108" s="58"/>
@@ -15319,7 +15553,10 @@
         <x:f>IF(W259="",AJ259,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U109" s="58"/>
+      <x:c r="U109" s="124" t="n">
+        <x:f>IF(ISNUMBER(L109),L109/(60000+L109),IF(L109="","",L109))</x:f>
+        <x:v>0.0000031485566279738292</x:v>
+      </x:c>
       <x:c r="V109" s="58"/>
       <x:c r="W109" s="58"/>
       <x:c r="X109" s="58"/>
@@ -15404,7 +15641,10 @@
         <x:f>IF(W260="",AJ260,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U110" s="58"/>
+      <x:c r="U110" s="124" t="n">
+        <x:f>IF(ISNUMBER(L110),L110/(60000+L110),IF(L110="","",L110))</x:f>
+        <x:v>0.000001574280792343026</x:v>
+      </x:c>
       <x:c r="V110" s="58"/>
       <x:c r="W110" s="58"/>
       <x:c r="X110" s="58"/>
@@ -15489,7 +15729,10 @@
         <x:f>IF(W261="",AJ261,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U111" s="58"/>
+      <x:c r="U111" s="124" t="n">
+        <x:f>IF(ISNUMBER(L111),L111/(60000+L111),IF(L111="","",L111))</x:f>
+        <x:v>0.0000010495210789756425</x:v>
+      </x:c>
       <x:c r="V111" s="58"/>
       <x:c r="W111" s="58"/>
       <x:c r="X111" s="58"/>
@@ -15574,7 +15817,10 @@
         <x:f>IF(W262="",AJ262,"")</x:f>
         <x:v>0.07141190318323679</x:v>
       </x:c>
-      <x:c r="U112" s="58"/>
+      <x:c r="U112" s="124" t="n">
+        <x:f>IF(ISNUMBER(L112),L112/(60000+L112),IF(L112="","",L112))</x:f>
+        <x:v>0.000002539195545582969</x:v>
+      </x:c>
       <x:c r="V112" s="58"/>
       <x:c r="W112" s="58"/>
       <x:c r="X112" s="58"/>
@@ -15659,7 +15905,10 @@
         <x:f>IF(W263="",AJ263,"")</x:f>
         <x:v>0.03570595159161839</x:v>
       </x:c>
-      <x:c r="U113" s="58"/>
+      <x:c r="U113" s="124" t="n">
+        <x:f>IF(ISNUMBER(L113),L113/(60000+L113),IF(L113="","",L113))</x:f>
+        <x:v>0.0000012695993846720357</x:v>
+      </x:c>
       <x:c r="V113" s="58"/>
       <x:c r="W113" s="58"/>
       <x:c r="X113" s="58"/>
@@ -15744,7 +15993,10 @@
         <x:f>IF(W264="",AJ264,"")</x:f>
         <x:v>0.017852975795809196</x:v>
       </x:c>
-      <x:c r="U114" s="58"/>
+      <x:c r="U114" s="124" t="n">
+        <x:f>IF(ISNUMBER(L114),L114/(60000+L114),IF(L114="","",L114))</x:f>
+        <x:v>6.34800095306923e-7</x:v>
+      </x:c>
       <x:c r="V114" s="58"/>
       <x:c r="W114" s="58"/>
       <x:c r="X114" s="58"/>
@@ -15829,7 +16081,10 @@
         <x:f>IF(W265="",AJ265,"")</x:f>
         <x:v>0.011901983863872798</x:v>
       </x:c>
-      <x:c r="U115" s="58"/>
+      <x:c r="U115" s="124" t="n">
+        <x:f>IF(ISNUMBER(L115),L115/(60000+L115),IF(L115="","",L115))</x:f>
+        <x:v>4.2320015308711454e-7</x:v>
+      </x:c>
       <x:c r="V115" s="58"/>
       <x:c r="W115" s="58"/>
       <x:c r="X115" s="58"/>
@@ -15914,7 +16169,10 @@
         <x:f>IF(W266="",AJ266,"")</x:f>
         <x:v>0.20323946682416733</x:v>
       </x:c>
-      <x:c r="U116" s="58"/>
+      <x:c r="U116" s="124" t="n">
+        <x:f>IF(ISNUMBER(L116),L116/(60000+L116),IF(L116="","",L116))</x:f>
+        <x:v>0.0000072265799989659895</x:v>
+      </x:c>
       <x:c r="V116" s="58"/>
       <x:c r="W116" s="58"/>
       <x:c r="X116" s="58"/>
@@ -15999,7 +16257,10 @@
         <x:f>IF(W267="",AJ267,"")</x:f>
         <x:v>0.10161973341208366</x:v>
       </x:c>
-      <x:c r="U117" s="58"/>
+      <x:c r="U117" s="124" t="n">
+        <x:f>IF(ISNUMBER(L117),L117/(60000+L117),IF(L117="","",L117))</x:f>
+        <x:v>0.00000361330305539479</x:v>
+      </x:c>
       <x:c r="V117" s="58"/>
       <x:c r="W117" s="58"/>
       <x:c r="X117" s="58"/>
@@ -16084,7 +16345,10 @@
         <x:f>IF(W268="",AJ268,"")</x:f>
         <x:v>0.05080986670604183</x:v>
       </x:c>
-      <x:c r="U118" s="58"/>
+      <x:c r="U118" s="124" t="n">
+        <x:f>IF(ISNUMBER(L118),L118/(60000+L118),IF(L118="","",L118))</x:f>
+        <x:v>0.0000018066547916930345</x:v>
+      </x:c>
       <x:c r="V118" s="58"/>
       <x:c r="W118" s="58"/>
       <x:c r="X118" s="58"/>
@@ -16169,7 +16433,10 @@
         <x:f>IF(W269="",AJ269,"")</x:f>
         <x:v>0.03387324447069455</x:v>
       </x:c>
-      <x:c r="U119" s="58"/>
+      <x:c r="U119" s="124" t="n">
+        <x:f>IF(ISNUMBER(L119),L119/(60000+L119),IF(L119="","",L119))</x:f>
+        <x:v>0.000001204437253129468</x:v>
+      </x:c>
       <x:c r="V119" s="58"/>
       <x:c r="W119" s="58"/>
       <x:c r="X119" s="58"/>
@@ -16254,7 +16521,10 @@
         <x:f>IF(W270="",AJ270,"")</x:f>
         <x:v>0.26930071420807705</x:v>
       </x:c>
-      <x:c r="U120" s="58"/>
+      <x:c r="U120" s="124" t="n">
+        <x:f>IF(ISNUMBER(L120),L120/(60000+L120),IF(L120="","",L120))</x:f>
+        <x:v>0.000009575496995704403</x:v>
+      </x:c>
       <x:c r="V120" s="58"/>
       <x:c r="W120" s="58"/>
       <x:c r="X120" s="58"/>
@@ -16339,7 +16609,10 @@
         <x:f>IF(W271="",AJ271,"")</x:f>
         <x:v>0.13465035710403853</x:v>
       </x:c>
-      <x:c r="U121" s="58"/>
+      <x:c r="U121" s="124" t="n">
+        <x:f>IF(ISNUMBER(L121),L121/(60000+L121),IF(L121="","",L121))</x:f>
+        <x:v>0.000004787771420497628</x:v>
+      </x:c>
       <x:c r="V121" s="58"/>
       <x:c r="W121" s="58"/>
       <x:c r="X121" s="58"/>
@@ -16424,7 +16697,10 @@
         <x:f>IF(W272="",AJ272,"")</x:f>
         <x:v>0.06732517855201926</x:v>
       </x:c>
-      <x:c r="U122" s="58"/>
+      <x:c r="U122" s="124" t="n">
+        <x:f>IF(ISNUMBER(L122),L122/(60000+L122),IF(L122="","",L122))</x:f>
+        <x:v>0.0000023938914409513264</x:v>
+      </x:c>
       <x:c r="V122" s="58"/>
       <x:c r="W122" s="58"/>
       <x:c r="X122" s="58"/>
@@ -16509,7 +16785,10 @@
         <x:f>IF(W273="",AJ273,"")</x:f>
         <x:v>0.04488345236801285</x:v>
       </x:c>
-      <x:c r="U123" s="58"/>
+      <x:c r="U123" s="124" t="n">
+        <x:f>IF(ISNUMBER(L123),L123/(60000+L123),IF(L123="","",L123))</x:f>
+        <x:v>0.000001595928900794396</x:v>
+      </x:c>
       <x:c r="V123" s="58"/>
       <x:c r="W123" s="58"/>
       <x:c r="X123" s="58"/>
@@ -16594,7 +16873,10 @@
         <x:f>IF(W274="",AJ274,"")</x:f>
         <x:v>0.07141190318323679</x:v>
       </x:c>
-      <x:c r="U124" s="58"/>
+      <x:c r="U124" s="124" t="n">
+        <x:f>IF(ISNUMBER(L124),L124/(60000+L124),IF(L124="","",L124))</x:f>
+        <x:v>0.0000025780138062870714</x:v>
+      </x:c>
       <x:c r="V124" s="58"/>
       <x:c r="W124" s="58"/>
       <x:c r="X124" s="58"/>
@@ -16679,7 +16961,10 @@
         <x:f>IF(W275="",AJ275,"")</x:f>
         <x:v>0.03570595159161839</x:v>
       </x:c>
-      <x:c r="U125" s="58"/>
+      <x:c r="U125" s="124" t="n">
+        <x:f>IF(ISNUMBER(L125),L125/(60000+L125),IF(L125="","",L125))</x:f>
+        <x:v>0.0000012890085646844738</x:v>
+      </x:c>
       <x:c r="V125" s="58"/>
       <x:c r="W125" s="58"/>
       <x:c r="X125" s="58"/>
@@ -16764,7 +17049,10 @@
         <x:f>IF(W276="",AJ276,"")</x:f>
         <x:v>0.017852975795809196</x:v>
       </x:c>
-      <x:c r="U126" s="58"/>
+      <x:c r="U126" s="124" t="n">
+        <x:f>IF(ISNUMBER(L126),L126/(60000+L126),IF(L126="","",L126))</x:f>
+        <x:v>6.445046977282746e-7</x:v>
+      </x:c>
       <x:c r="V126" s="58"/>
       <x:c r="W126" s="58"/>
       <x:c r="X126" s="58"/>
@@ -16849,7 +17137,10 @@
         <x:f>IF(W277="",AJ277,"")</x:f>
         <x:v>0.011901983863872798</x:v>
       </x:c>
-      <x:c r="U127" s="58"/>
+      <x:c r="U127" s="124" t="n">
+        <x:f>IF(ISNUMBER(L127),L127/(60000+L127),IF(L127="","",L127))</x:f>
+        <x:v>4.2966989079360415e-7</x:v>
+      </x:c>
       <x:c r="V127" s="58"/>
       <x:c r="W127" s="58"/>
       <x:c r="X127" s="58"/>
@@ -16934,7 +17225,10 @@
         <x:f>IF(W278="",AJ278,"")</x:f>
         <x:v>0.20323946682416733</x:v>
       </x:c>
-      <x:c r="U128" s="58"/>
+      <x:c r="U128" s="124" t="n">
+        <x:f>IF(ISNUMBER(L128),L128/(60000+L128),IF(L128="","",L128))</x:f>
+        <x:v>0.0000073370622644750296</x:v>
+      </x:c>
       <x:c r="V128" s="58"/>
       <x:c r="W128" s="58"/>
       <x:c r="X128" s="58"/>
@@ -17019,7 +17313,10 @@
         <x:f>IF(W279="",AJ279,"")</x:f>
         <x:v>0.10161973341208366</x:v>
       </x:c>
-      <x:c r="U129" s="58"/>
+      <x:c r="U129" s="124" t="n">
+        <x:f>IF(ISNUMBER(L129),L129/(60000+L129),IF(L129="","",L129))</x:f>
+        <x:v>0.0000036685445904075544</x:v>
+      </x:c>
       <x:c r="V129" s="58"/>
       <x:c r="W129" s="58"/>
       <x:c r="X129" s="58"/>
@@ -17104,7 +17401,10 @@
         <x:f>IF(W280="",AJ280,"")</x:f>
         <x:v>0.05080986670604183</x:v>
       </x:c>
-      <x:c r="U130" s="58"/>
+      <x:c r="U130" s="124" t="n">
+        <x:f>IF(ISNUMBER(L130),L130/(60000+L130),IF(L130="","",L130))</x:f>
+        <x:v>0.0000018342756597648016</x:v>
+      </x:c>
       <x:c r="V130" s="58"/>
       <x:c r="W130" s="58"/>
       <x:c r="X130" s="58"/>
@@ -17189,7 +17489,10 @@
         <x:f>IF(W281="",AJ281,"")</x:f>
         <x:v>0.03387324447069455</x:v>
       </x:c>
-      <x:c r="U131" s="58"/>
+      <x:c r="U131" s="124" t="n">
+        <x:f>IF(ISNUMBER(L131),L131/(60000+L131),IF(L131="","",L131))</x:f>
+        <x:v>0.0000012228511875252572</x:v>
+      </x:c>
       <x:c r="V131" s="58"/>
       <x:c r="W131" s="58"/>
       <x:c r="X131" s="58"/>
@@ -17274,7 +17577,10 @@
         <x:f>IF(W282="",AJ282,"")</x:f>
         <x:v>0.26930071420807705</x:v>
       </x:c>
-      <x:c r="U132" s="58"/>
+      <x:c r="U132" s="124" t="n">
+        <x:f>IF(ISNUMBER(L132),L132/(60000+L132),IF(L132="","",L132))</x:f>
+        <x:v>0.000009721890323698737</x:v>
+      </x:c>
       <x:c r="V132" s="58"/>
       <x:c r="W132" s="58"/>
       <x:c r="X132" s="58"/>
@@ -17359,7 +17665,10 @@
         <x:f>IF(W283="",AJ283,"")</x:f>
         <x:v>0.13465035710403853</x:v>
       </x:c>
-      <x:c r="U133" s="58"/>
+      <x:c r="U133" s="124" t="n">
+        <x:f>IF(ISNUMBER(L133),L133/(60000+L133),IF(L133="","",L133))</x:f>
+        <x:v>0.000004860968790752094</x:v>
+      </x:c>
       <x:c r="V133" s="58"/>
       <x:c r="W133" s="58"/>
       <x:c r="X133" s="58"/>
@@ -17444,7 +17753,10 @@
         <x:f>IF(W284="",AJ284,"")</x:f>
         <x:v>0.06732517855201926</x:v>
       </x:c>
-      <x:c r="U134" s="58"/>
+      <x:c r="U134" s="124" t="n">
+        <x:f>IF(ISNUMBER(L134),L134/(60000+L134),IF(L134="","",L134))</x:f>
+        <x:v>0.0000024304903026448005</x:v>
+      </x:c>
       <x:c r="V134" s="58"/>
       <x:c r="W134" s="58"/>
       <x:c r="X134" s="58"/>
@@ -17529,7 +17841,10 @@
         <x:f>IF(W285="",AJ285,"")</x:f>
         <x:v>0.04488345236801285</x:v>
       </x:c>
-      <x:c r="U135" s="58"/>
+      <x:c r="U135" s="124" t="n">
+        <x:f>IF(ISNUMBER(L135),L135/(60000+L135),IF(L135="","",L135))</x:f>
+        <x:v>0.000001620328181160511</x:v>
+      </x:c>
       <x:c r="V135" s="58"/>
       <x:c r="W135" s="58"/>
       <x:c r="X135" s="58"/>
@@ -17614,7 +17929,10 @@
         <x:f>IF(W286="",AJ286,"")</x:f>
         <x:v>0.03682465800726994</x:v>
       </x:c>
-      <x:c r="U136" s="58"/>
+      <x:c r="U136" s="124" t="n">
+        <x:f>IF(ISNUMBER(L136),L136/(60000+L136),IF(L136="","",L136))</x:f>
+        <x:v>0.0000014885785005423645</x:v>
+      </x:c>
       <x:c r="V136" s="58"/>
       <x:c r="W136" s="58"/>
       <x:c r="X136" s="58"/>
@@ -17699,7 +18017,10 @@
         <x:f>IF(W287="",AJ287,"")</x:f>
         <x:v>0.01841232900363497</x:v>
       </x:c>
-      <x:c r="U137" s="58"/>
+      <x:c r="U137" s="124" t="n">
+        <x:f>IF(ISNUMBER(L137),L137/(60000+L137),IF(L137="","",L137))</x:f>
+        <x:v>7.442898042380825e-7</x:v>
+      </x:c>
       <x:c r="V137" s="58"/>
       <x:c r="W137" s="58"/>
       <x:c r="X137" s="58"/>
@@ -17784,7 +18105,10 @@
         <x:f>IF(W288="",AJ288,"")</x:f>
         <x:v>0.009206164501817484</x:v>
       </x:c>
-      <x:c r="U138" s="58"/>
+      <x:c r="U138" s="124" t="n">
+        <x:f>IF(ISNUMBER(L138),L138/(60000+L138),IF(L138="","",L138))</x:f>
+        <x:v>3.7214504061092105e-7</x:v>
+      </x:c>
       <x:c r="V138" s="58"/>
       <x:c r="W138" s="58"/>
       <x:c r="X138" s="58"/>
@@ -17869,7 +18193,10 @@
         <x:f>IF(W289="",AJ289,"")</x:f>
         <x:v>0.006137443001211656</x:v>
       </x:c>
-      <x:c r="U139" s="58"/>
+      <x:c r="U139" s="124" t="n">
+        <x:f>IF(ISNUMBER(L139),L139/(60000+L139),IF(L139="","",L139))</x:f>
+        <x:v>2.480967245166025e-7</x:v>
+      </x:c>
       <x:c r="V139" s="58"/>
       <x:c r="W139" s="58"/>
       <x:c r="X139" s="58"/>
@@ -17954,7 +18281,10 @@
         <x:f>IF(W290="",AJ290,"")</x:f>
         <x:v>0.09968649439730395</x:v>
       </x:c>
-      <x:c r="U140" s="58"/>
+      <x:c r="U140" s="124" t="n">
+        <x:f>IF(ISNUMBER(L140),L140/(60000+L140),IF(L140="","",L140))</x:f>
+        <x:v>0.00000402968475183312</x:v>
+      </x:c>
       <x:c r="V140" s="58"/>
       <x:c r="W140" s="58"/>
       <x:c r="X140" s="58"/>
@@ -18039,7 +18369,10 @@
         <x:f>IF(W291="",AJ291,"")</x:f>
         <x:v>0.04984324719865198</x:v>
       </x:c>
-      <x:c r="U141" s="58"/>
+      <x:c r="U141" s="124" t="n">
+        <x:f>IF(ISNUMBER(L141),L141/(60000+L141),IF(L141="","",L141))</x:f>
+        <x:v>0.0000020148464355145392</x:v>
+      </x:c>
       <x:c r="V141" s="58"/>
       <x:c r="W141" s="58"/>
       <x:c r="X141" s="58"/>
@@ -18124,7 +18457,10 @@
         <x:f>IF(W292="",AJ292,"")</x:f>
         <x:v>0.02492162359932599</x:v>
       </x:c>
-      <x:c r="U142" s="58"/>
+      <x:c r="U142" s="124" t="n">
+        <x:f>IF(ISNUMBER(L142),L142/(60000+L142),IF(L142="","",L142))</x:f>
+        <x:v>0.0000010074242326598318</x:v>
+      </x:c>
       <x:c r="V142" s="58"/>
       <x:c r="W142" s="58"/>
       <x:c r="X142" s="58"/>
@@ -18209,7 +18545,10 @@
         <x:f>IF(W293="",AJ293,"")</x:f>
         <x:v>0.016614415732883994</x:v>
       </x:c>
-      <x:c r="U143" s="58"/>
+      <x:c r="U143" s="124" t="n">
+        <x:f>IF(ISNUMBER(L143),L143/(60000+L143),IF(L143="","",L143))</x:f>
+        <x:v>6.716163806407602e-7</x:v>
+      </x:c>
       <x:c r="V143" s="58"/>
       <x:c r="W143" s="58"/>
       <x:c r="X143" s="58"/>
@@ -18294,7 +18633,10 @@
         <x:f>IF(W294="",AJ294,"")</x:f>
         <x:v>0.13170516511467462</x:v>
       </x:c>
-      <x:c r="U144" s="58"/>
+      <x:c r="U144" s="124" t="n">
+        <x:f>IF(ISNUMBER(L144),L144/(60000+L144),IF(L144="","",L144))</x:f>
+        <x:v>0.000005323989155181612</x:v>
+      </x:c>
       <x:c r="V144" s="58"/>
       <x:c r="W144" s="58"/>
       <x:c r="X144" s="58"/>
@@ -18379,7 +18721,10 @@
         <x:f>IF(W295="",AJ295,"")</x:f>
         <x:v>0.06585258255733731</x:v>
       </x:c>
-      <x:c r="U145" s="58"/>
+      <x:c r="U145" s="124" t="n">
+        <x:f>IF(ISNUMBER(L145),L145/(60000+L145),IF(L145="","",L145))</x:f>
+        <x:v>0.0000026620016638248008</x:v>
+      </x:c>
       <x:c r="V145" s="58"/>
       <x:c r="W145" s="58"/>
       <x:c r="X145" s="58"/>
@@ -18464,7 +18809,10 @@
         <x:f>IF(W296="",AJ296,"")</x:f>
         <x:v>0.032926291278668654</x:v>
       </x:c>
-      <x:c r="U146" s="58"/>
+      <x:c r="U146" s="124" t="n">
+        <x:f>IF(ISNUMBER(L146),L146/(60000+L146),IF(L146="","",L146))</x:f>
+        <x:v>0.0000013310026034779731</x:v>
+      </x:c>
       <x:c r="V146" s="58"/>
       <x:c r="W146" s="58"/>
       <x:c r="X146" s="58"/>
@@ -18549,7 +18897,10 @@
         <x:f>IF(W297="",AJ297,"")</x:f>
         <x:v>0.02195086085244577</x:v>
       </x:c>
-      <x:c r="U147" s="58"/>
+      <x:c r="U147" s="124" t="n">
+        <x:f>IF(ISNUMBER(L147),L147/(60000+L147),IF(L147="","",L147))</x:f>
+        <x:v>8.873354626672523e-7</x:v>
+      </x:c>
       <x:c r="V147" s="58"/>
       <x:c r="W147" s="58"/>
       <x:c r="X147" s="58"/>
@@ -18634,7 +18985,10 @@
         <x:f>IF(W298="",AJ298,"")</x:f>
         <x:v>0.03682465800726994</x:v>
       </x:c>
-      <x:c r="U148" s="58"/>
+      <x:c r="U148" s="124" t="n">
+        <x:f>IF(ISNUMBER(L148),L148/(60000+L148),IF(L148="","",L148))</x:f>
+        <x:v>0.0000015132703706189044</x:v>
+      </x:c>
       <x:c r="V148" s="58"/>
       <x:c r="W148" s="58"/>
       <x:c r="X148" s="58"/>
@@ -18719,7 +19073,10 @@
         <x:f>IF(W299="",AJ299,"")</x:f>
         <x:v>0.01841232900363497</x:v>
       </x:c>
-      <x:c r="U149" s="58"/>
+      <x:c r="U149" s="124" t="n">
+        <x:f>IF(ISNUMBER(L149),L149/(60000+L149),IF(L149="","",L149))</x:f>
+        <x:v>7.56635757806689e-7</x:v>
+      </x:c>
       <x:c r="V149" s="58"/>
       <x:c r="W149" s="58"/>
       <x:c r="X149" s="58"/>
@@ -18804,7 +19161,10 @@
         <x:f>IF(W300="",AJ300,"")</x:f>
         <x:v>0.009206164501817484</x:v>
       </x:c>
-      <x:c r="U150" s="58"/>
+      <x:c r="U150" s="124" t="n">
+        <x:f>IF(ISNUMBER(L150),L150/(60000+L150),IF(L150="","",L150))</x:f>
+        <x:v>3.783180220278162e-7</x:v>
+      </x:c>
       <x:c r="V150" s="58"/>
       <x:c r="W150" s="58"/>
       <x:c r="X150" s="58"/>
@@ -18889,7 +19249,10 @@
         <x:f>IF(W301="",AJ301,"")</x:f>
         <x:v>0.006137443001211656</x:v>
       </x:c>
-      <x:c r="U151" s="58"/>
+      <x:c r="U151" s="124" t="n">
+        <x:f>IF(ISNUMBER(L151),L151/(60000+L151),IF(L151="","",L151))</x:f>
+        <x:v>2.522120464906649e-7</x:v>
+      </x:c>
       <x:c r="V151" s="58"/>
       <x:c r="W151" s="58"/>
       <x:c r="X151" s="58"/>
@@ -18974,7 +19337,10 @@
         <x:f>IF(W302="",AJ302,"")</x:f>
         <x:v>0.09968649439730395</x:v>
       </x:c>
-      <x:c r="U152" s="58"/>
+      <x:c r="U152" s="124" t="n">
+        <x:f>IF(ISNUMBER(L152),L152/(60000+L152),IF(L152="","",L152))</x:f>
+        <x:v>0.000004096530036728239</x:v>
+      </x:c>
       <x:c r="V152" s="58"/>
       <x:c r="W152" s="58"/>
       <x:c r="X152" s="58"/>
@@ -19059,7 +19425,10 @@
         <x:f>IF(W303="",AJ303,"")</x:f>
         <x:v>0.04984324719865198</x:v>
       </x:c>
-      <x:c r="U153" s="58"/>
+      <x:c r="U153" s="124" t="n">
+        <x:f>IF(ISNUMBER(L153),L153/(60000+L153),IF(L153="","",L153))</x:f>
+        <x:v>0.0000020482692137622983</x:v>
+      </x:c>
       <x:c r="V153" s="58"/>
       <x:c r="W153" s="58"/>
       <x:c r="X153" s="58"/>
@@ -19144,7 +19513,10 @@
         <x:f>IF(W304="",AJ304,"")</x:f>
         <x:v>0.02492162359932599</x:v>
       </x:c>
-      <x:c r="U154" s="58"/>
+      <x:c r="U154" s="124" t="n">
+        <x:f>IF(ISNUMBER(L154),L154/(60000+L154),IF(L154="","",L154))</x:f>
+        <x:v>0.0000010241356557339165</x:v>
+      </x:c>
       <x:c r="V154" s="58"/>
       <x:c r="W154" s="58"/>
       <x:c r="X154" s="58"/>
@@ -19229,7 +19601,10 @@
         <x:f>IF(W305="",AJ305,"")</x:f>
         <x:v>0.016614415732883994</x:v>
       </x:c>
-      <x:c r="U155" s="58"/>
+      <x:c r="U155" s="124" t="n">
+        <x:f>IF(ISNUMBER(L155),L155/(60000+L155),IF(L155="","",L155))</x:f>
+        <x:v>6.827573369013218e-7</x:v>
+      </x:c>
       <x:c r="V155" s="58"/>
       <x:c r="W155" s="58"/>
       <x:c r="X155" s="58"/>
@@ -19314,7 +19689,10 @@
         <x:f>IF(W306="",AJ306,"")</x:f>
         <x:v>0.13170516511467462</x:v>
       </x:c>
-      <x:c r="U156" s="58"/>
+      <x:c r="U156" s="124" t="n">
+        <x:f>IF(ISNUMBER(L156),L156/(60000+L156),IF(L156="","",L156))</x:f>
+        <x:v>0.0000054123047515661465</x:v>
+      </x:c>
       <x:c r="V156" s="58"/>
       <x:c r="W156" s="58"/>
       <x:c r="X156" s="58"/>
@@ -19399,7 +19777,10 @@
         <x:f>IF(W307="",AJ307,"")</x:f>
         <x:v>0.06585258255733731</x:v>
       </x:c>
-      <x:c r="U157" s="58"/>
+      <x:c r="U157" s="124" t="n">
+        <x:f>IF(ISNUMBER(L157),L157/(60000+L157),IF(L157="","",L157))</x:f>
+        <x:v>0.000002706159699063572</x:v>
+      </x:c>
       <x:c r="V157" s="58"/>
       <x:c r="W157" s="58"/>
       <x:c r="X157" s="58"/>
@@ -19484,7 +19865,10 @@
         <x:f>IF(W308="",AJ308,"")</x:f>
         <x:v>0.032926291278668654</x:v>
       </x:c>
-      <x:c r="U158" s="58"/>
+      <x:c r="U158" s="124" t="n">
+        <x:f>IF(ISNUMBER(L158),L158/(60000+L158),IF(L158="","",L158))</x:f>
+        <x:v>0.0000013530816803593426</x:v>
+      </x:c>
       <x:c r="V158" s="58"/>
       <x:c r="W158" s="58"/>
       <x:c r="X158" s="58"/>
@@ -19569,7 +19953,10 @@
         <x:f>IF(W309="",AJ309,"")</x:f>
         <x:v>0.02195086085244577</x:v>
       </x:c>
-      <x:c r="U159" s="58"/>
+      <x:c r="U159" s="124" t="n">
+        <x:f>IF(ISNUMBER(L159),L159/(60000+L159),IF(L159="","",L159))</x:f>
+        <x:v>9.020548604241971e-7</x:v>
+      </x:c>
       <x:c r="V159" s="58"/>
       <x:c r="W159" s="58"/>
       <x:c r="X159" s="58"/>
@@ -19654,7 +20041,10 @@
         <x:f>IF(W310="",AJ310,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U160" s="58"/>
+      <x:c r="U160" s="124" t="n">
+        <x:f>IF(ISNUMBER(L160),L160/(60000+L160),IF(L160="","",L160))</x:f>
+        <x:v>1.7847686302615647e-8</x:v>
+      </x:c>
       <x:c r="V160" s="58"/>
       <x:c r="W160" s="58"/>
       <x:c r="X160" s="58"/>
@@ -19739,7 +20129,10 @@
         <x:f>IF(W311="",AJ311,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U161" s="58"/>
+      <x:c r="U161" s="124" t="n">
+        <x:f>IF(ISNUMBER(L161),L161/(60000+L161),IF(L161="","",L161))</x:f>
+        <x:v>8.9238432309428e-9</x:v>
+      </x:c>
       <x:c r="V161" s="58"/>
       <x:c r="W161" s="58"/>
       <x:c r="X161" s="58"/>
@@ -19824,7 +20217,10 @@
         <x:f>IF(W312="",AJ312,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U162" s="58"/>
+      <x:c r="U162" s="124" t="n">
+        <x:f>IF(ISNUMBER(L162),L162/(60000+L162),IF(L162="","",L162))</x:f>
+        <x:v>4.461921635380145e-9</x:v>
+      </x:c>
       <x:c r="V162" s="58"/>
       <x:c r="W162" s="58"/>
       <x:c r="X162" s="58"/>
@@ -19909,7 +20305,10 @@
         <x:f>IF(W313="",AJ313,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U163" s="58"/>
+      <x:c r="U163" s="124" t="n">
+        <x:f>IF(ISNUMBER(L163),L163/(60000+L163),IF(L163="","",L163))</x:f>
+        <x:v>2.974614428010928e-9</x:v>
+      </x:c>
       <x:c r="V163" s="58"/>
       <x:c r="W163" s="58"/>
       <x:c r="X163" s="58"/>
@@ -19994,7 +20393,10 @@
         <x:f>IF(W314="",AJ314,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U164" s="58"/>
+      <x:c r="U164" s="124" t="n">
+        <x:f>IF(ISNUMBER(L164),L164/(60000+L164),IF(L164="","",L164))</x:f>
+        <x:v>4.7430939405203674e-8</x:v>
+      </x:c>
       <x:c r="V164" s="58"/>
       <x:c r="W164" s="58"/>
       <x:c r="X164" s="58"/>
@@ -20079,7 +20481,10 @@
         <x:f>IF(W315="",AJ315,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U165" s="58"/>
+      <x:c r="U165" s="124" t="n">
+        <x:f>IF(ISNUMBER(L165),L165/(60000+L165),IF(L165="","",L165))</x:f>
+        <x:v>2.3715470265025355e-8</x:v>
+      </x:c>
       <x:c r="V165" s="58"/>
       <x:c r="W165" s="58"/>
       <x:c r="X165" s="58"/>
@@ -20164,7 +20569,10 @@
         <x:f>IF(W316="",AJ316,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U166" s="58"/>
+      <x:c r="U166" s="124" t="n">
+        <x:f>IF(ISNUMBER(L166),L166/(60000+L166),IF(L166="","",L166))</x:f>
+        <x:v>1.185773527311856e-8</x:v>
+      </x:c>
       <x:c r="V166" s="58"/>
       <x:c r="W166" s="58"/>
       <x:c r="X166" s="58"/>
@@ -20249,7 +20657,10 @@
         <x:f>IF(W317="",AJ317,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U167" s="58"/>
+      <x:c r="U167" s="124" t="n">
+        <x:f>IF(ISNUMBER(L167),L167/(60000+L167),IF(L167="","",L167))</x:f>
+        <x:v>7.90515687999146e-9</x:v>
+      </x:c>
       <x:c r="V167" s="58"/>
       <x:c r="W167" s="58"/>
       <x:c r="X167" s="58"/>
@@ -20334,7 +20745,10 @@
         <x:f>IF(W318="",AJ318,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U168" s="58"/>
+      <x:c r="U168" s="124" t="n">
+        <x:f>IF(ISNUMBER(L168),L168/(60000+L168),IF(L168="","",L168))</x:f>
+        <x:v>6.259580791944164e-8</x:v>
+      </x:c>
       <x:c r="V168" s="58"/>
       <x:c r="W168" s="58"/>
       <x:c r="X168" s="58"/>
@@ -20419,7 +20833,10 @@
         <x:f>IF(W319="",AJ319,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U169" s="58"/>
+      <x:c r="U169" s="124" t="n">
+        <x:f>IF(ISNUMBER(L169),L169/(60000+L169),IF(L169="","",L169))</x:f>
+        <x:v>3.129790493927964e-8</x:v>
+      </x:c>
       <x:c r="V169" s="58"/>
       <x:c r="W169" s="58"/>
       <x:c r="X169" s="58"/>
@@ -20504,7 +20921,10 @@
         <x:f>IF(W320="",AJ320,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U170" s="58"/>
+      <x:c r="U170" s="124" t="n">
+        <x:f>IF(ISNUMBER(L170),L170/(60000+L170),IF(L170="","",L170))</x:f>
+        <x:v>1.5648952714529536e-8</x:v>
+      </x:c>
       <x:c r="V170" s="58"/>
       <x:c r="W170" s="58"/>
       <x:c r="X170" s="58"/>
@@ -20589,7 +21009,10 @@
         <x:f>IF(W321="",AJ321,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U171" s="58"/>
+      <x:c r="U171" s="124" t="n">
+        <x:f>IF(ISNUMBER(L171),L171/(60000+L171),IF(L171="","",L171))</x:f>
+        <x:v>1.0432635197439629e-8</x:v>
+      </x:c>
       <x:c r="V171" s="58"/>
       <x:c r="W171" s="58"/>
       <x:c r="X171" s="58"/>
@@ -20674,7 +21097,10 @@
         <x:f>IF(W322="",AJ322,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U172" s="58"/>
+      <x:c r="U172" s="124" t="n">
+        <x:f>IF(ISNUMBER(L172),L172/(60000+L172),IF(L172="","",L172))</x:f>
+        <x:v>1.835195748411923e-8</x:v>
+      </x:c>
       <x:c r="V172" s="58"/>
       <x:c r="W172" s="58"/>
       <x:c r="X172" s="58"/>
@@ -20759,7 +21185,10 @@
         <x:f>IF(W323="",AJ323,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U173" s="58"/>
+      <x:c r="U173" s="124" t="n">
+        <x:f>IF(ISNUMBER(L173),L173/(60000+L173),IF(L173="","",L173))</x:f>
+        <x:v>9.175978826258202e-9</x:v>
+      </x:c>
       <x:c r="V173" s="58"/>
       <x:c r="W173" s="58"/>
       <x:c r="X173" s="58"/>
@@ -20844,7 +21273,10 @@
         <x:f>IF(W324="",AJ324,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U174" s="58"/>
+      <x:c r="U174" s="124" t="n">
+        <x:f>IF(ISNUMBER(L174),L174/(60000+L174),IF(L174="","",L174))</x:f>
+        <x:v>4.587989434178748e-9</x:v>
+      </x:c>
       <x:c r="V174" s="58"/>
       <x:c r="W174" s="58"/>
       <x:c r="X174" s="58"/>
@@ -20929,7 +21361,10 @@
         <x:f>IF(W325="",AJ325,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U175" s="58"/>
+      <x:c r="U175" s="124" t="n">
+        <x:f>IF(ISNUMBER(L175),L175/(60000+L175),IF(L175="","",L175))</x:f>
+        <x:v>3.0586596274635314e-9</x:v>
+      </x:c>
       <x:c r="V175" s="58"/>
       <x:c r="W175" s="58"/>
       <x:c r="X175" s="58"/>
@@ -21014,7 +21449,10 @@
         <x:f>IF(W326="",AJ326,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U176" s="58"/>
+      <x:c r="U176" s="124" t="n">
+        <x:f>IF(ISNUMBER(L176),L176/(60000+L176),IF(L176="","",L176))</x:f>
+        <x:v>4.878097748682107e-8</x:v>
+      </x:c>
       <x:c r="V176" s="58"/>
       <x:c r="W176" s="58"/>
       <x:c r="X176" s="58"/>
@@ -21099,7 +21537,10 @@
         <x:f>IF(W327="",AJ327,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U177" s="58"/>
+      <x:c r="U177" s="124" t="n">
+        <x:f>IF(ISNUMBER(L177),L177/(60000+L177),IF(L177="","",L177))</x:f>
+        <x:v>2.4390489338306487e-8</x:v>
+      </x:c>
       <x:c r="V177" s="58"/>
       <x:c r="W177" s="58"/>
       <x:c r="X177" s="58"/>
@@ -21184,7 +21625,10 @@
         <x:f>IF(W328="",AJ328,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U178" s="58"/>
+      <x:c r="U178" s="124" t="n">
+        <x:f>IF(ISNUMBER(L178),L178/(60000+L178),IF(L178="","",L178))</x:f>
+        <x:v>1.2195244817877239e-8</x:v>
+      </x:c>
       <x:c r="V178" s="58"/>
       <x:c r="W178" s="58"/>
       <x:c r="X178" s="58"/>
@@ -21269,7 +21713,10 @@
         <x:f>IF(W329="",AJ329,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U179" s="58"/>
+      <x:c r="U179" s="124" t="n">
+        <x:f>IF(ISNUMBER(L179),L179/(60000+L179),IF(L179="","",L179))</x:f>
+        <x:v>8.130163244967935e-9</x:v>
+      </x:c>
       <x:c r="V179" s="58"/>
       <x:c r="W179" s="58"/>
       <x:c r="X179" s="58"/>
@@ -21354,7 +21801,10 @@
         <x:f>IF(W330="",AJ330,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U180" s="58"/>
+      <x:c r="U180" s="124" t="n">
+        <x:f>IF(ISNUMBER(L180),L180/(60000+L180),IF(L180="","",L180))</x:f>
+        <x:v>6.437828333327506e-8</x:v>
+      </x:c>
       <x:c r="V180" s="58"/>
       <x:c r="W180" s="58"/>
       <x:c r="X180" s="58"/>
@@ -21439,7 +21889,10 @@
         <x:f>IF(W331="",AJ331,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U181" s="58"/>
+      <x:c r="U181" s="124" t="n">
+        <x:f>IF(ISNUMBER(L181),L181/(60000+L181),IF(L181="","",L181))</x:f>
+        <x:v>3.21891427027784e-8</x:v>
+      </x:c>
       <x:c r="V181" s="58"/>
       <x:c r="W181" s="58"/>
       <x:c r="X181" s="58"/>
@@ -21524,7 +21977,10 @@
         <x:f>IF(W332="",AJ332,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U182" s="58"/>
+      <x:c r="U182" s="124" t="n">
+        <x:f>IF(ISNUMBER(L182),L182/(60000+L182),IF(L182="","",L182))</x:f>
+        <x:v>1.6094571610424433e-8</x:v>
+      </x:c>
       <x:c r="V182" s="58"/>
       <x:c r="W182" s="58"/>
       <x:c r="X182" s="58"/>
@@ -21609,13 +22065,18 @@
         <x:f>IF(W333="",AJ333,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U183" s="58"/>
+      <x:c r="U183" s="124" t="n">
+        <x:f>IF(ISNUMBER(L183),L183/(60000+L183),IF(L183="","",L183))</x:f>
+        <x:v>1.0729714464513006e-8</x:v>
+      </x:c>
       <x:c r="V183" s="58"/>
       <x:c r="W183" s="58"/>
       <x:c r="X183" s="58"/>
     </x:row>
     <x:row r="184" ht="18" customHeight="1">
-      <x:c r="A184" s="58"/>
+      <x:c r="A184" s="58" t="str">
+        <x:v>Decode throughput loss = Total overhead / (60000 + Total overhead). Fixed batch size and tokens/step; Decode stays busy.</x:v>
+      </x:c>
       <x:c r="B184" s="58"/>
       <x:c r="C184" s="58"/>
       <x:c r="D184" s="58"/>

</xml_diff>